<commit_message>
Generate first approved production article draft
</commit_message>
<xml_diff>
--- a/data/master_dashboard.xlsx
+++ b/data/master_dashboard.xlsx
@@ -452,7 +452,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -472,7 +472,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -482,7 +482,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -492,7 +492,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8">
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -617,22 +617,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>meetily Review 2026</t>
+          <t>The SaaS Apocalypse Is Real. Causal AI Is the Escape Route</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>meetily Review 2026</t>
+          <t>The SaaS Apocalypse Is Real. Causal AI Is the Escape Route</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>meetily-review-2026</t>
+          <t>the-saas-apocalypse-is-real-causal-ai-is-the-escape-route</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>commercial research</t>
+          <t>mixed informational and commercial</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -642,11 +642,11 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>meetily Review 2026</t>
+          <t>The SaaS Apocalypse Is Real. Causal AI Is the Escape Route</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>62.5</v>
+        <v>54.1</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -658,7 +658,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -668,12 +668,12 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>["meetily review 2026 faq", "how to use meetily review 2026", "meetily review 2026 pricing", "meetily review 2026 comparison", "meetily review 2026 alternatives"]</t>
+          <t>["the saas apocalypse is real causal ai is the escape route comparison", "the saas apocalypse is real causal ai is the escape route faq", "how to use the saas apocalypse is real causal ai is the escape route", "the saas apocalypse is real causal ai is the escape route alternatives", "the saas apocalypse is real causal ai is the escape route pricing"]</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>["Detected search intent 'commercial' from the query.", "Matched intent terms: review.", "Matched article-type terms: review.", "Intent confidence 0.9; article-type confidence 0.95.", "Detected search intent 'commercial' from the query.", "Intent depth classified as shallow based on query specificity."]</t>
+          <t>["Detected search intent 'commercial' from the query.", "Intent confidence 0.0; article-type confidence 0.0.", "Detected search intent 'informational' from the query.", "Intent depth classified as shallow based on query specificity.", "Scope classified as broad based on narrowing terms and product intent.", "Buyer journey stage is awareness and funnel stage is top."]</t>
         </is>
       </c>
     </row>
@@ -683,17 +683,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>system_prompts_leaks Review 2026</t>
+          <t>best ai productivity software</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>system_prompts_leaks Review 2026</t>
+          <t>best ai productivity software</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>system-prompts-leaks-review-2026</t>
+          <t>best-ai-productivity-software</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -708,11 +708,11 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>system_prompts_leaks Review 2026</t>
+          <t>best ai productivity software</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>62.3</v>
+        <v>51.7</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -724,22 +724,22 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>listicle</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>["system prompts leaks review 2026 comparison", "how to use system prompts leaks review 2026", "system prompts leaks review 2026 pricing", "system prompts leaks review 2026 alternatives", "system prompts leaks review 2026 faq"]</t>
+          <t>["how to use best ai productivity software", "best ai productivity software comparison", "best ai productivity software faq", "best ai productivity software alternatives", "best ai productivity software pricing"]</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>["Detected search intent 'commercial' from the query.", "Matched intent terms: review.", "Matched article-type terms: review.", "Intent confidence 0.9; article-type confidence 0.95.", "Detected search intent 'commercial' from the query.", "Intent depth classified as shallow based on query specificity."]</t>
+          <t>["Detected search intent 'commercial' from the query.", "Matched intent terms: best.", "Matched article-type terms: best.", "Intent confidence 0.95; article-type confidence 1.25.", "Detected search intent 'commercial' from the query.", "Intent depth classified as medium based on query specificity."]</t>
         </is>
       </c>
     </row>
@@ -749,17 +749,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>agent-skills Review 2026</t>
+          <t>best ai meeting software</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>agent-skills Review 2026</t>
+          <t>best ai meeting software</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>agent-skills-review-2026</t>
+          <t>best-ai-meeting-software</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -769,16 +769,16 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>AI Agents</t>
+          <t>AI Software</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>agent-skills Review 2026</t>
+          <t>best ai meeting software</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>61.5</v>
+        <v>50.5</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -790,22 +790,22 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>listicle</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>["agent-skills review 2026 faq", "agent-skills review 2026 alternatives", "agent-skills review 2026 comparison", "how to use agent-skills review 2026", "agent-skills review 2026 pricing"]</t>
+          <t>["best ai meeting software alternatives", "best ai meeting software comparison", "best ai meeting software pricing", "how to use best ai meeting software", "best ai meeting software faq"]</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>["Detected search intent 'commercial' from the query.", "Matched intent terms: review.", "Matched article-type terms: review.", "Intent confidence 0.9; article-type confidence 0.95.", "Detected search intent 'commercial' from the query.", "Intent depth classified as shallow based on query specificity."]</t>
+          <t>["Detected search intent 'commercial' from the query.", "Matched intent terms: best.", "Matched article-type terms: best.", "Intent confidence 0.95; article-type confidence 1.25.", "Detected search intent 'commercial' from the query.", "Intent depth classified as medium based on query specificity."]</t>
         </is>
       </c>
     </row>
@@ -815,17 +815,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>last30days-skill Review 2026</t>
+          <t>best ai voice software</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>last30days-skill Review 2026</t>
+          <t>best ai voice software</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>last30days-skill-review-2026</t>
+          <t>best-ai-voice-software</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -840,11 +840,11 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>last30days-skill Review 2026</t>
+          <t>best ai voice software</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>60.5</v>
+        <v>50.5</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -856,22 +856,22 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>listicle</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>["last30days-skill review 2026 pricing", "last30days-skill review 2026 alternatives", "last30days-skill review 2026 comparison", "how to use last30days-skill review 2026", "last30days-skill review 2026 faq"]</t>
+          <t>["best ai voice software pricing", "best ai voice software alternatives", "best ai voice software faq", "how to use best ai voice software", "best ai voice software comparison"]</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>["Detected search intent 'commercial' from the query.", "Matched intent terms: review.", "Matched article-type terms: review.", "Intent confidence 0.9; article-type confidence 0.95.", "Detected search intent 'commercial' from the query.", "Intent depth classified as shallow based on query specificity."]</t>
+          <t>["Detected search intent 'commercial' from the query.", "Matched intent terms: best.", "Matched article-type terms: best.", "Intent confidence 0.95; article-type confidence 1.25.", "Detected search intent 'commercial' from the query.", "Intent depth classified as medium based on query specificity."]</t>
         </is>
       </c>
     </row>
@@ -881,22 +881,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>taste-skill Review 2026</t>
+          <t>Impartner Redefines Partner Marketing Automation with Full Automation, AdTech and AI to Drive Measurable Revenue</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>taste-skill Review 2026</t>
+          <t>Impartner Redefines Partner Marketing Automation with Full Automation, AdTech and AI to Drive Measurable Revenue</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>taste-skill-review-2026</t>
+          <t>impartner-redefines-partner-marketing-automation-with-full-automation-adtech-and-ai-to-drive-measurable-revenue</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>commercial research</t>
+          <t>mixed informational and commercial</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -906,11 +906,11 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>taste-skill Review 2026</t>
+          <t>Impartner Redefines Partner Marketing Automation with Full Automation, AdTech and AI to Drive Measurable Revenue</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>58</v>
+        <v>50.3</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -922,7 +922,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -932,12 +932,12 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>["taste-skill review 2026 faq", "taste-skill review 2026 comparison", "taste-skill review 2026 pricing", "taste-skill review 2026 alternatives", "how to use taste-skill review 2026"]</t>
+          <t>["how to use impartner redefines partner marketing automation with full automation adtech and ai to drive measurable revenue", "impartner redefines partner marketing automation with full automation adtech and ai to drive measurable revenue faq", "impartner redefines partner marketing automation with full automation adtech and ai to drive measurable revenue alternatives", "impartner redefines partner marketing automation with full automation adtech and ai to drive measurable revenue comparison", "impartner redefines partner marketing automation with full automation adtech and ai to drive measurable revenue pricing"]</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>["Detected search intent 'commercial' from the query.", "Matched intent terms: review.", "Matched article-type terms: review.", "Intent confidence 0.9; article-type confidence 0.95.", "Detected search intent 'commercial' from the query.", "Intent depth classified as shallow based on query specificity."]</t>
+          <t>["Detected search intent 'commercial' from the query.", "Intent confidence 0.0; article-type confidence 0.0.", "Detected search intent 'informational' from the query.", "Intent depth classified as shallow based on query specificity.", "Scope classified as broad based on narrowing terms and product intent.", "Buyer journey stage is awareness and funnel stage is top."]</t>
         </is>
       </c>
     </row>
@@ -947,36 +947,36 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>karakeep Review 2026</t>
+          <t>AI coding tokens could soon cost as much as salaries</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>karakeep Review 2026</t>
+          <t>AI coding tokens could soon cost as much as salaries</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>karakeep-review-2026</t>
+          <t>ai-coding-tokens-could-soon-cost-as-much-as-salaries</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>commercial research</t>
+          <t>commercial investigation</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>AI Software</t>
+          <t>AI Coding</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>karakeep Review 2026</t>
+          <t>AI coding tokens could soon cost as much as salaries</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>55.7</v>
+        <v>49.8</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -988,22 +988,22 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>pricing</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>["karakeep review 2026 alternatives", "how to use karakeep review 2026", "karakeep review 2026 faq", "karakeep review 2026 comparison", "karakeep review 2026 pricing"]</t>
+          <t>["ai coding tokens could soon cost as much as salaries pricing", "ai coding tokens could soon cost as much as salaries faq", "how to use ai coding tokens could soon cost as much as salaries", "ai coding tokens could soon cost as much as salaries comparison", "ai coding tokens could soon cost as much as salaries alternatives"]</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>["Detected search intent 'commercial' from the query.", "Matched intent terms: review.", "Matched article-type terms: review.", "Intent confidence 0.9; article-type confidence 0.95.", "Detected search intent 'commercial' from the query.", "Intent depth classified as shallow based on query specificity."]</t>
+          <t>["Detected search intent 'transactional' from the query.", "Matched intent terms: cost.", "Matched article-type terms: cost.", "Intent confidence 0.95; article-type confidence 0.95.", "Detected search intent 'transactional' from the query.", "Intent depth classified as deep based on query specificity."]</t>
         </is>
       </c>
     </row>
@@ -1013,22 +1013,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>The SaaS Apocalypse Is Real. Causal AI Is the Escape Route</t>
+          <t>How AI is upending SaaS tools</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>The SaaS Apocalypse Is Real. Causal AI Is the Escape Route</t>
+          <t>How AI is upending SaaS tools</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>the-saas-apocalypse-is-real-causal-ai-is-the-escape-route</t>
+          <t>how-ai-is-upending-saas-tools</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>mixed informational and commercial</t>
+          <t>commercial research</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1038,11 +1038,11 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>The SaaS Apocalypse Is Real. Causal AI Is the Escape Route</t>
+          <t>How AI is upending SaaS tools</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>54.1</v>
+        <v>49.3</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -1059,12 +1059,12 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>listicle</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>["the saas apocalypse is real causal ai is the escape route pricing", "the saas apocalypse is real causal ai is the escape route comparison", "the saas apocalypse is real causal ai is the escape route alternatives", "the saas apocalypse is real causal ai is the escape route faq", "how to use the saas apocalypse is real causal ai is the escape route"]</t>
+          <t>["how ai is upending saas tools pricing", "how ai is upending saas tools faq", "how ai is upending saas tools alternatives", "how to use how ai is upending saas tools", "how ai is upending saas tools comparison"]</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1079,17 +1079,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>best ai productivity software</t>
+          <t>Shopify launches AI-powered marketing automation tool</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>best ai productivity software</t>
+          <t>Shopify launches AI-powered marketing automation tool</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>best-ai-productivity-software</t>
+          <t>shopify-launches-ai-powered-marketing-automation-tool</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1104,11 +1104,11 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>best ai productivity software</t>
+          <t>Shopify launches AI-powered marketing automation tool</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>51.7</v>
+        <v>48.9</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -1125,17 +1125,17 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>listicle</t>
+          <t>news/update</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>["best ai productivity software comparison", "how to use best ai productivity software", "best ai productivity software faq", "best ai productivity software alternatives", "best ai productivity software pricing"]</t>
+          <t>["shopify launches ai-powered marketing automation tool comparison", "how to use shopify launches ai-powered marketing automation tool", "shopify launches ai-powered marketing automation tool alternatives", "shopify launches ai-powered marketing automation tool faq", "shopify launches ai-powered marketing automation tool pricing"]</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>["Detected search intent 'commercial' from the query.", "Matched intent terms: best.", "Matched article-type terms: best.", "Intent confidence 0.95; article-type confidence 1.25.", "Detected search intent 'commercial' from the query.", "Intent depth classified as medium based on query specificity."]</t>
+          <t>["Detected search intent 'commercial' from the query.", "Intent confidence 0.0; article-type confidence 0.0.", "Detected search intent 'informational' from the query.", "Intent depth classified as shallow based on query specificity.", "Scope classified as broad based on narrowing terms and product intent.", "Buyer journey stage is awareness and funnel stage is top."]</t>
         </is>
       </c>
     </row>
@@ -1145,17 +1145,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>best ai meeting software</t>
+          <t>best ai meeting tools</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>best ai meeting software</t>
+          <t>best ai meeting tools</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>best-ai-meeting-software</t>
+          <t>best-ai-meeting-tools</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1170,11 +1170,11 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>best ai meeting software</t>
+          <t>best ai meeting tools</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>50.5</v>
+        <v>48.8</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -1196,7 +1196,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>["how to use best ai meeting software", "best ai meeting software pricing", "best ai meeting software faq", "best ai meeting software alternatives", "best ai meeting software comparison"]</t>
+          <t>["how to use best ai meeting tools", "best ai meeting tools comparison", "best ai meeting tools alternatives", "best ai meeting tools faq", "best ai meeting tools pricing"]</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1211,36 +1211,36 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>best ai voice software</t>
+          <t>AI coding costs could exceed developer salaries by 2028</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>best ai voice software</t>
+          <t>AI coding costs could exceed developer salaries by 2028</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>best-ai-voice-software</t>
+          <t>ai-coding-costs-could-exceed-developer-salaries-by-2028</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>commercial research</t>
+          <t>commercial investigation</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>AI Software</t>
+          <t>AI Coding</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>best ai voice software</t>
+          <t>AI coding costs could exceed developer salaries by 2028</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>50.5</v>
+        <v>48.6</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -1257,17 +1257,17 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>listicle</t>
+          <t>pricing</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>["best ai voice software comparison", "how to use best ai voice software", "best ai voice software pricing", "best ai voice software faq", "best ai voice software alternatives"]</t>
+          <t>["ai coding costs could exceed developer salaries by 2028 pricing", "ai coding costs could exceed developer salaries by 2028 faq", "how to use ai coding costs could exceed developer salaries by 2028", "ai coding costs could exceed developer salaries by 2028 alternatives", "ai coding costs could exceed developer salaries by 2028 comparison"]</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>["Detected search intent 'commercial' from the query.", "Matched intent terms: best.", "Matched article-type terms: best.", "Intent confidence 0.95; article-type confidence 1.25.", "Detected search intent 'commercial' from the query.", "Intent depth classified as medium based on query specificity."]</t>
+          <t>["Detected search intent 'transactional' from the query.", "Matched intent terms: cost.", "Matched article-type terms: cost.", "Intent confidence 0.95; article-type confidence 0.95.", "Detected search intent 'transactional' from the query.", "Intent depth classified as deep based on query specificity."]</t>
         </is>
       </c>
     </row>
@@ -1282,13 +1282,150 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>empty</t>
+          <t>publish_date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>day_of_week</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>parent_keyword</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>parent_slug</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>slug</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>stage</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>article_type</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>cluster</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>priority</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>intent</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>related_keywords</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>reasoning</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>best ai productivity software</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>best-ai-productivity-software</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>best ai productivity software</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>best ai productivity software</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>best-ai-productivity-software</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>pillar</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>listicle</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>best ai productivity software</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>commercial research</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>["how to use best ai productivity software", "best ai productivity software comparison", "best ai productivity software faq", "best ai productivity software alternatives", "best ai productivity software pricing"]</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>["Monday editorial expansion for best ai productivity software.", "Detected search intent 'commercial' from the query.", "Matched intent terms: best.", "Matched article-type terms: best."]</t>
         </is>
       </c>
     </row>
@@ -1303,13 +1440,196 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:U2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>empty</t>
+          <t>slug</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>checked_at</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>failures</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>research_quality_passed</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>verified_source_score_passed</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>knowledge_freshness_passed</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>ai_review_passed</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>human_approval_passed</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>broken_links</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>duplicate_title_meta</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>affiliate_disclosure_present</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>minimum_business_score_passed</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>minimum_readability_score_passed</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>business_score</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>readability_score</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>publish_ready</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>best-ai-productivity-software</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>best ai productivity software</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-07-07T11:51:48.169437+00:00</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>["human approval missing"]</t>
+        </is>
+      </c>
+      <c r="F2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H2" t="b">
+        <v>1</v>
+      </c>
+      <c r="I2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J2" t="b">
+        <v>0</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="L2" t="b">
+        <v>0</v>
+      </c>
+      <c r="M2" t="b">
+        <v>1</v>
+      </c>
+      <c r="N2" t="b">
+        <v>1</v>
+      </c>
+      <c r="O2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P2" t="n">
+        <v>61.35</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>58.37</v>
+      </c>
+      <c r="R2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>https://smileaireviewhub.com/best-ai-productivity-software/</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>best ai productivity software 2026: Pricing, Pros, Cons</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Independent best ai productivity software guide with pricing checks, pros, cons, alternatives, FAQs, and buyer-focused workflow advice.</t>
         </is>
       </c>
     </row>
@@ -1324,15 +1644,78 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>empty</t>
-        </is>
-      </c>
+          <t>slug</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>reviewed_at</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>approved_at</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>approved_by</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>best-ai-productivity-software</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>best ai productivity software</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="D2" t="b">
+        <v>1</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-07-07T11:51:48.162268+00:00</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1345,7 +1728,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R10"/>
+  <dimension ref="A1:R11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1475,12 +1858,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-07-07T09:38:56.586490+00:00</t>
+          <t>2026-07-07T09:39:33.140144+00:00</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>needs_enrichment</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="K2" t="n">
@@ -1553,12 +1936,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-07-07T09:38:56.859663+00:00</t>
+          <t>2026-07-07T09:39:33.147772+00:00</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>needs_enrichment</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="K3" t="n">
@@ -1631,12 +2014,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-07-07T09:38:57.100585+00:00</t>
+          <t>2026-07-07T09:39:33.179929+00:00</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>needs_enrichment</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="K4" t="n">
@@ -1709,12 +2092,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-07-07T09:38:57.305735+00:00</t>
+          <t>2026-07-07T09:39:33.209943+00:00</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>needs_enrichment</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="K5" t="n">
@@ -1787,12 +2170,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-07-07T09:38:57.498105+00:00</t>
+          <t>2026-07-07T09:39:33.242931+00:00</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>needs_enrichment</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="K6" t="n">
@@ -1865,12 +2248,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-07-07T09:38:57.719879+00:00</t>
+          <t>2026-07-07T09:39:33.271421+00:00</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>needs_enrichment</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="K7" t="n">
@@ -1943,12 +2326,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-07-07T09:38:57.945870+00:00</t>
+          <t>2026-07-07T09:39:48.182992+00:00</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>needs_enrichment</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="K8" t="n">
@@ -2021,12 +2404,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-07-07T09:38:58.268317+00:00</t>
+          <t>2026-07-07T09:39:48.204668+00:00</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>needs_enrichment</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="K9" t="n">
@@ -2099,12 +2482,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-07-07T09:38:58.460659+00:00</t>
+          <t>2026-07-07T09:39:48.139069+00:00</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>needs_enrichment</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="K10" t="n">
@@ -2139,6 +2522,66 @@
         </is>
       </c>
       <c r="R10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Impartner Redefines Partner Marketing Automation with Full Automation, AdTech and AI to Drive Measurable Revenue</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>impartner-redefines-partner-marketing-automation-with-full-automation-adtech-and-ai-to-drive-measurable-revenue</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>20</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" t="n">
+        <v>5</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>competitor coverage is limited; official_docs_score 0.0 below 20.0; pricing_source_score 0.0 below 20.0; affiliate_source_score 0.0 below 10.0; total_verified_source_score 0.0 below 35.0; verified_sources 0 below 1; official_verified_sources 0 below 1</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-07-07T09:39:48.231145+00:00</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>62.43</v>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="R11" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2229,7 +2672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U11"/>
+  <dimension ref="A1:U2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2342,808 +2785,79 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>the-saas-apocalypse-is-real-causal-ai-is-the-escape-route</t>
+          <t>best-ai-productivity-software</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>The SaaS Apocalypse Is Real. Causal AI Is the Escape Route</t>
+          <t>best ai productivity software</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>43.71</v>
+        <v>62.36</v>
       </c>
       <c r="D2" t="n">
         <v>72</v>
       </c>
       <c r="E2" t="n">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="F2" t="n">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["affiliate_networks", "integrations", "use_cases", "target_audience", "competitors"]</t>
         </is>
       </c>
       <c r="H2" t="n">
         <v>68</v>
       </c>
       <c r="I2" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J2" t="n">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="K2" t="n">
-        <v>5</v>
+        <v>89.5</v>
       </c>
       <c r="L2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="M2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="N2" t="n">
-        <v>0</v>
+        <v>98</v>
       </c>
       <c r="O2" t="n">
-        <v>0</v>
+        <v>79</v>
       </c>
       <c r="P2" t="n">
-        <v>0</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>needs enrichment</t>
+          <t>ready</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>["trusted sources are thin", "official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["Notion", "Gamma", "Notion AI"]</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
-        <is>
-          <t>D:\AFFILATE BOT\data\research\the-saas-apocalypse-is-real-causal-ai-is-the-escape-route</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>best-ai-voice-software</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>best ai voice software</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>57.79</v>
-      </c>
-      <c r="D3" t="n">
-        <v>72</v>
-      </c>
-      <c r="E3" t="n">
-        <v>60</v>
-      </c>
-      <c r="F3" t="n">
-        <v>60</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>["affiliate_networks", "integrations", "use_cases", "target_audience", "competitors"]</t>
-        </is>
-      </c>
-      <c r="H3" t="n">
-        <v>68</v>
-      </c>
-      <c r="I3" t="n">
-        <v>80</v>
-      </c>
-      <c r="J3" t="n">
-        <v>49</v>
-      </c>
-      <c r="K3" t="n">
-        <v>65.5</v>
-      </c>
-      <c r="L3" t="n">
-        <v>100</v>
-      </c>
-      <c r="M3" t="n">
-        <v>100</v>
-      </c>
-      <c r="N3" t="n">
-        <v>99</v>
-      </c>
-      <c r="O3" t="n">
-        <v>79</v>
-      </c>
-      <c r="P3" t="n">
-        <v>92</v>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>verified</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>needs enrichment</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>["competitor coverage is limited"]</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>["ElevenLabs"]</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>D:\AFFILATE BOT\data\research\best-ai-voice-software</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>best-ai-meeting-software</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>best ai meeting software</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>57.79</v>
-      </c>
-      <c r="D4" t="n">
-        <v>72</v>
-      </c>
-      <c r="E4" t="n">
-        <v>60</v>
-      </c>
-      <c r="F4" t="n">
-        <v>60</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>["affiliate_networks", "integrations", "use_cases", "target_audience", "competitors"]</t>
-        </is>
-      </c>
-      <c r="H4" t="n">
-        <v>68</v>
-      </c>
-      <c r="I4" t="n">
-        <v>80</v>
-      </c>
-      <c r="J4" t="n">
-        <v>49</v>
-      </c>
-      <c r="K4" t="n">
-        <v>65.5</v>
-      </c>
-      <c r="L4" t="n">
-        <v>99</v>
-      </c>
-      <c r="M4" t="n">
-        <v>100</v>
-      </c>
-      <c r="N4" t="n">
-        <v>99</v>
-      </c>
-      <c r="O4" t="n">
-        <v>79</v>
-      </c>
-      <c r="P4" t="n">
-        <v>91.59999999999999</v>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>verified</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>needs enrichment</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>["competitor coverage is limited"]</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>["Reclaim AI"]</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>D:\AFFILATE BOT\data\research\best-ai-meeting-software</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>karakeep-review-2026</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>karakeep Review 2026</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>45.14</v>
-      </c>
-      <c r="D5" t="n">
-        <v>72</v>
-      </c>
-      <c r="E5" t="n">
-        <v>36</v>
-      </c>
-      <c r="F5" t="n">
-        <v>36</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
-        </is>
-      </c>
-      <c r="H5" t="n">
-        <v>68</v>
-      </c>
-      <c r="I5" t="n">
-        <v>80</v>
-      </c>
-      <c r="J5" t="n">
-        <v>45</v>
-      </c>
-      <c r="K5" t="n">
-        <v>5</v>
-      </c>
-      <c r="L5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>needs enrichment</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>["trusted sources are thin", "official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>D:\AFFILATE BOT\data\research\karakeep-review-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>taste-skill-review-2026</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>taste-skill Review 2026</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>45.14</v>
-      </c>
-      <c r="D6" t="n">
-        <v>72</v>
-      </c>
-      <c r="E6" t="n">
-        <v>36</v>
-      </c>
-      <c r="F6" t="n">
-        <v>36</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
-        </is>
-      </c>
-      <c r="H6" t="n">
-        <v>68</v>
-      </c>
-      <c r="I6" t="n">
-        <v>80</v>
-      </c>
-      <c r="J6" t="n">
-        <v>45</v>
-      </c>
-      <c r="K6" t="n">
-        <v>5</v>
-      </c>
-      <c r="L6" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>needs enrichment</t>
-        </is>
-      </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>["trusted sources are thin", "official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>D:\AFFILATE BOT\data\research\taste-skill-review-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>last30days-skill-review-2026</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>last30days-skill Review 2026</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>45.14</v>
-      </c>
-      <c r="D7" t="n">
-        <v>72</v>
-      </c>
-      <c r="E7" t="n">
-        <v>36</v>
-      </c>
-      <c r="F7" t="n">
-        <v>36</v>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
-        </is>
-      </c>
-      <c r="H7" t="n">
-        <v>68</v>
-      </c>
-      <c r="I7" t="n">
-        <v>80</v>
-      </c>
-      <c r="J7" t="n">
-        <v>45</v>
-      </c>
-      <c r="K7" t="n">
-        <v>5</v>
-      </c>
-      <c r="L7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>needs enrichment</t>
-        </is>
-      </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>["trusted sources are thin", "official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
-        </is>
-      </c>
-      <c r="T7" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>D:\AFFILATE BOT\data\research\last30days-skill-review-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>agent-skills-review-2026</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>agent-skills Review 2026</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>45.14</v>
-      </c>
-      <c r="D8" t="n">
-        <v>72</v>
-      </c>
-      <c r="E8" t="n">
-        <v>36</v>
-      </c>
-      <c r="F8" t="n">
-        <v>36</v>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
-        </is>
-      </c>
-      <c r="H8" t="n">
-        <v>68</v>
-      </c>
-      <c r="I8" t="n">
-        <v>80</v>
-      </c>
-      <c r="J8" t="n">
-        <v>45</v>
-      </c>
-      <c r="K8" t="n">
-        <v>5</v>
-      </c>
-      <c r="L8" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" t="n">
-        <v>0</v>
-      </c>
-      <c r="O8" t="n">
-        <v>0</v>
-      </c>
-      <c r="P8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>needs enrichment</t>
-        </is>
-      </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>["trusted sources are thin", "official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
-        </is>
-      </c>
-      <c r="T8" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>D:\AFFILATE BOT\data\research\agent-skills-review-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>system-prompts-leaks-review-2026</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>system_prompts_leaks Review 2026</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>45.14</v>
-      </c>
-      <c r="D9" t="n">
-        <v>72</v>
-      </c>
-      <c r="E9" t="n">
-        <v>36</v>
-      </c>
-      <c r="F9" t="n">
-        <v>36</v>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
-        </is>
-      </c>
-      <c r="H9" t="n">
-        <v>68</v>
-      </c>
-      <c r="I9" t="n">
-        <v>80</v>
-      </c>
-      <c r="J9" t="n">
-        <v>45</v>
-      </c>
-      <c r="K9" t="n">
-        <v>5</v>
-      </c>
-      <c r="L9" t="n">
-        <v>0</v>
-      </c>
-      <c r="M9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N9" t="n">
-        <v>0</v>
-      </c>
-      <c r="O9" t="n">
-        <v>0</v>
-      </c>
-      <c r="P9" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>needs enrichment</t>
-        </is>
-      </c>
-      <c r="S9" t="inlineStr">
-        <is>
-          <t>["trusted sources are thin", "official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
-        </is>
-      </c>
-      <c r="T9" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>D:\AFFILATE BOT\data\research\system-prompts-leaks-review-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>meetily-review-2026</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>meetily Review 2026</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>45.14</v>
-      </c>
-      <c r="D10" t="n">
-        <v>72</v>
-      </c>
-      <c r="E10" t="n">
-        <v>36</v>
-      </c>
-      <c r="F10" t="n">
-        <v>36</v>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
-        </is>
-      </c>
-      <c r="H10" t="n">
-        <v>68</v>
-      </c>
-      <c r="I10" t="n">
-        <v>80</v>
-      </c>
-      <c r="J10" t="n">
-        <v>45</v>
-      </c>
-      <c r="K10" t="n">
-        <v>5</v>
-      </c>
-      <c r="L10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" t="n">
-        <v>0</v>
-      </c>
-      <c r="O10" t="n">
-        <v>0</v>
-      </c>
-      <c r="P10" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>needs enrichment</t>
-        </is>
-      </c>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>["trusted sources are thin", "official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
-        </is>
-      </c>
-      <c r="T10" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>D:\AFFILATE BOT\data\research\meetily-review-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>best-ai-productivity-software</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>best ai productivity software</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>62.36</v>
-      </c>
-      <c r="D11" t="n">
-        <v>72</v>
-      </c>
-      <c r="E11" t="n">
-        <v>60</v>
-      </c>
-      <c r="F11" t="n">
-        <v>60</v>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>["affiliate_networks", "integrations", "use_cases", "target_audience", "competitors"]</t>
-        </is>
-      </c>
-      <c r="H11" t="n">
-        <v>68</v>
-      </c>
-      <c r="I11" t="n">
-        <v>80</v>
-      </c>
-      <c r="J11" t="n">
-        <v>57</v>
-      </c>
-      <c r="K11" t="n">
-        <v>89.5</v>
-      </c>
-      <c r="L11" t="n">
-        <v>100</v>
-      </c>
-      <c r="M11" t="n">
-        <v>100</v>
-      </c>
-      <c r="N11" t="n">
-        <v>98</v>
-      </c>
-      <c r="O11" t="n">
-        <v>79</v>
-      </c>
-      <c r="P11" t="n">
-        <v>91.59999999999999</v>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>verified</t>
-        </is>
-      </c>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t>ready</t>
-        </is>
-      </c>
-      <c r="S11" t="inlineStr">
-        <is>
-          <t>["competitor coverage is limited"]</t>
-        </is>
-      </c>
-      <c r="T11" t="inlineStr">
-        <is>
-          <t>["Notion", "Gamma", "Notion AI"]</t>
-        </is>
-      </c>
-      <c r="U11" t="inlineStr">
         <is>
           <t>D:\AFFILATE BOT\data\research\best-ai-productivity-software</t>
         </is>

</xml_diff>

<commit_message>
Improve editorial console operator workflow and custom topic requests
</commit_message>
<xml_diff>
--- a/data/master_dashboard.xlsx
+++ b/data/master_dashboard.xlsx
@@ -462,7 +462,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -472,7 +472,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -482,7 +482,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -1440,196 +1440,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U2"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>slug</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>topic</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>checked_at</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>failures</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>research_quality_passed</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>verified_source_score_passed</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>knowledge_freshness_passed</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>ai_review_passed</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>human_approval_passed</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>broken_links</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>duplicate_title_meta</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>affiliate_disclosure_present</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>minimum_business_score_passed</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>minimum_readability_score_passed</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>business_score</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>readability_score</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>publish_ready</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>best-ai-productivity-software</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>best ai productivity software</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>blocked</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-07-07T11:51:48.169437+00:00</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>["human approval missing"]</t>
-        </is>
-      </c>
-      <c r="F2" t="b">
-        <v>1</v>
-      </c>
-      <c r="G2" t="b">
-        <v>1</v>
-      </c>
-      <c r="H2" t="b">
-        <v>1</v>
-      </c>
-      <c r="I2" t="b">
-        <v>1</v>
-      </c>
-      <c r="J2" t="b">
-        <v>0</v>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="L2" t="b">
-        <v>0</v>
-      </c>
-      <c r="M2" t="b">
-        <v>1</v>
-      </c>
-      <c r="N2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P2" t="n">
-        <v>61.35</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>58.37</v>
-      </c>
-      <c r="R2" t="b">
-        <v>0</v>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>https://smileaireviewhub.com/best-ai-productivity-software/</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>best ai productivity software 2026: Pricing, Pros, Cons</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>Independent best ai productivity software guide with pricing checks, pros, cons, alternatives, FAQs, and buyer-focused workflow advice.</t>
+          <t>empty</t>
         </is>
       </c>
     </row>
@@ -1644,78 +1461,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>slug</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>topic</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>required</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>reviewed_at</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>approved_at</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>approved_by</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>reason</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>best-ai-productivity-software</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>best ai productivity software</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>needs_human_review</t>
-        </is>
-      </c>
-      <c r="D2" t="b">
-        <v>1</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>2026-07-07T11:51:48.162268+00:00</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
+          <t>empty</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Publish ready daily articles 2026-07-09
</commit_message>
<xml_diff>
--- a/data/master_dashboard.xlsx
+++ b/data/master_dashboard.xlsx
@@ -462,7 +462,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -472,7 +472,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6">
@@ -492,7 +492,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8">
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="10">
@@ -1440,13 +1440,777 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:U9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>empty</t>
+          <t>slug</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>checked_at</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>failures</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>research_quality_passed</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>verified_source_score_passed</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>knowledge_freshness_passed</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>ai_review_passed</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>human_approval_passed</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>broken_links</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>duplicate_title_meta</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>affiliate_disclosure_present</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>minimum_business_score_passed</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>minimum_readability_score_passed</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>business_score</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>readability_score</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>publish_ready</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>agent-skills-review-2026</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>agent-skills Review 2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-07-08T22:18:36.107297+00:00</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>["verified source score failed", "knowledge freshness failed", "AI review failed"]</t>
+        </is>
+      </c>
+      <c r="F2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J2" t="b">
+        <v>1</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="L2" t="b">
+        <v>0</v>
+      </c>
+      <c r="M2" t="b">
+        <v>1</v>
+      </c>
+      <c r="N2" t="b">
+        <v>1</v>
+      </c>
+      <c r="O2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P2" t="n">
+        <v>57.15</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>59.22</v>
+      </c>
+      <c r="R2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>https://smileaireviewhub.com/agent-skills-review-2026/</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>agent-skills Review 2026: Pricing, Pros, Cons</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Independent agent-skills Review 2026 guide with pricing checks, pros, cons, alternatives, FAQs, and buyer-focused workflow advice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>meetily-review-2026</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>meetily Review 2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-07-08T22:19:22.916589+00:00</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>["verified source score failed", "knowledge freshness failed", "AI review failed"]</t>
+        </is>
+      </c>
+      <c r="F3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G3" t="b">
+        <v>0</v>
+      </c>
+      <c r="H3" t="b">
+        <v>0</v>
+      </c>
+      <c r="I3" t="b">
+        <v>0</v>
+      </c>
+      <c r="J3" t="b">
+        <v>1</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="L3" t="b">
+        <v>0</v>
+      </c>
+      <c r="M3" t="b">
+        <v>1</v>
+      </c>
+      <c r="N3" t="b">
+        <v>1</v>
+      </c>
+      <c r="O3" t="b">
+        <v>1</v>
+      </c>
+      <c r="P3" t="n">
+        <v>57.15</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>59.48</v>
+      </c>
+      <c r="R3" t="b">
+        <v>0</v>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>https://smileaireviewhub.com/meetily-review-2026/</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>meetily Review 2026: Pricing, Pros, Cons</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Independent meetily Review 2026 guide with pricing checks, pros, cons, alternatives, FAQs, and buyer-focused workflow advice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>system-prompts-leaks-review-2026</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>system_prompts_leaks Review 2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-07-08T22:19:57.113612+00:00</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>["verified source score failed", "knowledge freshness failed", "AI review failed"]</t>
+        </is>
+      </c>
+      <c r="F4" t="b">
+        <v>1</v>
+      </c>
+      <c r="G4" t="b">
+        <v>0</v>
+      </c>
+      <c r="H4" t="b">
+        <v>0</v>
+      </c>
+      <c r="I4" t="b">
+        <v>0</v>
+      </c>
+      <c r="J4" t="b">
+        <v>1</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="L4" t="b">
+        <v>0</v>
+      </c>
+      <c r="M4" t="b">
+        <v>1</v>
+      </c>
+      <c r="N4" t="b">
+        <v>1</v>
+      </c>
+      <c r="O4" t="b">
+        <v>1</v>
+      </c>
+      <c r="P4" t="n">
+        <v>57.15</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>58.73</v>
+      </c>
+      <c r="R4" t="b">
+        <v>0</v>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>https://smileaireviewhub.com/system-prompts-leaks-review-2026/</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>system_prompts_leaks Review 2026: Pricing, Pros, Cons</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Independent system_prompts_leaks Review 2026 guide with pricing checks, pros, cons, alternatives, FAQs, and buyer-focused workflow advice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ai-job-search-review-2026</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ai-job-search Review 2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2026-07-08T22:20:05.263013+00:00</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>["verified source score failed", "knowledge freshness failed", "AI review failed"]</t>
+        </is>
+      </c>
+      <c r="F5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G5" t="b">
+        <v>0</v>
+      </c>
+      <c r="H5" t="b">
+        <v>0</v>
+      </c>
+      <c r="I5" t="b">
+        <v>0</v>
+      </c>
+      <c r="J5" t="b">
+        <v>1</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="L5" t="b">
+        <v>0</v>
+      </c>
+      <c r="M5" t="b">
+        <v>1</v>
+      </c>
+      <c r="N5" t="b">
+        <v>1</v>
+      </c>
+      <c r="O5" t="b">
+        <v>1</v>
+      </c>
+      <c r="P5" t="n">
+        <v>57.15</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>59.25</v>
+      </c>
+      <c r="R5" t="b">
+        <v>0</v>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>https://smileaireviewhub.com/ai-job-search-review-2026/</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>ai-job-search Review 2026: Pricing, Pros, Cons</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Independent ai-job-search Review 2026 guide with pricing checks, pros, cons, alternatives, FAQs, and buyer-focused workflow advice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>officecli-review-2026</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>OfficeCLI Review 2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026-07-08T22:20:12.568712+00:00</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>["verified source score failed", "knowledge freshness failed", "AI review failed"]</t>
+        </is>
+      </c>
+      <c r="F6" t="b">
+        <v>1</v>
+      </c>
+      <c r="G6" t="b">
+        <v>0</v>
+      </c>
+      <c r="H6" t="b">
+        <v>0</v>
+      </c>
+      <c r="I6" t="b">
+        <v>0</v>
+      </c>
+      <c r="J6" t="b">
+        <v>1</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="L6" t="b">
+        <v>0</v>
+      </c>
+      <c r="M6" t="b">
+        <v>1</v>
+      </c>
+      <c r="N6" t="b">
+        <v>1</v>
+      </c>
+      <c r="O6" t="b">
+        <v>1</v>
+      </c>
+      <c r="P6" t="n">
+        <v>57.15</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>59.32</v>
+      </c>
+      <c r="R6" t="b">
+        <v>0</v>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>https://smileaireviewhub.com/officecli-review-2026/</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>OfficeCLI Review 2026: Pricing, Pros, Cons</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Independent OfficeCLI Review 2026 guide with pricing checks, pros, cons, alternatives, FAQs, and buyer-focused workflow advice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>cubesandbox-review-2026</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>CubeSandbox Review 2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026-07-08T22:20:19.442623+00:00</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>["verified source score failed", "knowledge freshness failed", "AI review failed"]</t>
+        </is>
+      </c>
+      <c r="F7" t="b">
+        <v>1</v>
+      </c>
+      <c r="G7" t="b">
+        <v>0</v>
+      </c>
+      <c r="H7" t="b">
+        <v>0</v>
+      </c>
+      <c r="I7" t="b">
+        <v>0</v>
+      </c>
+      <c r="J7" t="b">
+        <v>1</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="L7" t="b">
+        <v>0</v>
+      </c>
+      <c r="M7" t="b">
+        <v>1</v>
+      </c>
+      <c r="N7" t="b">
+        <v>1</v>
+      </c>
+      <c r="O7" t="b">
+        <v>1</v>
+      </c>
+      <c r="P7" t="n">
+        <v>57.15</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>59.17</v>
+      </c>
+      <c r="R7" t="b">
+        <v>0</v>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>https://smileaireviewhub.com/cubesandbox-review-2026/</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>CubeSandbox Review 2026: Pricing, Pros, Cons</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>Independent CubeSandbox Review 2026 guide with pricing checks, pros, cons, alternatives, FAQs, and buyer-focused workflow advice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>skills-review-2026</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>skills Review 2026</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2026-07-08T22:20:27.803787+00:00</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>["verified source score failed", "knowledge freshness failed", "AI review failed"]</t>
+        </is>
+      </c>
+      <c r="F8" t="b">
+        <v>1</v>
+      </c>
+      <c r="G8" t="b">
+        <v>0</v>
+      </c>
+      <c r="H8" t="b">
+        <v>0</v>
+      </c>
+      <c r="I8" t="b">
+        <v>0</v>
+      </c>
+      <c r="J8" t="b">
+        <v>1</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="L8" t="b">
+        <v>0</v>
+      </c>
+      <c r="M8" t="b">
+        <v>1</v>
+      </c>
+      <c r="N8" t="b">
+        <v>1</v>
+      </c>
+      <c r="O8" t="b">
+        <v>1</v>
+      </c>
+      <c r="P8" t="n">
+        <v>57.15</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>59.56</v>
+      </c>
+      <c r="R8" t="b">
+        <v>0</v>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>https://smileaireviewhub.com/skills-review-2026/</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>skills Review 2026: Pricing, Pros, Cons</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>Independent skills Review 2026 guide with pricing checks, pros, cons, alternatives, FAQs, and buyer-focused workflow advice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>companies-are-buying-ai-tools-that-doesn-t-mean-they-know-what-to-do-with-them</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Companies are buying AI tools. That doesn't mean they know what to do with them.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2026-07-08T22:20:34.366057+00:00</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>["verified source score failed", "knowledge freshness failed", "AI review failed"]</t>
+        </is>
+      </c>
+      <c r="F9" t="b">
+        <v>1</v>
+      </c>
+      <c r="G9" t="b">
+        <v>0</v>
+      </c>
+      <c r="H9" t="b">
+        <v>0</v>
+      </c>
+      <c r="I9" t="b">
+        <v>0</v>
+      </c>
+      <c r="J9" t="b">
+        <v>1</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="L9" t="b">
+        <v>0</v>
+      </c>
+      <c r="M9" t="b">
+        <v>1</v>
+      </c>
+      <c r="N9" t="b">
+        <v>1</v>
+      </c>
+      <c r="O9" t="b">
+        <v>1</v>
+      </c>
+      <c r="P9" t="n">
+        <v>57.15</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>64.19</v>
+      </c>
+      <c r="R9" t="b">
+        <v>0</v>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>https://smileaireviewhub.com/companies-are-buying-ai-tools-that-doesn-t-mean-they-know-what-to-do-with-them/</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>Companies are buying AI tools. That doesn't mean they kn</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Independent Companies are buying AI tools. That doesn't mean they know what to do with them. guide with pricing checks, pros, cons, alternatives, FAQs, an.</t>
         </is>
       </c>
     </row>
@@ -1612,7 +2376,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-07-07T09:39:33.140144+00:00</t>
+          <t>2026-07-08T01:42:03.376492+00:00</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -1690,7 +2454,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-07-07T09:39:33.147772+00:00</t>
+          <t>2026-07-08T01:42:03.397359+00:00</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -1768,7 +2532,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-07-07T09:39:33.179929+00:00</t>
+          <t>2026-07-08T01:42:03.353277+00:00</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -2080,7 +2844,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-07-07T09:39:48.182992+00:00</t>
+          <t>2026-07-08T01:42:03.553994+00:00</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -2539,16 +3303,16 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>best-ai-productivity-software</t>
+          <t>best-ai-meeting-tools</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>best ai productivity software</t>
+          <t>best ai meeting tools</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>62.36</v>
+        <v>57.79</v>
       </c>
       <c r="D2" t="n">
         <v>72</v>
@@ -2571,19 +3335,19 @@
         <v>80</v>
       </c>
       <c r="J2" t="n">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="K2" t="n">
-        <v>89.5</v>
+        <v>65.5</v>
       </c>
       <c r="L2" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M2" t="n">
         <v>100</v>
       </c>
       <c r="N2" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="O2" t="n">
         <v>79</v>
@@ -2598,7 +3362,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>ready</t>
+          <t>needs enrichment</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -2608,12 +3372,12 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>["Notion", "Gamma", "Notion AI"]</t>
+          <t>["Reclaim AI"]</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\best-ai-productivity-software</t>
+          <t>D:\AFFILATE BOT\data\research\best-ai-meeting-tools</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish ready daily articles 2026-07-13
</commit_message>
<xml_diff>
--- a/data/master_dashboard.xlsx
+++ b/data/master_dashboard.xlsx
@@ -462,7 +462,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -472,7 +472,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>8</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6">
@@ -482,7 +482,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>11</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>11</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10">
@@ -1440,7 +1440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U9"/>
+  <dimension ref="A1:U11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1553,12 +1553,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>agent-skills-review-2026</t>
+          <t>best-ai-productivity-software</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>agent-skills Review 2026</t>
+          <t>best ai productivity software</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1568,28 +1568,28 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-07-08T22:18:36.107297+00:00</t>
+          <t>2026-07-10T06:55:09.428985+00:00</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>["verified source score failed", "knowledge freshness failed", "AI review failed"]</t>
+          <t>["human approval missing"]</t>
         </is>
       </c>
       <c r="F2" t="b">
         <v>1</v>
       </c>
       <c r="G2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -1609,39 +1609,39 @@
         <v>1</v>
       </c>
       <c r="P2" t="n">
-        <v>57.15</v>
+        <v>61.35</v>
       </c>
       <c r="Q2" t="n">
-        <v>59.22</v>
+        <v>56.35</v>
       </c>
       <c r="R2" t="b">
         <v>0</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>https://smileaireviewhub.com/agent-skills-review-2026/</t>
+          <t>https://smileaireviewhub.com/best-ai-productivity-software/</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>agent-skills Review 2026: Pricing, Pros, Cons</t>
+          <t>best ai productivity software 2026: Pricing, Pros, Cons</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>Independent agent-skills Review 2026 guide with pricing checks, pros, cons, alternatives, FAQs, and buyer-focused workflow advice.</t>
+          <t>Independent best ai productivity software guide with pricing checks, pros, cons, alternatives, FAQs, and buyer-focused workflow advice.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>meetily-review-2026</t>
+          <t>agent-skills-review-2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>meetily Review 2026</t>
+          <t>agent-skills Review 2026</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1651,7 +1651,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-07-08T22:19:22.916589+00:00</t>
+          <t>2026-07-08T22:18:36.107297+00:00</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -1695,36 +1695,36 @@
         <v>57.15</v>
       </c>
       <c r="Q3" t="n">
-        <v>59.48</v>
+        <v>59.22</v>
       </c>
       <c r="R3" t="b">
         <v>0</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>https://smileaireviewhub.com/meetily-review-2026/</t>
+          <t>https://smileaireviewhub.com/agent-skills-review-2026/</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>meetily Review 2026: Pricing, Pros, Cons</t>
+          <t>agent-skills Review 2026: Pricing, Pros, Cons</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Independent meetily Review 2026 guide with pricing checks, pros, cons, alternatives, FAQs, and buyer-focused workflow advice.</t>
+          <t>Independent agent-skills Review 2026 guide with pricing checks, pros, cons, alternatives, FAQs, and buyer-focused workflow advice.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>system-prompts-leaks-review-2026</t>
+          <t>meetily-review-2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>system_prompts_leaks Review 2026</t>
+          <t>meetily Review 2026</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1734,7 +1734,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-07-08T22:19:57.113612+00:00</t>
+          <t>2026-07-08T22:19:22.916589+00:00</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -1778,36 +1778,36 @@
         <v>57.15</v>
       </c>
       <c r="Q4" t="n">
-        <v>58.73</v>
+        <v>59.48</v>
       </c>
       <c r="R4" t="b">
         <v>0</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>https://smileaireviewhub.com/system-prompts-leaks-review-2026/</t>
+          <t>https://smileaireviewhub.com/meetily-review-2026/</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>system_prompts_leaks Review 2026: Pricing, Pros, Cons</t>
+          <t>meetily Review 2026: Pricing, Pros, Cons</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>Independent system_prompts_leaks Review 2026 guide with pricing checks, pros, cons, alternatives, FAQs, and buyer-focused workflow advice.</t>
+          <t>Independent meetily Review 2026 guide with pricing checks, pros, cons, alternatives, FAQs, and buyer-focused workflow advice.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ai-job-search-review-2026</t>
+          <t>system-prompts-leaks-review-2026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ai-job-search Review 2026</t>
+          <t>system_prompts_leaks Review 2026</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1817,7 +1817,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-07-08T22:20:05.263013+00:00</t>
+          <t>2026-07-08T22:19:57.113612+00:00</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -1861,36 +1861,36 @@
         <v>57.15</v>
       </c>
       <c r="Q5" t="n">
-        <v>59.25</v>
+        <v>58.73</v>
       </c>
       <c r="R5" t="b">
         <v>0</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>https://smileaireviewhub.com/ai-job-search-review-2026/</t>
+          <t>https://smileaireviewhub.com/system-prompts-leaks-review-2026/</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>ai-job-search Review 2026: Pricing, Pros, Cons</t>
+          <t>system_prompts_leaks Review 2026: Pricing, Pros, Cons</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>Independent ai-job-search Review 2026 guide with pricing checks, pros, cons, alternatives, FAQs, and buyer-focused workflow advice.</t>
+          <t>Independent system_prompts_leaks Review 2026 guide with pricing checks, pros, cons, alternatives, FAQs, and buyer-focused workflow advice.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>officecli-review-2026</t>
+          <t>ai-job-search-review-2026</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>OfficeCLI Review 2026</t>
+          <t>ai-job-search Review 2026</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1900,7 +1900,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-07-08T22:20:12.568712+00:00</t>
+          <t>2026-07-08T22:20:05.263013+00:00</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1944,36 +1944,36 @@
         <v>57.15</v>
       </c>
       <c r="Q6" t="n">
-        <v>59.32</v>
+        <v>59.25</v>
       </c>
       <c r="R6" t="b">
         <v>0</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>https://smileaireviewhub.com/officecli-review-2026/</t>
+          <t>https://smileaireviewhub.com/ai-job-search-review-2026/</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>OfficeCLI Review 2026: Pricing, Pros, Cons</t>
+          <t>ai-job-search Review 2026: Pricing, Pros, Cons</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>Independent OfficeCLI Review 2026 guide with pricing checks, pros, cons, alternatives, FAQs, and buyer-focused workflow advice.</t>
+          <t>Independent ai-job-search Review 2026 guide with pricing checks, pros, cons, alternatives, FAQs, and buyer-focused workflow advice.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>cubesandbox-review-2026</t>
+          <t>officecli-review-2026</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CubeSandbox Review 2026</t>
+          <t>OfficeCLI Review 2026</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-07-08T22:20:19.442623+00:00</t>
+          <t>2026-07-08T22:20:12.568712+00:00</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -2027,36 +2027,36 @@
         <v>57.15</v>
       </c>
       <c r="Q7" t="n">
-        <v>59.17</v>
+        <v>59.32</v>
       </c>
       <c r="R7" t="b">
         <v>0</v>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>https://smileaireviewhub.com/cubesandbox-review-2026/</t>
+          <t>https://smileaireviewhub.com/officecli-review-2026/</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>CubeSandbox Review 2026: Pricing, Pros, Cons</t>
+          <t>OfficeCLI Review 2026: Pricing, Pros, Cons</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>Independent CubeSandbox Review 2026 guide with pricing checks, pros, cons, alternatives, FAQs, and buyer-focused workflow advice.</t>
+          <t>Independent OfficeCLI Review 2026 guide with pricing checks, pros, cons, alternatives, FAQs, and buyer-focused workflow advice.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>skills-review-2026</t>
+          <t>cubesandbox-review-2026</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>skills Review 2026</t>
+          <t>CubeSandbox Review 2026</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -2066,7 +2066,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-07-08T22:20:27.803787+00:00</t>
+          <t>2026-07-08T22:20:19.442623+00:00</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -2110,36 +2110,36 @@
         <v>57.15</v>
       </c>
       <c r="Q8" t="n">
-        <v>59.56</v>
+        <v>59.17</v>
       </c>
       <c r="R8" t="b">
         <v>0</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>https://smileaireviewhub.com/skills-review-2026/</t>
+          <t>https://smileaireviewhub.com/cubesandbox-review-2026/</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>skills Review 2026: Pricing, Pros, Cons</t>
+          <t>CubeSandbox Review 2026: Pricing, Pros, Cons</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>Independent skills Review 2026 guide with pricing checks, pros, cons, alternatives, FAQs, and buyer-focused workflow advice.</t>
+          <t>Independent CubeSandbox Review 2026 guide with pricing checks, pros, cons, alternatives, FAQs, and buyer-focused workflow advice.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>companies-are-buying-ai-tools-that-doesn-t-mean-they-know-what-to-do-with-them</t>
+          <t>skills-review-2026</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Companies are buying AI tools. That doesn't mean they know what to do with them.</t>
+          <t>skills Review 2026</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2149,7 +2149,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-07-08T22:20:34.366057+00:00</t>
+          <t>2026-07-08T22:20:27.803787+00:00</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -2193,24 +2193,190 @@
         <v>57.15</v>
       </c>
       <c r="Q9" t="n">
+        <v>59.56</v>
+      </c>
+      <c r="R9" t="b">
+        <v>0</v>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>https://smileaireviewhub.com/skills-review-2026/</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>skills Review 2026: Pricing, Pros, Cons</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Independent skills Review 2026 guide with pricing checks, pros, cons, alternatives, FAQs, and buyer-focused workflow advice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>companies-are-buying-ai-tools-that-doesn-t-mean-they-know-what-to-do-with-them</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Companies are buying AI tools. That doesn't mean they know what to do with them.</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2026-07-08T22:20:34.366057+00:00</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>["verified source score failed", "knowledge freshness failed", "AI review failed"]</t>
+        </is>
+      </c>
+      <c r="F10" t="b">
+        <v>1</v>
+      </c>
+      <c r="G10" t="b">
+        <v>0</v>
+      </c>
+      <c r="H10" t="b">
+        <v>0</v>
+      </c>
+      <c r="I10" t="b">
+        <v>0</v>
+      </c>
+      <c r="J10" t="b">
+        <v>1</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="L10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M10" t="b">
+        <v>1</v>
+      </c>
+      <c r="N10" t="b">
+        <v>1</v>
+      </c>
+      <c r="O10" t="b">
+        <v>1</v>
+      </c>
+      <c r="P10" t="n">
+        <v>57.15</v>
+      </c>
+      <c r="Q10" t="n">
         <v>64.19</v>
       </c>
-      <c r="R9" t="b">
-        <v>0</v>
-      </c>
-      <c r="S9" t="inlineStr">
+      <c r="R10" t="b">
+        <v>0</v>
+      </c>
+      <c r="S10" t="inlineStr">
         <is>
           <t>https://smileaireviewhub.com/companies-are-buying-ai-tools-that-doesn-t-mean-they-know-what-to-do-with-them/</t>
         </is>
       </c>
-      <c r="T9" t="inlineStr">
+      <c r="T10" t="inlineStr">
         <is>
           <t>Companies are buying AI tools. That doesn't mean they kn</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr">
+      <c r="U10" t="inlineStr">
         <is>
           <t>Independent Companies are buying AI tools. That doesn't mean they know what to do with them. guide with pricing checks, pros, cons, alternatives, FAQs, an.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>best-ai-meeting-software</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>best ai meeting software</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2026-07-10T06:55:08.118027+00:00</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>["AI review failed", "human approval missing"]</t>
+        </is>
+      </c>
+      <c r="F11" t="b">
+        <v>1</v>
+      </c>
+      <c r="G11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I11" t="b">
+        <v>0</v>
+      </c>
+      <c r="J11" t="b">
+        <v>0</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="L11" t="b">
+        <v>0</v>
+      </c>
+      <c r="M11" t="b">
+        <v>1</v>
+      </c>
+      <c r="N11" t="b">
+        <v>1</v>
+      </c>
+      <c r="O11" t="b">
+        <v>1</v>
+      </c>
+      <c r="P11" t="n">
+        <v>58.55</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>57.05</v>
+      </c>
+      <c r="R11" t="b">
+        <v>0</v>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>https://smileaireviewhub.com/best-ai-meeting-software/</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>best ai meeting software 2026: Pricing, Pros, Cons</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>Independent best ai meeting software guide with pricing checks, pros, cons, alternatives, FAQs, and buyer-focused workflow advice.</t>
         </is>
       </c>
     </row>
@@ -2225,15 +2391,78 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>empty</t>
-        </is>
-      </c>
+          <t>slug</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>required</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>reviewed_at</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>approved_at</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>approved_by</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>best-ai-productivity-software</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>best ai productivity software</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="D2" t="b">
+        <v>1</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-07-10T06:55:09.408911+00:00</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2890,39 +3119,39 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>best ai voice software</t>
+          <t>The SaaS Apocalypse Is Real. Causal AI Is the Escape Route</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>best-ai-voice-software</t>
+          <t>the-saas-apocalypse-is-real-causal-ai-is-the-escape-route</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D9" t="n">
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F9" t="n">
         <v>1</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>competitor coverage is limited</t>
+          <t>trusted sources are thin; official sources are insufficiently verified; pricing sources need verification; affiliate sources need verification; competitor coverage is limited; entity extraction needs richer tool coverage; official_docs_score 0.0 below 20.0; pricing_source_score 0.0 below 20.0; affiliate_source_score 0.0 below 10.0; total_verified_source_score 0.0 below 35.0; verified_sources 0 below 1; official_verified_sources 0 below 1</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-07-07T09:39:48.204668+00:00</t>
+          <t>2026-07-07T09:39:48.139069+00:00</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -2931,76 +3160,76 @@
         </is>
       </c>
       <c r="K9" t="n">
-        <v>57.79</v>
+        <v>43.71</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-07-07T09:38:58.035479+00:00</t>
+          <t>2026-07-07T09:38:58.325848+00:00</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-07-07T09:38:58.300049+00:00</t>
+          <t>2026-07-07T09:38:58.485959+00:00</t>
         </is>
       </c>
       <c r="N9" t="n">
-        <v>57.79</v>
+        <v>43.71</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["trusted sources are thin", "official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>["competitor_article"]</t>
+          <t>["official_docs", "pricing_page", "affiliate_program_page", "release_notes", "competitor_article"]</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>verified</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="R9" t="n">
-        <v>92</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>The SaaS Apocalypse Is Real. Causal AI Is the Escape Route</t>
+          <t>Impartner Redefines Partner Marketing Automation with Full Automation, AdTech and AI to Drive Measurable Revenue</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>the-saas-apocalypse-is-real-causal-ai-is-the-escape-route</t>
+          <t>impartner-redefines-partner-marketing-automation-with-full-automation-adtech-and-ai-to-drive-measurable-revenue</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="D10" t="n">
         <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F10" t="n">
         <v>1</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>trusted sources are thin; official sources are insufficiently verified; pricing sources need verification; affiliate sources need verification; competitor coverage is limited; entity extraction needs richer tool coverage; official_docs_score 0.0 below 20.0; pricing_source_score 0.0 below 20.0; affiliate_source_score 0.0 below 10.0; total_verified_source_score 0.0 below 35.0; verified_sources 0 below 1; official_verified_sources 0 below 1</t>
+          <t>competitor coverage is limited; official_docs_score 0.0 below 20.0; pricing_source_score 0.0 below 20.0; affiliate_source_score 0.0 below 10.0; total_verified_source_score 0.0 below 35.0; verified_sources 0 below 2; official_verified_sources 0 below 1</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-07-07T09:39:48.139069+00:00</t>
+          <t>2026-07-13T07:43:34.242629+00:00</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -3009,29 +3238,11 @@
         </is>
       </c>
       <c r="K10" t="n">
-        <v>43.71</v>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>2026-07-07T09:38:58.325848+00:00</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>2026-07-07T09:38:58.485959+00:00</t>
-        </is>
-      </c>
-      <c r="N10" t="n">
-        <v>43.71</v>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>["trusted sources are thin", "official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
-        </is>
+        <v>62.43</v>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>["official_docs", "pricing_page", "affiliate_program_page", "release_notes", "competitor_article"]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
@@ -3046,16 +3257,16 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Impartner Redefines Partner Marketing Automation with Full Automation, AdTech and AI to Drive Measurable Revenue</t>
+          <t>AI coding tokens could soon cost as much as salaries</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>impartner-redefines-partner-marketing-automation-with-full-automation-adtech-and-ai-to-drive-measurable-revenue</t>
+          <t>ai-coding-tokens-could-soon-cost-as-much-as-salaries</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D11" t="n">
         <v>1</v>
@@ -3068,17 +3279,17 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>competitor coverage is limited; official_docs_score 0.0 below 20.0; pricing_source_score 0.0 below 20.0; affiliate_source_score 0.0 below 10.0; total_verified_source_score 0.0 below 35.0; verified_sources 0 below 1; official_verified_sources 0 below 1</t>
+          <t>official sources are insufficiently verified; pricing sources need verification; affiliate sources need verification; competitor coverage is limited; official_docs_score 0.0 below 20.0; pricing_source_score 0.0 below 20.0; affiliate_source_score 0.0 below 10.0; total_verified_source_score 0.0 below 35.0; verified_sources 0 below 1; official_verified_sources 0 below 1</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-07-07T09:39:48.231145+00:00</t>
+          <t>2026-07-07T09:39:48.338049+00:00</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -3087,11 +3298,11 @@
         </is>
       </c>
       <c r="K11" t="n">
-        <v>62.43</v>
+        <v>54.86</v>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["official_docs", "pricing_page", "affiliate_program_page", "release_notes", "competitor_article"]</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
@@ -3303,58 +3514,58 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>best-ai-meeting-tools</t>
+          <t>how-ai-is-upending-saas-tools</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>best ai meeting tools</t>
+          <t>How AI is upending SaaS tools</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>57.79</v>
+        <v>55.14</v>
       </c>
       <c r="D2" t="n">
         <v>72</v>
       </c>
       <c r="E2" t="n">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="F2" t="n">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>["affiliate_networks", "integrations", "use_cases", "target_audience", "competitors"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H2" t="n">
         <v>68</v>
       </c>
       <c r="I2" t="n">
+        <v>70</v>
+      </c>
+      <c r="J2" t="n">
+        <v>45</v>
+      </c>
+      <c r="K2" t="n">
+        <v>85</v>
+      </c>
+      <c r="L2" t="n">
+        <v>20</v>
+      </c>
+      <c r="M2" t="n">
+        <v>20</v>
+      </c>
+      <c r="N2" t="n">
+        <v>10</v>
+      </c>
+      <c r="O2" t="n">
+        <v>70</v>
+      </c>
+      <c r="P2" t="n">
         <v>80</v>
       </c>
-      <c r="J2" t="n">
-        <v>49</v>
-      </c>
-      <c r="K2" t="n">
-        <v>65.5</v>
-      </c>
-      <c r="L2" t="n">
-        <v>99</v>
-      </c>
-      <c r="M2" t="n">
-        <v>100</v>
-      </c>
-      <c r="N2" t="n">
-        <v>99</v>
-      </c>
-      <c r="O2" t="n">
-        <v>79</v>
-      </c>
-      <c r="P2" t="n">
-        <v>91.59999999999999</v>
-      </c>
       <c r="Q2" t="inlineStr">
         <is>
           <t>verified</t>
@@ -3367,17 +3578,17 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>["Reclaim AI"]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\best-ai-meeting-tools</t>
+          <t>D:\AFFILATE BOT\data\research\how-ai-is-upending-saas-tools</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish ready daily articles 2026-07-15
</commit_message>
<xml_diff>
--- a/data/master_dashboard.xlsx
+++ b/data/master_dashboard.xlsx
@@ -462,7 +462,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5">
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>31</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>31</v>
+        <v>38</v>
       </c>
     </row>
     <row r="10">
@@ -3401,7 +3401,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U2"/>
+  <dimension ref="A1:U11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3514,36 +3514,36 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>how-ai-is-upending-saas-tools</t>
+          <t>how-ai-is-upending-saas-tools-comparison-and-alternatives</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>How AI is upending SaaS tools</t>
+          <t>How AI is upending SaaS tools comparison and alternatives</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>55.14</v>
+        <v>58.86</v>
       </c>
       <c r="D2" t="n">
         <v>72</v>
       </c>
       <c r="E2" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="F2" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H2" t="n">
         <v>68</v>
       </c>
       <c r="I2" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J2" t="n">
         <v>45</v>
@@ -3578,17 +3578,746 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
+          <t>["competitor coverage is limited"]</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>D:\AFFILATE BOT\data\research\how-ai-is-upending-saas-tools-comparison-and-alternatives</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>automation-without-understanding-comparison-and-alternatives</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Automation Without Understanding comparison and alternatives</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>68</v>
+      </c>
+      <c r="D3" t="n">
+        <v>72</v>
+      </c>
+      <c r="E3" t="n">
+        <v>100</v>
+      </c>
+      <c r="F3" t="n">
+        <v>100</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>["use_cases", "target_audience", "affiliate_networks", "competitors", "integrations"]</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>68</v>
+      </c>
+      <c r="I3" t="n">
+        <v>80</v>
+      </c>
+      <c r="J3" t="n">
+        <v>61</v>
+      </c>
+      <c r="K3" t="n">
+        <v>85</v>
+      </c>
+      <c r="L3" t="n">
+        <v>20</v>
+      </c>
+      <c r="M3" t="n">
+        <v>20</v>
+      </c>
+      <c r="N3" t="n">
+        <v>10</v>
+      </c>
+      <c r="O3" t="n">
+        <v>70</v>
+      </c>
+      <c r="P3" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>ready</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>["competitor coverage is limited"]</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>["Make", "Zapier"]</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>D:\AFFILATE BOT\data\research\automation-without-understanding-comparison-and-alternatives</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>mastra-ai-review-2026-comparison-and-alternatives</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Mastra AI Review 2026 comparison and alternatives</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>54.43</v>
+      </c>
+      <c r="D4" t="n">
+        <v>72</v>
+      </c>
+      <c r="E4" t="n">
+        <v>52</v>
+      </c>
+      <c r="F4" t="n">
+        <v>52</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>68</v>
+      </c>
+      <c r="I4" t="n">
+        <v>80</v>
+      </c>
+      <c r="J4" t="n">
+        <v>45</v>
+      </c>
+      <c r="K4" t="n">
+        <v>54</v>
+      </c>
+      <c r="L4" t="n">
+        <v>20</v>
+      </c>
+      <c r="M4" t="n">
+        <v>20</v>
+      </c>
+      <c r="N4" t="n">
+        <v>10</v>
+      </c>
+      <c r="O4" t="n">
+        <v>70</v>
+      </c>
+      <c r="P4" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>needs enrichment</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>["competitor coverage is limited"]</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>D:\AFFILATE BOT\data\research\mastra-ai-review-2026-comparison-and-alternatives</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>n8n-ai-agents-review-2026-comparison-and-alternatives</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>n8n AI Agents Review 2026 comparison and alternatives</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>54.43</v>
+      </c>
+      <c r="D5" t="n">
+        <v>72</v>
+      </c>
+      <c r="E5" t="n">
+        <v>52</v>
+      </c>
+      <c r="F5" t="n">
+        <v>52</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>68</v>
+      </c>
+      <c r="I5" t="n">
+        <v>80</v>
+      </c>
+      <c r="J5" t="n">
+        <v>45</v>
+      </c>
+      <c r="K5" t="n">
+        <v>54</v>
+      </c>
+      <c r="L5" t="n">
+        <v>20</v>
+      </c>
+      <c r="M5" t="n">
+        <v>20</v>
+      </c>
+      <c r="N5" t="n">
+        <v>10</v>
+      </c>
+      <c r="O5" t="n">
+        <v>70</v>
+      </c>
+      <c r="P5" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>needs enrichment</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>["competitor coverage is limited"]</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>D:\AFFILATE BOT\data\research\n8n-ai-agents-review-2026-comparison-and-alternatives</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>pydantic-ai-review-2026-comparison-and-alternatives</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Pydantic AI Review 2026 comparison and alternatives</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>54.43</v>
+      </c>
+      <c r="D6" t="n">
+        <v>72</v>
+      </c>
+      <c r="E6" t="n">
+        <v>52</v>
+      </c>
+      <c r="F6" t="n">
+        <v>52</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>68</v>
+      </c>
+      <c r="I6" t="n">
+        <v>80</v>
+      </c>
+      <c r="J6" t="n">
+        <v>45</v>
+      </c>
+      <c r="K6" t="n">
+        <v>54</v>
+      </c>
+      <c r="L6" t="n">
+        <v>20</v>
+      </c>
+      <c r="M6" t="n">
+        <v>20</v>
+      </c>
+      <c r="N6" t="n">
+        <v>10</v>
+      </c>
+      <c r="O6" t="n">
+        <v>70</v>
+      </c>
+      <c r="P6" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>needs enrichment</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>["competitor coverage is limited"]</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>D:\AFFILATE BOT\data\research\pydantic-ai-review-2026-comparison-and-alternatives</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>best-ai-voice-software-comparison-and-alternatives</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>best ai voice software comparison and alternatives</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>63.5</v>
+      </c>
+      <c r="D7" t="n">
+        <v>72</v>
+      </c>
+      <c r="E7" t="n">
+        <v>76</v>
+      </c>
+      <c r="F7" t="n">
+        <v>76</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>["affiliate_networks", "integrations", "competitors", "use_cases", "target_audience"]</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>68</v>
+      </c>
+      <c r="I7" t="n">
+        <v>80</v>
+      </c>
+      <c r="J7" t="n">
+        <v>49</v>
+      </c>
+      <c r="K7" t="n">
+        <v>89.5</v>
+      </c>
+      <c r="L7" t="n">
+        <v>99</v>
+      </c>
+      <c r="M7" t="n">
+        <v>100</v>
+      </c>
+      <c r="N7" t="n">
+        <v>99</v>
+      </c>
+      <c r="O7" t="n">
+        <v>79</v>
+      </c>
+      <c r="P7" t="n">
+        <v>92</v>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>ready</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>["competitor coverage is limited"]</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>["ElevenLabs"]</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>D:\AFFILATE BOT\data\research\best-ai-voice-software-comparison-and-alternatives</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>project-nomad-review-2026-comparison-and-alternatives</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>project-nomad Review 2026 comparison and alternatives</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>55.43</v>
+      </c>
+      <c r="D8" t="n">
+        <v>72</v>
+      </c>
+      <c r="E8" t="n">
+        <v>52</v>
+      </c>
+      <c r="F8" t="n">
+        <v>52</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>68</v>
+      </c>
+      <c r="I8" t="n">
+        <v>80</v>
+      </c>
+      <c r="J8" t="n">
+        <v>45</v>
+      </c>
+      <c r="K8" t="n">
+        <v>61</v>
+      </c>
+      <c r="L8" t="n">
+        <v>20</v>
+      </c>
+      <c r="M8" t="n">
+        <v>20</v>
+      </c>
+      <c r="N8" t="n">
+        <v>10</v>
+      </c>
+      <c r="O8" t="n">
+        <v>70</v>
+      </c>
+      <c r="P8" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>needs enrichment</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>["competitor coverage is limited"]</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>D:\AFFILATE BOT\data\research\project-nomad-review-2026-comparison-and-alternatives</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>how-ai-is-upending-saas-tools-pricing</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>How AI is upending SaaS tools pricing</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>55.14</v>
+      </c>
+      <c r="D9" t="n">
+        <v>72</v>
+      </c>
+      <c r="E9" t="n">
+        <v>36</v>
+      </c>
+      <c r="F9" t="n">
+        <v>36</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>68</v>
+      </c>
+      <c r="I9" t="n">
+        <v>70</v>
+      </c>
+      <c r="J9" t="n">
+        <v>45</v>
+      </c>
+      <c r="K9" t="n">
+        <v>85</v>
+      </c>
+      <c r="L9" t="n">
+        <v>20</v>
+      </c>
+      <c r="M9" t="n">
+        <v>20</v>
+      </c>
+      <c r="N9" t="n">
+        <v>10</v>
+      </c>
+      <c r="O9" t="n">
+        <v>70</v>
+      </c>
+      <c r="P9" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>needs enrichment</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
           <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="T9" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>D:\AFFILATE BOT\data\research\how-ai-is-upending-saas-tools</t>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>D:\AFFILATE BOT\data\research\how-ai-is-upending-saas-tools-pricing</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>impartner-redefines-partner-marketing-automation-with-full-automation-adtech-and-ai-to-drive-measurable-revenue-pricing</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Impartner Redefines Partner Marketing Automation with Full Automation, AdTech and AI to Drive Measurable Revenue pricing</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>64.29000000000001</v>
+      </c>
+      <c r="D10" t="n">
+        <v>72</v>
+      </c>
+      <c r="E10" t="n">
+        <v>84</v>
+      </c>
+      <c r="F10" t="n">
+        <v>84</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>["use_cases", "target_audience", "affiliate_networks", "competitors", "integrations"]</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>68</v>
+      </c>
+      <c r="I10" t="n">
+        <v>70</v>
+      </c>
+      <c r="J10" t="n">
+        <v>61</v>
+      </c>
+      <c r="K10" t="n">
+        <v>85</v>
+      </c>
+      <c r="L10" t="n">
+        <v>20</v>
+      </c>
+      <c r="M10" t="n">
+        <v>20</v>
+      </c>
+      <c r="N10" t="n">
+        <v>10</v>
+      </c>
+      <c r="O10" t="n">
+        <v>70</v>
+      </c>
+      <c r="P10" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>ready</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>["competitor coverage is limited"]</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>["Make", "AdCreative AI", "Zapier"]</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>D:\AFFILATE BOT\data\research\impartner-redefines-partner-marketing-automation-with-full-automation-adtech-and-ai-to-drive-measurable-revenue-pricing</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>migrating-a-production-ai-agent-to-gpt-5-6-2-2x-faster-27-cheaper-pricing</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Migrating a production AI agent to GPT-5.6: 2.2x faster, 27% cheaper pricing</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>55.14</v>
+      </c>
+      <c r="D11" t="n">
+        <v>72</v>
+      </c>
+      <c r="E11" t="n">
+        <v>36</v>
+      </c>
+      <c r="F11" t="n">
+        <v>36</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>68</v>
+      </c>
+      <c r="I11" t="n">
+        <v>70</v>
+      </c>
+      <c r="J11" t="n">
+        <v>45</v>
+      </c>
+      <c r="K11" t="n">
+        <v>85</v>
+      </c>
+      <c r="L11" t="n">
+        <v>20</v>
+      </c>
+      <c r="M11" t="n">
+        <v>20</v>
+      </c>
+      <c r="N11" t="n">
+        <v>10</v>
+      </c>
+      <c r="O11" t="n">
+        <v>70</v>
+      </c>
+      <c r="P11" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>needs enrichment</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>D:\AFFILATE BOT\data\research\migrating-a-production-ai-agent-to-gpt-5-6-2-2x-faster-27-cheaper-pricing</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish ready daily articles 2026-07-16
</commit_message>
<xml_diff>
--- a/data/master_dashboard.xlsx
+++ b/data/master_dashboard.xlsx
@@ -472,7 +472,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6">
@@ -492,7 +492,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>32</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8">
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>38</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>38</v>
+        <v>44</v>
       </c>
     </row>
     <row r="10">
@@ -2217,12 +2217,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>companies-are-buying-ai-tools-that-doesn-t-mean-they-know-what-to-do-with-them</t>
+          <t>best-ai-meeting-software</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Companies are buying AI tools. That doesn't mean they know what to do with them.</t>
+          <t>best ai meeting software</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -2232,28 +2232,28 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-07-08T22:20:34.366057+00:00</t>
+          <t>2026-07-10T06:55:08.118027+00:00</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>["verified source score failed", "knowledge freshness failed", "AI review failed"]</t>
+          <t>["AI review failed", "human approval missing"]</t>
         </is>
       </c>
       <c r="F10" t="b">
         <v>1</v>
       </c>
       <c r="G10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I10" t="b">
         <v>0</v>
       </c>
       <c r="J10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -2273,39 +2273,39 @@
         <v>1</v>
       </c>
       <c r="P10" t="n">
-        <v>57.15</v>
+        <v>58.55</v>
       </c>
       <c r="Q10" t="n">
-        <v>64.19</v>
+        <v>57.05</v>
       </c>
       <c r="R10" t="b">
         <v>0</v>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>https://smileaireviewhub.com/companies-are-buying-ai-tools-that-doesn-t-mean-they-know-what-to-do-with-them/</t>
+          <t>https://smileaireviewhub.com/best-ai-meeting-software/</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>Companies are buying AI tools. That doesn't mean they kn</t>
+          <t>best ai meeting software 2026: Pricing, Pros, Cons</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>Independent Companies are buying AI tools. That doesn't mean they know what to do with them. guide with pricing checks, pros, cons, alternatives, FAQs, an.</t>
+          <t>Independent best ai meeting software guide with pricing checks, pros, cons, alternatives, FAQs, and buyer-focused workflow advice.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>best-ai-meeting-software</t>
+          <t>best-ai-meeting-tools</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>best ai meeting software</t>
+          <t>best ai meeting tools</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -2315,7 +2315,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-07-10T06:55:08.118027+00:00</t>
+          <t>2026-07-10T06:55:08.751450+00:00</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -2359,24 +2359,24 @@
         <v>58.55</v>
       </c>
       <c r="Q11" t="n">
-        <v>57.05</v>
+        <v>57.31</v>
       </c>
       <c r="R11" t="b">
         <v>0</v>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>https://smileaireviewhub.com/best-ai-meeting-software/</t>
+          <t>https://smileaireviewhub.com/best-ai-meeting-tools/</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>best ai meeting software 2026: Pricing, Pros, Cons</t>
+          <t>best ai meeting tools 2026: Pricing, Pros, Cons</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>Independent best ai meeting software guide with pricing checks, pros, cons, alternatives, FAQs, and buyer-focused workflow advice.</t>
+          <t>Independent best ai meeting tools guide with pricing checks, pros, cons, alternatives, FAQs, and buyer-focused workflow advice.</t>
         </is>
       </c>
     </row>
@@ -2600,12 +2600,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>trusted sources are thin; official sources are insufficiently verified; pricing sources need verification; affiliate sources need verification; competitor coverage is limited; entity extraction needs richer tool coverage; official_docs_score 0.0 below 20.0; pricing_source_score 0.0 below 20.0; affiliate_source_score 0.0 below 10.0; total_verified_source_score 0.0 below 35.0; verified_sources 0 below 1; official_verified_sources 0 below 1</t>
+          <t>trusted sources are thin; official sources are insufficiently verified; pricing sources need verification; affiliate sources need verification; competitor coverage is limited; entity extraction needs richer tool coverage; 0 usable sources below critical minimum 1; research_quality_score 45.14 below initial threshold 50.0; official_docs_score 0.0 below 20.0; pricing_source_score 0.0 below 20.0; affiliate_source_score 0.0 below 10.0; total_verified_source_score 0.0 below 35.0; verified_sources 0 below 2; official_verified_sources 0 below 1; entity_coverage_score 36.0 below initial threshold 40.0; competitor_coverage_score 10.0 below initial threshold 30.0; freshness_score 0.0 below initial threshold 40.0</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-07-08T01:42:03.376492+00:00</t>
+          <t>2026-07-15T22:05:03.930298+00:00</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -2678,12 +2678,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>trusted sources are thin; official sources are insufficiently verified; pricing sources need verification; affiliate sources need verification; competitor coverage is limited; entity extraction needs richer tool coverage; official_docs_score 0.0 below 20.0; pricing_source_score 0.0 below 20.0; affiliate_source_score 0.0 below 10.0; total_verified_source_score 0.0 below 35.0; verified_sources 0 below 1; official_verified_sources 0 below 1</t>
+          <t>trusted sources are thin; official sources are insufficiently verified; pricing sources need verification; affiliate sources need verification; competitor coverage is limited; entity extraction needs richer tool coverage; 0 usable sources below critical minimum 1; research_quality_score 45.14 below initial threshold 50.0; official_docs_score 0.0 below 20.0; pricing_source_score 0.0 below 20.0; affiliate_source_score 0.0 below 10.0; total_verified_source_score 0.0 below 35.0; verified_sources 0 below 2; official_verified_sources 0 below 1; entity_coverage_score 36.0 below initial threshold 40.0; competitor_coverage_score 10.0 below initial threshold 30.0; freshness_score 0.0 below initial threshold 40.0</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-07-08T01:42:03.397359+00:00</t>
+          <t>2026-07-15T22:05:04.963085+00:00</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -2756,12 +2756,12 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>trusted sources are thin; official sources are insufficiently verified; pricing sources need verification; affiliate sources need verification; competitor coverage is limited; entity extraction needs richer tool coverage; official_docs_score 0.0 below 20.0; pricing_source_score 0.0 below 20.0; affiliate_source_score 0.0 below 10.0; total_verified_source_score 0.0 below 35.0; verified_sources 0 below 1; official_verified_sources 0 below 1</t>
+          <t>trusted sources are thin; official sources are insufficiently verified; pricing sources need verification; affiliate sources need verification; competitor coverage is limited; entity extraction needs richer tool coverage; 0 usable sources below critical minimum 1; research_quality_score 45.14 below initial threshold 50.0; official_docs_score 0.0 below 20.0; pricing_source_score 0.0 below 20.0; affiliate_source_score 0.0 below 10.0; total_verified_source_score 0.0 below 35.0; verified_sources 0 below 2; official_verified_sources 0 below 1; entity_coverage_score 36.0 below initial threshold 40.0; competitor_coverage_score 10.0 below initial threshold 30.0; freshness_score 0.0 below initial threshold 40.0</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-07-08T01:42:03.353277+00:00</t>
+          <t>2026-07-15T22:05:02.724397+00:00</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -3073,7 +3073,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-07-08T01:42:03.553994+00:00</t>
+          <t>2026-07-07T09:39:48.182992+00:00</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -3119,39 +3119,39 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>The SaaS Apocalypse Is Real. Causal AI Is the Escape Route</t>
+          <t>best ai voice software</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>the-saas-apocalypse-is-real-causal-ai-is-the-escape-route</t>
+          <t>best-ai-voice-software</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D9" t="n">
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F9" t="n">
         <v>1</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>trusted sources are thin; official sources are insufficiently verified; pricing sources need verification; affiliate sources need verification; competitor coverage is limited; entity extraction needs richer tool coverage; official_docs_score 0.0 below 20.0; pricing_source_score 0.0 below 20.0; affiliate_source_score 0.0 below 10.0; total_verified_source_score 0.0 below 35.0; verified_sources 0 below 1; official_verified_sources 0 below 1</t>
+          <t>competitor coverage is limited</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-07-07T09:39:48.139069+00:00</t>
+          <t>2026-07-07T09:39:48.204668+00:00</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -3160,76 +3160,76 @@
         </is>
       </c>
       <c r="K9" t="n">
-        <v>43.71</v>
+        <v>57.79</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-07-07T09:38:58.325848+00:00</t>
+          <t>2026-07-07T09:38:58.035479+00:00</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-07-07T09:38:58.485959+00:00</t>
+          <t>2026-07-07T09:38:58.300049+00:00</t>
         </is>
       </c>
       <c r="N9" t="n">
-        <v>43.71</v>
+        <v>57.79</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>["trusted sources are thin", "official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>["official_docs", "pricing_page", "affiliate_program_page", "release_notes", "competitor_article"]</t>
+          <t>["competitor_article"]</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="R9" t="n">
-        <v>0</v>
+        <v>92</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Impartner Redefines Partner Marketing Automation with Full Automation, AdTech and AI to Drive Measurable Revenue</t>
+          <t>The SaaS Apocalypse Is Real. Causal AI Is the Escape Route</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>impartner-redefines-partner-marketing-automation-with-full-automation-adtech-and-ai-to-drive-measurable-revenue</t>
+          <t>the-saas-apocalypse-is-real-causal-ai-is-the-escape-route</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="D10" t="n">
         <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F10" t="n">
         <v>1</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>competitor coverage is limited; official_docs_score 0.0 below 20.0; pricing_source_score 0.0 below 20.0; affiliate_source_score 0.0 below 10.0; total_verified_source_score 0.0 below 35.0; verified_sources 0 below 2; official_verified_sources 0 below 1</t>
+          <t>trusted sources are thin; official sources are insufficiently verified; pricing sources need verification; affiliate sources need verification; competitor coverage is limited; entity extraction needs richer tool coverage; official_docs_score 0.0 below 20.0; pricing_source_score 0.0 below 20.0; affiliate_source_score 0.0 below 10.0; total_verified_source_score 0.0 below 35.0; verified_sources 0 below 1; official_verified_sources 0 below 1</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-07-13T07:43:34.242629+00:00</t>
+          <t>2026-07-07T09:39:48.139069+00:00</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -3238,11 +3238,29 @@
         </is>
       </c>
       <c r="K10" t="n">
-        <v>62.43</v>
+        <v>43.71</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-07-07T09:38:58.325848+00:00</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>2026-07-07T09:38:58.485959+00:00</t>
+        </is>
+      </c>
+      <c r="N10" t="n">
+        <v>43.71</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>["trusted sources are thin", "official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+        </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["official_docs", "pricing_page", "affiliate_program_page", "release_notes", "competitor_article"]</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
@@ -3257,16 +3275,16 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>AI coding tokens could soon cost as much as salaries</t>
+          <t>Impartner Redefines Partner Marketing Automation with Full Automation, AdTech and AI to Drive Measurable Revenue</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ai-coding-tokens-could-soon-cost-as-much-as-salaries</t>
+          <t>impartner-redefines-partner-marketing-automation-with-full-automation-adtech-and-ai-to-drive-measurable-revenue</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D11" t="n">
         <v>1</v>
@@ -3279,17 +3297,17 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>official sources are insufficiently verified; pricing sources need verification; affiliate sources need verification; competitor coverage is limited; official_docs_score 0.0 below 20.0; pricing_source_score 0.0 below 20.0; affiliate_source_score 0.0 below 10.0; total_verified_source_score 0.0 below 35.0; verified_sources 0 below 1; official_verified_sources 0 below 1</t>
+          <t>competitor coverage is limited; official_docs_score 0.0 below 20.0; pricing_source_score 0.0 below 20.0; affiliate_source_score 0.0 below 10.0; total_verified_source_score 0.0 below 35.0; verified_sources 0 below 1; official_verified_sources 0 below 1</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-07-07T09:39:48.338049+00:00</t>
+          <t>2026-07-07T09:39:48.231145+00:00</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -3298,11 +3316,11 @@
         </is>
       </c>
       <c r="K11" t="n">
-        <v>54.86</v>
+        <v>62.43</v>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>["official_docs", "pricing_page", "affiliate_program_page", "release_notes", "competitor_article"]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
@@ -3514,42 +3532,42 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>how-ai-is-upending-saas-tools-comparison-and-alternatives</t>
+          <t>new-ai-tools-by-ifttt</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>How AI is upending SaaS tools comparison and alternatives</t>
+          <t>New AI tools by IFTTT</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>58.86</v>
+        <v>51.71</v>
       </c>
       <c r="D2" t="n">
         <v>72</v>
       </c>
       <c r="E2" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="F2" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H2" t="n">
         <v>68</v>
       </c>
       <c r="I2" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J2" t="n">
         <v>45</v>
       </c>
       <c r="K2" t="n">
-        <v>85</v>
+        <v>61</v>
       </c>
       <c r="L2" t="n">
         <v>20</v>
@@ -3578,7 +3596,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -3588,32 +3606,32 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\how-ai-is-upending-saas-tools-comparison-and-alternatives</t>
+          <t>D:\AFFILATE BOT\data\research\new-ai-tools-by-ifttt</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>automation-without-understanding-comparison-and-alternatives</t>
+          <t>ai-in-healthcare-marketing-moving-from-automation-to-intelligent-engagement</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Automation Without Understanding comparison and alternatives</t>
+          <t>AI In Healthcare Marketing: Moving From Automation To Intelligent Engagement</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>68</v>
+        <v>64.29000000000001</v>
       </c>
       <c r="D3" t="n">
         <v>72</v>
       </c>
       <c r="E3" t="n">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="F3" t="n">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -3624,7 +3642,7 @@
         <v>68</v>
       </c>
       <c r="I3" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J3" t="n">
         <v>61</v>
@@ -3664,54 +3682,54 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>["Make", "Zapier"]</t>
+          <t>["Make", "AdCreative AI", "Zapier"]</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\automation-without-understanding-comparison-and-alternatives</t>
+          <t>D:\AFFILATE BOT\data\research\ai-in-healthcare-marketing-moving-from-automation-to-intelligent-engagement</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>mastra-ai-review-2026-comparison-and-alternatives</t>
+          <t>how-to-overcome-real-world-challenges-in-ai-marketing-automation</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Mastra AI Review 2026 comparison and alternatives</t>
+          <t>How To Overcome Real-World Challenges In AI Marketing Automation</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>54.43</v>
+        <v>64.29000000000001</v>
       </c>
       <c r="D4" t="n">
         <v>72</v>
       </c>
       <c r="E4" t="n">
-        <v>52</v>
+        <v>84</v>
       </c>
       <c r="F4" t="n">
-        <v>52</v>
+        <v>84</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+          <t>["use_cases", "target_audience", "affiliate_networks", "competitors", "integrations"]</t>
         </is>
       </c>
       <c r="H4" t="n">
         <v>68</v>
       </c>
       <c r="I4" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J4" t="n">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="K4" t="n">
-        <v>54</v>
+        <v>85</v>
       </c>
       <c r="L4" t="n">
         <v>20</v>
@@ -3735,7 +3753,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>needs enrichment</t>
+          <t>ready</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -3745,54 +3763,54 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["Make", "AdCreative AI", "Zapier"]</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\mastra-ai-review-2026-comparison-and-alternatives</t>
+          <t>D:\AFFILATE BOT\data\research\how-to-overcome-real-world-challenges-in-ai-marketing-automation</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>n8n-ai-agents-review-2026-comparison-and-alternatives</t>
+          <t>reco-launches-industry-first-ai-agent-security-to-tackle-agent-sprawl-across-saas</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>n8n AI Agents Review 2026 comparison and alternatives</t>
+          <t>Reco Launches Industry-First AI Agent Security to Tackle Agent Sprawl Across SaaS</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>54.43</v>
+        <v>51.71</v>
       </c>
       <c r="D5" t="n">
         <v>72</v>
       </c>
       <c r="E5" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="F5" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H5" t="n">
         <v>68</v>
       </c>
       <c r="I5" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J5" t="n">
         <v>45</v>
       </c>
       <c r="K5" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="L5" t="n">
         <v>20</v>
@@ -3821,7 +3839,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -3831,49 +3849,49 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\n8n-ai-agents-review-2026-comparison-and-alternatives</t>
+          <t>D:\AFFILATE BOT\data\research\reco-launches-industry-first-ai-agent-security-to-tackle-agent-sprawl-across-saas</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>pydantic-ai-review-2026-comparison-and-alternatives</t>
+          <t>microsoft-study-finds-ai-coding-agents-lift-pull-requests-by-24</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Pydantic AI Review 2026 comparison and alternatives</t>
+          <t>Microsoft Study Finds AI Coding Agents Lift Pull Requests by 24%</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>54.43</v>
+        <v>64.29000000000001</v>
       </c>
       <c r="D6" t="n">
         <v>72</v>
       </c>
       <c r="E6" t="n">
-        <v>52</v>
+        <v>84</v>
       </c>
       <c r="F6" t="n">
-        <v>52</v>
+        <v>84</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+          <t>["use_cases", "target_audience", "affiliate_networks", "integrations", "competitors"]</t>
         </is>
       </c>
       <c r="H6" t="n">
         <v>68</v>
       </c>
       <c r="I6" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J6" t="n">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="K6" t="n">
-        <v>54</v>
+        <v>85</v>
       </c>
       <c r="L6" t="n">
         <v>20</v>
@@ -3897,7 +3915,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>needs enrichment</t>
+          <t>ready</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -3907,41 +3925,41 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["Cursor", "GitHub Copilot", "Windsurf"]</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\pydantic-ai-review-2026-comparison-and-alternatives</t>
+          <t>D:\AFFILATE BOT\data\research\microsoft-study-finds-ai-coding-agents-lift-pull-requests-by-24</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>best-ai-voice-software-comparison-and-alternatives</t>
+          <t>top-10-marketing-automation-software-platforms-for-businesses-in-2026</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>best ai voice software comparison and alternatives</t>
+          <t>Top 10 Marketing Automation Software Platforms for Businesses in 2026</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>63.5</v>
+        <v>65.70999999999999</v>
       </c>
       <c r="D7" t="n">
         <v>72</v>
       </c>
       <c r="E7" t="n">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="F7" t="n">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>["affiliate_networks", "integrations", "competitors", "use_cases", "target_audience"]</t>
+          <t>["use_cases", "target_audience", "affiliate_networks", "competitors", "integrations"]</t>
         </is>
       </c>
       <c r="H7" t="n">
@@ -3951,25 +3969,25 @@
         <v>80</v>
       </c>
       <c r="J7" t="n">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="K7" t="n">
-        <v>89.5</v>
+        <v>85</v>
       </c>
       <c r="L7" t="n">
-        <v>99</v>
+        <v>20</v>
       </c>
       <c r="M7" t="n">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="N7" t="n">
-        <v>99</v>
+        <v>10</v>
       </c>
       <c r="O7" t="n">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="P7" t="n">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -3988,54 +4006,54 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>["ElevenLabs"]</t>
+          <t>["Make", "AdCreative AI", "Zapier"]</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\best-ai-voice-software-comparison-and-alternatives</t>
+          <t>D:\AFFILATE BOT\data\research\top-10-marketing-automation-software-platforms-for-businesses-in-2026</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>project-nomad-review-2026-comparison-and-alternatives</t>
+          <t>most-companies-have-ai-tools-but-many-don-t-rewire-themselves-for-ai</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>project-nomad Review 2026 comparison and alternatives</t>
+          <t>Most Companies Have AI Tools, But Many Don't Rewire Themselves For AI</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>55.43</v>
+        <v>55.14</v>
       </c>
       <c r="D8" t="n">
         <v>72</v>
       </c>
       <c r="E8" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="F8" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H8" t="n">
         <v>68</v>
       </c>
       <c r="I8" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J8" t="n">
         <v>45</v>
       </c>
       <c r="K8" t="n">
-        <v>61</v>
+        <v>85</v>
       </c>
       <c r="L8" t="n">
         <v>20</v>
@@ -4064,7 +4082,7 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -4074,23 +4092,23 @@
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\project-nomad-review-2026-comparison-and-alternatives</t>
+          <t>D:\AFFILATE BOT\data\research\most-companies-have-ai-tools-but-many-don-t-rewire-themselves-for-ai</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>how-ai-is-upending-saas-tools-pricing</t>
+          <t>companies-are-buying-ai-tools-that-doesn-t-mean-they-know-what-to-do-with-them</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>How AI is upending SaaS tools pricing</t>
+          <t>Companies are buying AI tools. That doesn't mean they know what to do with them.</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>55.14</v>
+        <v>51.71</v>
       </c>
       <c r="D9" t="n">
         <v>72</v>
@@ -4116,7 +4134,7 @@
         <v>45</v>
       </c>
       <c r="K9" t="n">
-        <v>85</v>
+        <v>61</v>
       </c>
       <c r="L9" t="n">
         <v>20</v>
@@ -4155,49 +4173,49 @@
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\how-ai-is-upending-saas-tools-pricing</t>
+          <t>D:\AFFILATE BOT\data\research\companies-are-buying-ai-tools-that-doesn-t-mean-they-know-what-to-do-with-them</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>impartner-redefines-partner-marketing-automation-with-full-automation-adtech-and-ai-to-drive-measurable-revenue-pricing</t>
+          <t>review-by-eddie-ai</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Impartner Redefines Partner Marketing Automation with Full Automation, AdTech and AI to Drive Measurable Revenue pricing</t>
+          <t>Review by Eddie AI</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>64.29000000000001</v>
+        <v>54.14</v>
       </c>
       <c r="D10" t="n">
         <v>72</v>
       </c>
       <c r="E10" t="n">
-        <v>84</v>
+        <v>36</v>
       </c>
       <c r="F10" t="n">
-        <v>84</v>
+        <v>36</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>["use_cases", "target_audience", "affiliate_networks", "competitors", "integrations"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H10" t="n">
         <v>68</v>
       </c>
       <c r="I10" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J10" t="n">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="K10" t="n">
-        <v>85</v>
+        <v>68</v>
       </c>
       <c r="L10" t="n">
         <v>20</v>
@@ -4221,38 +4239,38 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>ready</t>
+          <t>needs enrichment</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>["Make", "AdCreative AI", "Zapier"]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\impartner-redefines-partner-marketing-automation-with-full-automation-adtech-and-ai-to-drive-measurable-revenue-pricing</t>
+          <t>D:\AFFILATE BOT\data\research\review-by-eddie-ai</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>migrating-a-production-ai-agent-to-gpt-5-6-2-2x-faster-27-cheaper-pricing</t>
+          <t>airi-review-2026</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Migrating a production AI agent to GPT-5.6: 2.2x faster, 27% cheaper pricing</t>
+          <t>airi Review 2026</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>55.14</v>
+        <v>52.14</v>
       </c>
       <c r="D11" t="n">
         <v>72</v>
@@ -4272,13 +4290,13 @@
         <v>68</v>
       </c>
       <c r="I11" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J11" t="n">
         <v>45</v>
       </c>
       <c r="K11" t="n">
-        <v>85</v>
+        <v>54</v>
       </c>
       <c r="L11" t="n">
         <v>20</v>
@@ -4317,7 +4335,7 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\migrating-a-production-ai-agent-to-gpt-5-6-2-2x-faster-27-cheaper-pricing</t>
+          <t>D:\AFFILATE BOT\data\research\airi-review-2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish ready daily articles 2026-07-17
</commit_message>
<xml_diff>
--- a/data/master_dashboard.xlsx
+++ b/data/master_dashboard.xlsx
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>44</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>44</v>
+        <v>54</v>
       </c>
     </row>
     <row r="10">
@@ -3532,16 +3532,16 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>new-ai-tools-by-ifttt</t>
+          <t>best-new-ai-tools-by-ifttt-workflows-and-use-cases</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>New AI tools by IFTTT</t>
+          <t>best New AI tools by IFTTT workflows and use cases</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>51.71</v>
+        <v>53.14</v>
       </c>
       <c r="D2" t="n">
         <v>72</v>
@@ -3561,7 +3561,7 @@
         <v>68</v>
       </c>
       <c r="I2" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J2" t="n">
         <v>45</v>
@@ -3606,23 +3606,23 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\new-ai-tools-by-ifttt</t>
+          <t>D:\AFFILATE BOT\data\research\best-new-ai-tools-by-ifttt-workflows-and-use-cases</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ai-in-healthcare-marketing-moving-from-automation-to-intelligent-engagement</t>
+          <t>best-ai-in-healthcare-marketing-moving-from-automation-to-intelligent-engagement-workflows-and-use-cases</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>AI In Healthcare Marketing: Moving From Automation To Intelligent Engagement</t>
+          <t>best AI In Healthcare Marketing: Moving From Automation To Intelligent Engagement workflows and use cases</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>64.29000000000001</v>
+        <v>65.70999999999999</v>
       </c>
       <c r="D3" t="n">
         <v>72</v>
@@ -3642,7 +3642,7 @@
         <v>68</v>
       </c>
       <c r="I3" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J3" t="n">
         <v>61</v>
@@ -3687,19 +3687,19 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\ai-in-healthcare-marketing-moving-from-automation-to-intelligent-engagement</t>
+          <t>D:\AFFILATE BOT\data\research\best-ai-in-healthcare-marketing-moving-from-automation-to-intelligent-engagement-workflows-and-use-cases</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>how-to-overcome-real-world-challenges-in-ai-marketing-automation</t>
+          <t>best-how-to-overcome-real-world-challenges-in-ai-marketing-automation-workflows-and-use-cases</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>How To Overcome Real-World Challenges In AI Marketing Automation</t>
+          <t>best How To Overcome Real-World Challenges In AI Marketing Automation workflows and use cases</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -3768,23 +3768,23 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\how-to-overcome-real-world-challenges-in-ai-marketing-automation</t>
+          <t>D:\AFFILATE BOT\data\research\best-how-to-overcome-real-world-challenges-in-ai-marketing-automation-workflows-and-use-cases</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>reco-launches-industry-first-ai-agent-security-to-tackle-agent-sprawl-across-saas</t>
+          <t>best-reco-launches-industry-first-ai-agent-security-to-tackle-agent-sprawl-across-saas-workflows-and-use-cases</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Reco Launches Industry-First AI Agent Security to Tackle Agent Sprawl Across SaaS</t>
+          <t>best Reco Launches Industry-First AI Agent Security to Tackle Agent Sprawl Across SaaS workflows and use cases</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>51.71</v>
+        <v>53.14</v>
       </c>
       <c r="D5" t="n">
         <v>72</v>
@@ -3804,7 +3804,7 @@
         <v>68</v>
       </c>
       <c r="I5" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J5" t="n">
         <v>45</v>
@@ -3849,23 +3849,23 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\reco-launches-industry-first-ai-agent-security-to-tackle-agent-sprawl-across-saas</t>
+          <t>D:\AFFILATE BOT\data\research\best-reco-launches-industry-first-ai-agent-security-to-tackle-agent-sprawl-across-saas-workflows-and-use-cases</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>microsoft-study-finds-ai-coding-agents-lift-pull-requests-by-24</t>
+          <t>best-microsoft-study-finds-ai-coding-agents-lift-pull-requests-by-24-workflows-and-use-cases</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Microsoft Study Finds AI Coding Agents Lift Pull Requests by 24%</t>
+          <t>best Microsoft Study Finds AI Coding Agents Lift Pull Requests by 24% workflows and use cases</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>64.29000000000001</v>
+        <v>65.70999999999999</v>
       </c>
       <c r="D6" t="n">
         <v>72</v>
@@ -3885,7 +3885,7 @@
         <v>68</v>
       </c>
       <c r="I6" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J6" t="n">
         <v>61</v>
@@ -3930,19 +3930,19 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\microsoft-study-finds-ai-coding-agents-lift-pull-requests-by-24</t>
+          <t>D:\AFFILATE BOT\data\research\best-microsoft-study-finds-ai-coding-agents-lift-pull-requests-by-24-workflows-and-use-cases</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>top-10-marketing-automation-software-platforms-for-businesses-in-2026</t>
+          <t>best-top-10-marketing-automation-software-platforms-for-businesses-in-2026-workflows-and-use-cases</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Top 10 Marketing Automation Software Platforms for Businesses in 2026</t>
+          <t>best Top 10 Marketing Automation Software Platforms for Businesses in 2026 workflows and use cases</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -4011,23 +4011,23 @@
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\top-10-marketing-automation-software-platforms-for-businesses-in-2026</t>
+          <t>D:\AFFILATE BOT\data\research\best-top-10-marketing-automation-software-platforms-for-businesses-in-2026-workflows-and-use-cases</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>most-companies-have-ai-tools-but-many-don-t-rewire-themselves-for-ai</t>
+          <t>best-most-companies-have-ai-tools-but-many-don-t-rewire-themselves-for-ai-workflows-and-use-cases</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Most Companies Have AI Tools, But Many Don't Rewire Themselves For AI</t>
+          <t>best Most Companies Have AI Tools, But Many Don't Rewire Themselves For AI workflows and use cases</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>55.14</v>
+        <v>56.57</v>
       </c>
       <c r="D8" t="n">
         <v>72</v>
@@ -4047,7 +4047,7 @@
         <v>68</v>
       </c>
       <c r="I8" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J8" t="n">
         <v>45</v>
@@ -4092,19 +4092,19 @@
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\most-companies-have-ai-tools-but-many-don-t-rewire-themselves-for-ai</t>
+          <t>D:\AFFILATE BOT\data\research\best-most-companies-have-ai-tools-but-many-don-t-rewire-themselves-for-ai-workflows-and-use-cases</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>companies-are-buying-ai-tools-that-doesn-t-mean-they-know-what-to-do-with-them</t>
+          <t>best-companies-are-buying-ai-tools-that-doesn-t-mean-they-know-what-to-do-with-them-workflows-and-use-cases</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Companies are buying AI tools. That doesn't mean they know what to do with them.</t>
+          <t>best Companies are buying AI tools. That doesn't mean they know what to do with them. workflows and use cases</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -4173,19 +4173,19 @@
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\companies-are-buying-ai-tools-that-doesn-t-mean-they-know-what-to-do-with-them</t>
+          <t>D:\AFFILATE BOT\data\research\best-companies-are-buying-ai-tools-that-doesn-t-mean-they-know-what-to-do-with-them-workflows-and-use-cases</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>review-by-eddie-ai</t>
+          <t>best-review-by-eddie-ai-workflows-and-use-cases</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Review by Eddie AI</t>
+          <t>best Review by Eddie AI workflows and use cases</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -4254,19 +4254,19 @@
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\review-by-eddie-ai</t>
+          <t>D:\AFFILATE BOT\data\research\best-review-by-eddie-ai-workflows-and-use-cases</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>airi-review-2026</t>
+          <t>best-airi-review-2026-workflows-and-use-cases</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>airi Review 2026</t>
+          <t>best airi Review 2026 workflows and use cases</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -4335,7 +4335,7 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\airi-review-2026</t>
+          <t>D:\AFFILATE BOT\data\research\best-airi-review-2026-workflows-and-use-cases</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish ready daily articles 2026-07-18
</commit_message>
<xml_diff>
--- a/data/master_dashboard.xlsx
+++ b/data/master_dashboard.xlsx
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>54</v>
+        <v>63</v>
       </c>
     </row>
     <row r="9">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>54</v>
+        <v>63</v>
       </c>
     </row>
     <row r="10">
@@ -3532,16 +3532,16 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>best-new-ai-tools-by-ifttt-workflows-and-use-cases</t>
+          <t>common-new-ai-tools-by-ifttt-mistakes-and-troubleshooting</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>best New AI tools by IFTTT workflows and use cases</t>
+          <t>common New AI tools by IFTTT mistakes and troubleshooting</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>53.14</v>
+        <v>51.71</v>
       </c>
       <c r="D2" t="n">
         <v>72</v>
@@ -3561,7 +3561,7 @@
         <v>68</v>
       </c>
       <c r="I2" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J2" t="n">
         <v>45</v>
@@ -3606,23 +3606,23 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\best-new-ai-tools-by-ifttt-workflows-and-use-cases</t>
+          <t>D:\AFFILATE BOT\data\research\common-new-ai-tools-by-ifttt-mistakes-and-troubleshooting</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>best-ai-in-healthcare-marketing-moving-from-automation-to-intelligent-engagement-workflows-and-use-cases</t>
+          <t>common-ai-in-healthcare-marketing-moving-from-automation-to-intelligent-engagement-mistakes-and-troubleshooting</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>best AI In Healthcare Marketing: Moving From Automation To Intelligent Engagement workflows and use cases</t>
+          <t>common AI In Healthcare Marketing: Moving From Automation To Intelligent Engagement mistakes and troubleshooting</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>65.70999999999999</v>
+        <v>64.29000000000001</v>
       </c>
       <c r="D3" t="n">
         <v>72</v>
@@ -3642,7 +3642,7 @@
         <v>68</v>
       </c>
       <c r="I3" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J3" t="n">
         <v>61</v>
@@ -3687,19 +3687,19 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\best-ai-in-healthcare-marketing-moving-from-automation-to-intelligent-engagement-workflows-and-use-cases</t>
+          <t>D:\AFFILATE BOT\data\research\common-ai-in-healthcare-marketing-moving-from-automation-to-intelligent-engagement-mistakes-and-troubleshooting</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>best-how-to-overcome-real-world-challenges-in-ai-marketing-automation-workflows-and-use-cases</t>
+          <t>common-how-to-overcome-real-world-challenges-in-ai-marketing-automation-mistakes-and-troubleshooting</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>best How To Overcome Real-World Challenges In AI Marketing Automation workflows and use cases</t>
+          <t>common How To Overcome Real-World Challenges In AI Marketing Automation mistakes and troubleshooting</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -3768,23 +3768,23 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\best-how-to-overcome-real-world-challenges-in-ai-marketing-automation-workflows-and-use-cases</t>
+          <t>D:\AFFILATE BOT\data\research\common-how-to-overcome-real-world-challenges-in-ai-marketing-automation-mistakes-and-troubleshooting</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>best-reco-launches-industry-first-ai-agent-security-to-tackle-agent-sprawl-across-saas-workflows-and-use-cases</t>
+          <t>common-reco-launches-industry-first-ai-agent-security-to-tackle-agent-sprawl-across-saas-mistakes-and-troubleshooting</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>best Reco Launches Industry-First AI Agent Security to Tackle Agent Sprawl Across SaaS workflows and use cases</t>
+          <t>common Reco Launches Industry-First AI Agent Security to Tackle Agent Sprawl Across SaaS mistakes and troubleshooting</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>53.14</v>
+        <v>51.71</v>
       </c>
       <c r="D5" t="n">
         <v>72</v>
@@ -3804,7 +3804,7 @@
         <v>68</v>
       </c>
       <c r="I5" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J5" t="n">
         <v>45</v>
@@ -3849,23 +3849,23 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\best-reco-launches-industry-first-ai-agent-security-to-tackle-agent-sprawl-across-saas-workflows-and-use-cases</t>
+          <t>D:\AFFILATE BOT\data\research\common-reco-launches-industry-first-ai-agent-security-to-tackle-agent-sprawl-across-saas-mistakes-and-troubleshooting</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>best-microsoft-study-finds-ai-coding-agents-lift-pull-requests-by-24-workflows-and-use-cases</t>
+          <t>common-microsoft-study-finds-ai-coding-agents-lift-pull-requests-by-24-mistakes-and-troubleshooting</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>best Microsoft Study Finds AI Coding Agents Lift Pull Requests by 24% workflows and use cases</t>
+          <t>common Microsoft Study Finds AI Coding Agents Lift Pull Requests by 24% mistakes and troubleshooting</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>65.70999999999999</v>
+        <v>64.29000000000001</v>
       </c>
       <c r="D6" t="n">
         <v>72</v>
@@ -3885,7 +3885,7 @@
         <v>68</v>
       </c>
       <c r="I6" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J6" t="n">
         <v>61</v>
@@ -3930,19 +3930,19 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\best-microsoft-study-finds-ai-coding-agents-lift-pull-requests-by-24-workflows-and-use-cases</t>
+          <t>D:\AFFILATE BOT\data\research\common-microsoft-study-finds-ai-coding-agents-lift-pull-requests-by-24-mistakes-and-troubleshooting</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>best-top-10-marketing-automation-software-platforms-for-businesses-in-2026-workflows-and-use-cases</t>
+          <t>common-top-10-marketing-automation-software-platforms-for-businesses-in-2026-mistakes-and-troubleshooting</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>best Top 10 Marketing Automation Software Platforms for Businesses in 2026 workflows and use cases</t>
+          <t>common Top 10 Marketing Automation Software Platforms for Businesses in 2026 mistakes and troubleshooting</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -4011,23 +4011,23 @@
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\best-top-10-marketing-automation-software-platforms-for-businesses-in-2026-workflows-and-use-cases</t>
+          <t>D:\AFFILATE BOT\data\research\common-top-10-marketing-automation-software-platforms-for-businesses-in-2026-mistakes-and-troubleshooting</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>best-most-companies-have-ai-tools-but-many-don-t-rewire-themselves-for-ai-workflows-and-use-cases</t>
+          <t>common-most-companies-have-ai-tools-but-many-don-t-rewire-themselves-for-ai-mistakes-and-troubleshooting</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>best Most Companies Have AI Tools, But Many Don't Rewire Themselves For AI workflows and use cases</t>
+          <t>common Most Companies Have AI Tools, But Many Don't Rewire Themselves For AI mistakes and troubleshooting</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>56.57</v>
+        <v>55.14</v>
       </c>
       <c r="D8" t="n">
         <v>72</v>
@@ -4047,7 +4047,7 @@
         <v>68</v>
       </c>
       <c r="I8" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J8" t="n">
         <v>45</v>
@@ -4092,23 +4092,23 @@
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\best-most-companies-have-ai-tools-but-many-don-t-rewire-themselves-for-ai-workflows-and-use-cases</t>
+          <t>D:\AFFILATE BOT\data\research\common-most-companies-have-ai-tools-but-many-don-t-rewire-themselves-for-ai-mistakes-and-troubleshooting</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>best-companies-are-buying-ai-tools-that-doesn-t-mean-they-know-what-to-do-with-them-workflows-and-use-cases</t>
+          <t>common-review-by-eddie-ai-mistakes-and-troubleshooting</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>best Companies are buying AI tools. That doesn't mean they know what to do with them. workflows and use cases</t>
+          <t>common Review by Eddie AI mistakes and troubleshooting</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>51.71</v>
+        <v>54.14</v>
       </c>
       <c r="D9" t="n">
         <v>72</v>
@@ -4128,13 +4128,13 @@
         <v>68</v>
       </c>
       <c r="I9" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J9" t="n">
         <v>45</v>
       </c>
       <c r="K9" t="n">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="L9" t="n">
         <v>20</v>
@@ -4173,23 +4173,23 @@
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\best-companies-are-buying-ai-tools-that-doesn-t-mean-they-know-what-to-do-with-them-workflows-and-use-cases</t>
+          <t>D:\AFFILATE BOT\data\research\common-review-by-eddie-ai-mistakes-and-troubleshooting</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>best-review-by-eddie-ai-workflows-and-use-cases</t>
+          <t>common-airi-review-2026-mistakes-and-troubleshooting</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>best Review by Eddie AI workflows and use cases</t>
+          <t>common airi Review 2026 mistakes and troubleshooting</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>54.14</v>
+        <v>52.14</v>
       </c>
       <c r="D10" t="n">
         <v>72</v>
@@ -4215,7 +4215,7 @@
         <v>45</v>
       </c>
       <c r="K10" t="n">
-        <v>68</v>
+        <v>54</v>
       </c>
       <c r="L10" t="n">
         <v>20</v>
@@ -4254,23 +4254,23 @@
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\best-review-by-eddie-ai-workflows-and-use-cases</t>
+          <t>D:\AFFILATE BOT\data\research\common-airi-review-2026-mistakes-and-troubleshooting</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>best-airi-review-2026-workflows-and-use-cases</t>
+          <t>best-new-ai-tools-by-ifttt-workflows-and-use-cases</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>best airi Review 2026 workflows and use cases</t>
+          <t>best New AI tools by IFTTT workflows and use cases</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>52.14</v>
+        <v>53.14</v>
       </c>
       <c r="D11" t="n">
         <v>72</v>
@@ -4296,7 +4296,7 @@
         <v>45</v>
       </c>
       <c r="K11" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="L11" t="n">
         <v>20</v>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\best-airi-review-2026-workflows-and-use-cases</t>
+          <t>D:\AFFILATE BOT\data\research\best-new-ai-tools-by-ifttt-workflows-and-use-cases</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish ready daily articles 2026-07-19
</commit_message>
<xml_diff>
--- a/data/master_dashboard.xlsx
+++ b/data/master_dashboard.xlsx
@@ -472,7 +472,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6">
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="9">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="10">
@@ -3532,36 +3532,36 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>common-new-ai-tools-by-ifttt-mistakes-and-troubleshooting</t>
+          <t>is-new-ai-tools-by-ifttt-worth-it-for-small-business</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>common New AI tools by IFTTT mistakes and troubleshooting</t>
+          <t>is New AI tools by IFTTT worth it for small business</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>51.71</v>
+        <v>55.43</v>
       </c>
       <c r="D2" t="n">
         <v>72</v>
       </c>
       <c r="E2" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="F2" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H2" t="n">
         <v>68</v>
       </c>
       <c r="I2" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J2" t="n">
         <v>45</v>
@@ -3596,7 +3596,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -3606,32 +3606,32 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\common-new-ai-tools-by-ifttt-mistakes-and-troubleshooting</t>
+          <t>D:\AFFILATE BOT\data\research\is-new-ai-tools-by-ifttt-worth-it-for-small-business</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>common-ai-in-healthcare-marketing-moving-from-automation-to-intelligent-engagement-mistakes-and-troubleshooting</t>
+          <t>is-ai-in-healthcare-marketing-moving-from-automation-to-intelligent-engagement-worth-it-for-small-business</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>common AI In Healthcare Marketing: Moving From Automation To Intelligent Engagement mistakes and troubleshooting</t>
+          <t>is AI In Healthcare Marketing: Moving From Automation To Intelligent Engagement worth it for small business</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>64.29000000000001</v>
+        <v>68</v>
       </c>
       <c r="D3" t="n">
         <v>72</v>
       </c>
       <c r="E3" t="n">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="F3" t="n">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -3642,7 +3642,7 @@
         <v>68</v>
       </c>
       <c r="I3" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J3" t="n">
         <v>61</v>
@@ -3687,32 +3687,32 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\common-ai-in-healthcare-marketing-moving-from-automation-to-intelligent-engagement-mistakes-and-troubleshooting</t>
+          <t>D:\AFFILATE BOT\data\research\is-ai-in-healthcare-marketing-moving-from-automation-to-intelligent-engagement-worth-it-for-small-business</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>common-how-to-overcome-real-world-challenges-in-ai-marketing-automation-mistakes-and-troubleshooting</t>
+          <t>is-how-to-overcome-real-world-challenges-in-ai-marketing-automation-worth-it-for-small-business</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>common How To Overcome Real-World Challenges In AI Marketing Automation mistakes and troubleshooting</t>
+          <t>is How To Overcome Real-World Challenges In AI Marketing Automation worth it for small business</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>64.29000000000001</v>
+        <v>66.56999999999999</v>
       </c>
       <c r="D4" t="n">
         <v>72</v>
       </c>
       <c r="E4" t="n">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="F4" t="n">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -3768,43 +3768,43 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\common-how-to-overcome-real-world-challenges-in-ai-marketing-automation-mistakes-and-troubleshooting</t>
+          <t>D:\AFFILATE BOT\data\research\is-how-to-overcome-real-world-challenges-in-ai-marketing-automation-worth-it-for-small-business</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>common-reco-launches-industry-first-ai-agent-security-to-tackle-agent-sprawl-across-saas-mistakes-and-troubleshooting</t>
+          <t>is-reco-launches-industry-first-ai-agent-security-to-tackle-agent-sprawl-across-saas-worth-it-for-small-business</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>common Reco Launches Industry-First AI Agent Security to Tackle Agent Sprawl Across SaaS mistakes and troubleshooting</t>
+          <t>is Reco Launches Industry-First AI Agent Security to Tackle Agent Sprawl Across SaaS worth it for small business</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>51.71</v>
+        <v>55.43</v>
       </c>
       <c r="D5" t="n">
         <v>72</v>
       </c>
       <c r="E5" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="F5" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H5" t="n">
         <v>68</v>
       </c>
       <c r="I5" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J5" t="n">
         <v>45</v>
@@ -3839,7 +3839,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -3849,32 +3849,32 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\common-reco-launches-industry-first-ai-agent-security-to-tackle-agent-sprawl-across-saas-mistakes-and-troubleshooting</t>
+          <t>D:\AFFILATE BOT\data\research\is-reco-launches-industry-first-ai-agent-security-to-tackle-agent-sprawl-across-saas-worth-it-for-small-business</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>common-microsoft-study-finds-ai-coding-agents-lift-pull-requests-by-24-mistakes-and-troubleshooting</t>
+          <t>is-microsoft-study-finds-ai-coding-agents-lift-pull-requests-by-24-worth-it-for-small-business</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>common Microsoft Study Finds AI Coding Agents Lift Pull Requests by 24% mistakes and troubleshooting</t>
+          <t>is Microsoft Study Finds AI Coding Agents Lift Pull Requests by 24% worth it for small business</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>64.29000000000001</v>
+        <v>68</v>
       </c>
       <c r="D6" t="n">
         <v>72</v>
       </c>
       <c r="E6" t="n">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="F6" t="n">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -3885,7 +3885,7 @@
         <v>68</v>
       </c>
       <c r="I6" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J6" t="n">
         <v>61</v>
@@ -3930,32 +3930,32 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\common-microsoft-study-finds-ai-coding-agents-lift-pull-requests-by-24-mistakes-and-troubleshooting</t>
+          <t>D:\AFFILATE BOT\data\research\is-microsoft-study-finds-ai-coding-agents-lift-pull-requests-by-24-worth-it-for-small-business</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>common-top-10-marketing-automation-software-platforms-for-businesses-in-2026-mistakes-and-troubleshooting</t>
+          <t>is-top-10-marketing-automation-software-platforms-for-businesses-in-2026-worth-it-for-small-business</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>common Top 10 Marketing Automation Software Platforms for Businesses in 2026 mistakes and troubleshooting</t>
+          <t>is Top 10 Marketing Automation Software Platforms for Businesses in 2026 worth it for small business</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>65.70999999999999</v>
+        <v>68</v>
       </c>
       <c r="D7" t="n">
         <v>72</v>
       </c>
       <c r="E7" t="n">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="F7" t="n">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -4011,43 +4011,43 @@
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\common-top-10-marketing-automation-software-platforms-for-businesses-in-2026-mistakes-and-troubleshooting</t>
+          <t>D:\AFFILATE BOT\data\research\is-top-10-marketing-automation-software-platforms-for-businesses-in-2026-worth-it-for-small-business</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>common-most-companies-have-ai-tools-but-many-don-t-rewire-themselves-for-ai-mistakes-and-troubleshooting</t>
+          <t>is-most-companies-have-ai-tools-but-many-don-t-rewire-themselves-for-ai-worth-it-for-small-business</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>common Most Companies Have AI Tools, But Many Don't Rewire Themselves For AI mistakes and troubleshooting</t>
+          <t>is Most Companies Have AI Tools, But Many Don't Rewire Themselves For AI worth it for small business</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>55.14</v>
+        <v>58.86</v>
       </c>
       <c r="D8" t="n">
         <v>72</v>
       </c>
       <c r="E8" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="F8" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H8" t="n">
         <v>68</v>
       </c>
       <c r="I8" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J8" t="n">
         <v>45</v>
@@ -4082,7 +4082,7 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -4092,49 +4092,49 @@
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\common-most-companies-have-ai-tools-but-many-don-t-rewire-themselves-for-ai-mistakes-and-troubleshooting</t>
+          <t>D:\AFFILATE BOT\data\research\is-most-companies-have-ai-tools-but-many-don-t-rewire-themselves-for-ai-worth-it-for-small-business</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>common-review-by-eddie-ai-mistakes-and-troubleshooting</t>
+          <t>is-companies-are-buying-ai-tools-that-doesn-t-mean-they-know-what-to-do-with-them-worth-it-for-small-business</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>common Review by Eddie AI mistakes and troubleshooting</t>
+          <t>is Companies are buying AI tools. That doesn't mean they know what to do with them. worth it for small business</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>54.14</v>
+        <v>54</v>
       </c>
       <c r="D9" t="n">
         <v>72</v>
       </c>
       <c r="E9" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="F9" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H9" t="n">
         <v>68</v>
       </c>
       <c r="I9" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J9" t="n">
         <v>45</v>
       </c>
       <c r="K9" t="n">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="L9" t="n">
         <v>20</v>
@@ -4163,7 +4163,7 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -4173,36 +4173,36 @@
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\common-review-by-eddie-ai-mistakes-and-troubleshooting</t>
+          <t>D:\AFFILATE BOT\data\research\is-companies-are-buying-ai-tools-that-doesn-t-mean-they-know-what-to-do-with-them-worth-it-for-small-business</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>common-airi-review-2026-mistakes-and-troubleshooting</t>
+          <t>is-review-by-eddie-ai-worth-it-for-small-business</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>common airi Review 2026 mistakes and troubleshooting</t>
+          <t>is Review by Eddie AI worth it for small business</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>52.14</v>
+        <v>56.43</v>
       </c>
       <c r="D10" t="n">
         <v>72</v>
       </c>
       <c r="E10" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="F10" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H10" t="n">
@@ -4215,7 +4215,7 @@
         <v>45</v>
       </c>
       <c r="K10" t="n">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="L10" t="n">
         <v>20</v>
@@ -4244,7 +4244,7 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -4254,36 +4254,36 @@
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\common-airi-review-2026-mistakes-and-troubleshooting</t>
+          <t>D:\AFFILATE BOT\data\research\is-review-by-eddie-ai-worth-it-for-small-business</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>best-new-ai-tools-by-ifttt-workflows-and-use-cases</t>
+          <t>is-airi-review-2026-worth-it-for-small-business</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>best New AI tools by IFTTT workflows and use cases</t>
+          <t>is airi Review 2026 worth it for small business</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>53.14</v>
+        <v>54.43</v>
       </c>
       <c r="D11" t="n">
         <v>72</v>
       </c>
       <c r="E11" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="F11" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H11" t="n">
@@ -4296,7 +4296,7 @@
         <v>45</v>
       </c>
       <c r="K11" t="n">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="L11" t="n">
         <v>20</v>
@@ -4325,7 +4325,7 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -4335,7 +4335,7 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\best-new-ai-tools-by-ifttt-workflows-and-use-cases</t>
+          <t>D:\AFFILATE BOT\data\research\is-airi-review-2026-worth-it-for-small-business</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish ready daily articles 2026-07-20
</commit_message>
<xml_diff>
--- a/data/master_dashboard.xlsx
+++ b/data/master_dashboard.xlsx
@@ -472,7 +472,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6">
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
     </row>
     <row r="10">
@@ -3532,42 +3532,42 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>is-new-ai-tools-by-ifttt-worth-it-for-small-business</t>
+          <t>atlassian-team-launches-ai-native-jira-tools-for-the-full-development-workflow</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>is New AI tools by IFTTT worth it for small business</t>
+          <t>Atlassian (TEAM) Launches AI Native Jira Tools For The Full Development Workflow</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>55.43</v>
+        <v>51.86</v>
       </c>
       <c r="D2" t="n">
         <v>72</v>
       </c>
       <c r="E2" t="n">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="F2" t="n">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H2" t="n">
         <v>68</v>
       </c>
       <c r="I2" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J2" t="n">
         <v>45</v>
       </c>
       <c r="K2" t="n">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="L2" t="n">
         <v>20</v>
@@ -3596,7 +3596,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -3606,49 +3606,49 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\is-new-ai-tools-by-ifttt-worth-it-for-small-business</t>
+          <t>D:\AFFILATE BOT\data\research\atlassian-team-launches-ai-native-jira-tools-for-the-full-development-workflow</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>is-ai-in-healthcare-marketing-moving-from-automation-to-intelligent-engagement-worth-it-for-small-business</t>
+          <t>free-ai-tools</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>is AI In Healthcare Marketing: Moving From Automation To Intelligent Engagement worth it for small business</t>
+          <t>Free AI Tools</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>68</v>
+        <v>51.71</v>
       </c>
       <c r="D3" t="n">
         <v>72</v>
       </c>
       <c r="E3" t="n">
-        <v>100</v>
+        <v>36</v>
       </c>
       <c r="F3" t="n">
-        <v>100</v>
+        <v>36</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>["use_cases", "target_audience", "affiliate_networks", "competitors", "integrations"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H3" t="n">
         <v>68</v>
       </c>
       <c r="I3" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J3" t="n">
+        <v>45</v>
+      </c>
+      <c r="K3" t="n">
         <v>61</v>
-      </c>
-      <c r="K3" t="n">
-        <v>85</v>
       </c>
       <c r="L3" t="n">
         <v>20</v>
@@ -3672,64 +3672,64 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>ready</t>
+          <t>needs enrichment</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>["Make", "AdCreative AI", "Zapier"]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\is-ai-in-healthcare-marketing-moving-from-automation-to-intelligent-engagement-worth-it-for-small-business</t>
+          <t>D:\AFFILATE BOT\data\research\free-ai-tools</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>is-how-to-overcome-real-world-challenges-in-ai-marketing-automation-worth-it-for-small-business</t>
+          <t>wrenai-review-2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>is How To Overcome Real-World Challenges In AI Marketing Automation worth it for small business</t>
+          <t>WrenAI Review 2026</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>66.56999999999999</v>
+        <v>52.14</v>
       </c>
       <c r="D4" t="n">
         <v>72</v>
       </c>
       <c r="E4" t="n">
-        <v>100</v>
+        <v>36</v>
       </c>
       <c r="F4" t="n">
-        <v>100</v>
+        <v>36</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>["use_cases", "target_audience", "affiliate_networks", "competitors", "integrations"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H4" t="n">
         <v>68</v>
       </c>
       <c r="I4" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J4" t="n">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="K4" t="n">
-        <v>85</v>
+        <v>54</v>
       </c>
       <c r="L4" t="n">
         <v>20</v>
@@ -3753,51 +3753,51 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>ready</t>
+          <t>needs enrichment</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>["Make", "AdCreative AI", "Zapier"]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\is-how-to-overcome-real-world-challenges-in-ai-marketing-automation-worth-it-for-small-business</t>
+          <t>D:\AFFILATE BOT\data\research\wrenai-review-2026</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>is-reco-launches-industry-first-ai-agent-security-to-tackle-agent-sprawl-across-saas-worth-it-for-small-business</t>
+          <t>ktransformers-review-2026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>is Reco Launches Industry-First AI Agent Security to Tackle Agent Sprawl Across SaaS worth it for small business</t>
+          <t>ktransformers Review 2026</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>55.43</v>
+        <v>52.14</v>
       </c>
       <c r="D5" t="n">
         <v>72</v>
       </c>
       <c r="E5" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="F5" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H5" t="n">
@@ -3810,7 +3810,7 @@
         <v>45</v>
       </c>
       <c r="K5" t="n">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="L5" t="n">
         <v>20</v>
@@ -3839,7 +3839,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -3849,36 +3849,36 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\is-reco-launches-industry-first-ai-agent-security-to-tackle-agent-sprawl-across-saas-worth-it-for-small-business</t>
+          <t>D:\AFFILATE BOT\data\research\ktransformers-review-2026</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>is-microsoft-study-finds-ai-coding-agents-lift-pull-requests-by-24-worth-it-for-small-business</t>
+          <t>voicebox-review-2026</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>is Microsoft Study Finds AI Coding Agents Lift Pull Requests by 24% worth it for small business</t>
+          <t>voicebox Review 2026</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>68</v>
+        <v>52.14</v>
       </c>
       <c r="D6" t="n">
         <v>72</v>
       </c>
       <c r="E6" t="n">
-        <v>100</v>
+        <v>36</v>
       </c>
       <c r="F6" t="n">
-        <v>100</v>
+        <v>36</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>["use_cases", "target_audience", "affiliate_networks", "integrations", "competitors"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H6" t="n">
@@ -3888,10 +3888,10 @@
         <v>80</v>
       </c>
       <c r="J6" t="n">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="K6" t="n">
-        <v>85</v>
+        <v>54</v>
       </c>
       <c r="L6" t="n">
         <v>20</v>
@@ -3915,51 +3915,51 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>ready</t>
+          <t>needs enrichment</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>["Cursor", "GitHub Copilot", "Windsurf"]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\is-microsoft-study-finds-ai-coding-agents-lift-pull-requests-by-24-worth-it-for-small-business</t>
+          <t>D:\AFFILATE BOT\data\research\voicebox-review-2026</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>is-top-10-marketing-automation-software-platforms-for-businesses-in-2026-worth-it-for-small-business</t>
+          <t>code-review-graph-review-2026</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>is Top 10 Marketing Automation Software Platforms for Businesses in 2026 worth it for small business</t>
+          <t>code-review-graph Review 2026</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>68</v>
+        <v>52.14</v>
       </c>
       <c r="D7" t="n">
         <v>72</v>
       </c>
       <c r="E7" t="n">
-        <v>100</v>
+        <v>36</v>
       </c>
       <c r="F7" t="n">
-        <v>100</v>
+        <v>36</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>["use_cases", "target_audience", "affiliate_networks", "competitors", "integrations"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H7" t="n">
@@ -3969,10 +3969,10 @@
         <v>80</v>
       </c>
       <c r="J7" t="n">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="K7" t="n">
-        <v>85</v>
+        <v>54</v>
       </c>
       <c r="L7" t="n">
         <v>20</v>
@@ -3996,51 +3996,51 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>ready</t>
+          <t>needs enrichment</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>["Make", "AdCreative AI", "Zapier"]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\is-top-10-marketing-automation-software-platforms-for-businesses-in-2026-worth-it-for-small-business</t>
+          <t>D:\AFFILATE BOT\data\research\code-review-graph-review-2026</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>is-most-companies-have-ai-tools-but-many-don-t-rewire-themselves-for-ai-worth-it-for-small-business</t>
+          <t>copilot-sdk-review-2026</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>is Most Companies Have AI Tools, But Many Don't Rewire Themselves For AI worth it for small business</t>
+          <t>copilot-sdk Review 2026</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>58.86</v>
+        <v>52.14</v>
       </c>
       <c r="D8" t="n">
         <v>72</v>
       </c>
       <c r="E8" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="F8" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H8" t="n">
@@ -4053,7 +4053,7 @@
         <v>45</v>
       </c>
       <c r="K8" t="n">
-        <v>85</v>
+        <v>54</v>
       </c>
       <c r="L8" t="n">
         <v>20</v>
@@ -4082,7 +4082,7 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -4092,49 +4092,49 @@
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\is-most-companies-have-ai-tools-but-many-don-t-rewire-themselves-for-ai-worth-it-for-small-business</t>
+          <t>D:\AFFILATE BOT\data\research\copilot-sdk-review-2026</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>is-companies-are-buying-ai-tools-that-doesn-t-mean-they-know-what-to-do-with-them-worth-it-for-small-business</t>
+          <t>posthog-review-2026</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>is Companies are buying AI tools. That doesn't mean they know what to do with them. worth it for small business</t>
+          <t>posthog Review 2026</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>54</v>
+        <v>52.14</v>
       </c>
       <c r="D9" t="n">
         <v>72</v>
       </c>
       <c r="E9" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="F9" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H9" t="n">
         <v>68</v>
       </c>
       <c r="I9" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J9" t="n">
         <v>45</v>
       </c>
       <c r="K9" t="n">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="L9" t="n">
         <v>20</v>
@@ -4163,7 +4163,7 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -4173,36 +4173,36 @@
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\is-companies-are-buying-ai-tools-that-doesn-t-mean-they-know-what-to-do-with-them-worth-it-for-small-business</t>
+          <t>D:\AFFILATE BOT\data\research\posthog-review-2026</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>is-review-by-eddie-ai-worth-it-for-small-business</t>
+          <t>wigolo-review-2026</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>is Review by Eddie AI worth it for small business</t>
+          <t>wigolo Review 2026</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>56.43</v>
+        <v>52.14</v>
       </c>
       <c r="D10" t="n">
         <v>72</v>
       </c>
       <c r="E10" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="F10" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H10" t="n">
@@ -4215,7 +4215,7 @@
         <v>45</v>
       </c>
       <c r="K10" t="n">
-        <v>68</v>
+        <v>54</v>
       </c>
       <c r="L10" t="n">
         <v>20</v>
@@ -4244,7 +4244,7 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -4254,36 +4254,36 @@
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\is-review-by-eddie-ai-worth-it-for-small-business</t>
+          <t>D:\AFFILATE BOT\data\research\wigolo-review-2026</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>is-airi-review-2026-worth-it-for-small-business</t>
+          <t>astrbot-review-2026</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>is airi Review 2026 worth it for small business</t>
+          <t>AstrBot Review 2026</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>54.43</v>
+        <v>52.14</v>
       </c>
       <c r="D11" t="n">
         <v>72</v>
       </c>
       <c r="E11" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="F11" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H11" t="n">
@@ -4325,7 +4325,7 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -4335,7 +4335,7 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\is-airi-review-2026-worth-it-for-small-business</t>
+          <t>D:\AFFILATE BOT\data\research\astrbot-review-2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish ready daily articles 2026-07-22
</commit_message>
<xml_diff>
--- a/data/master_dashboard.xlsx
+++ b/data/master_dashboard.xlsx
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>80</v>
+        <v>89</v>
       </c>
     </row>
     <row r="9">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>80</v>
+        <v>89</v>
       </c>
     </row>
     <row r="10">
@@ -3532,42 +3532,42 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>atlassian-team-launches-ai-native-jira-tools-for-the-full-development-workflow</t>
+          <t>free-ai-tools-comparison-and-alternatives</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Atlassian (TEAM) Launches AI Native Jira Tools For The Full Development Workflow</t>
+          <t>Free AI Tools comparison and alternatives</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>51.86</v>
+        <v>55.43</v>
       </c>
       <c r="D2" t="n">
         <v>72</v>
       </c>
       <c r="E2" t="n">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="F2" t="n">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H2" t="n">
         <v>68</v>
       </c>
       <c r="I2" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J2" t="n">
         <v>45</v>
       </c>
       <c r="K2" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="L2" t="n">
         <v>20</v>
@@ -3596,7 +3596,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -3606,49 +3606,49 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\atlassian-team-launches-ai-native-jira-tools-for-the-full-development-workflow</t>
+          <t>D:\AFFILATE BOT\data\research\free-ai-tools-comparison-and-alternatives</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>free-ai-tools</t>
+          <t>wrenai-review-2026-comparison-and-alternatives</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Free AI Tools</t>
+          <t>WrenAI Review 2026 comparison and alternatives</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>51.71</v>
+        <v>54.43</v>
       </c>
       <c r="D3" t="n">
         <v>72</v>
       </c>
       <c r="E3" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="F3" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H3" t="n">
         <v>68</v>
       </c>
       <c r="I3" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J3" t="n">
         <v>45</v>
       </c>
       <c r="K3" t="n">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="L3" t="n">
         <v>20</v>
@@ -3677,7 +3677,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -3687,36 +3687,36 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\free-ai-tools</t>
+          <t>D:\AFFILATE BOT\data\research\wrenai-review-2026-comparison-and-alternatives</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>wrenai-review-2026</t>
+          <t>ktransformers-review-2026-comparison-and-alternatives</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>WrenAI Review 2026</t>
+          <t>ktransformers Review 2026 comparison and alternatives</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>52.14</v>
+        <v>54.43</v>
       </c>
       <c r="D4" t="n">
         <v>72</v>
       </c>
       <c r="E4" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="F4" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H4" t="n">
@@ -3758,7 +3758,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -3768,36 +3768,36 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\wrenai-review-2026</t>
+          <t>D:\AFFILATE BOT\data\research\ktransformers-review-2026-comparison-and-alternatives</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ktransformers-review-2026</t>
+          <t>voicebox-review-2026-comparison-and-alternatives</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ktransformers Review 2026</t>
+          <t>voicebox Review 2026 comparison and alternatives</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>52.14</v>
+        <v>54.43</v>
       </c>
       <c r="D5" t="n">
         <v>72</v>
       </c>
       <c r="E5" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="F5" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H5" t="n">
@@ -3839,7 +3839,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -3849,36 +3849,36 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\ktransformers-review-2026</t>
+          <t>D:\AFFILATE BOT\data\research\voicebox-review-2026-comparison-and-alternatives</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>voicebox-review-2026</t>
+          <t>code-review-graph-review-2026-comparison-and-alternatives</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>voicebox Review 2026</t>
+          <t>code-review-graph Review 2026 comparison and alternatives</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>52.14</v>
+        <v>54.43</v>
       </c>
       <c r="D6" t="n">
         <v>72</v>
       </c>
       <c r="E6" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="F6" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H6" t="n">
@@ -3920,7 +3920,7 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -3930,36 +3930,36 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\voicebox-review-2026</t>
+          <t>D:\AFFILATE BOT\data\research\code-review-graph-review-2026-comparison-and-alternatives</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>code-review-graph-review-2026</t>
+          <t>copilot-sdk-review-2026-comparison-and-alternatives</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>code-review-graph Review 2026</t>
+          <t>copilot-sdk Review 2026 comparison and alternatives</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>52.14</v>
+        <v>54.43</v>
       </c>
       <c r="D7" t="n">
         <v>72</v>
       </c>
       <c r="E7" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="F7" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H7" t="n">
@@ -4001,7 +4001,7 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -4011,36 +4011,36 @@
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\code-review-graph-review-2026</t>
+          <t>D:\AFFILATE BOT\data\research\copilot-sdk-review-2026-comparison-and-alternatives</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>copilot-sdk-review-2026</t>
+          <t>posthog-review-2026-comparison-and-alternatives</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>copilot-sdk Review 2026</t>
+          <t>posthog Review 2026 comparison and alternatives</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>52.14</v>
+        <v>54.43</v>
       </c>
       <c r="D8" t="n">
         <v>72</v>
       </c>
       <c r="E8" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="F8" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H8" t="n">
@@ -4082,7 +4082,7 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -4092,36 +4092,36 @@
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\copilot-sdk-review-2026</t>
+          <t>D:\AFFILATE BOT\data\research\posthog-review-2026-comparison-and-alternatives</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>posthog-review-2026</t>
+          <t>wigolo-review-2026-comparison-and-alternatives</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>posthog Review 2026</t>
+          <t>wigolo Review 2026 comparison and alternatives</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>52.14</v>
+        <v>54.43</v>
       </c>
       <c r="D9" t="n">
         <v>72</v>
       </c>
       <c r="E9" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="F9" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H9" t="n">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -4173,36 +4173,36 @@
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\posthog-review-2026</t>
+          <t>D:\AFFILATE BOT\data\research\wigolo-review-2026-comparison-and-alternatives</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>wigolo-review-2026</t>
+          <t>astrbot-review-2026-comparison-and-alternatives</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>wigolo Review 2026</t>
+          <t>AstrBot Review 2026 comparison and alternatives</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>52.14</v>
+        <v>54.43</v>
       </c>
       <c r="D10" t="n">
         <v>72</v>
       </c>
       <c r="E10" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="F10" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H10" t="n">
@@ -4244,7 +4244,7 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -4254,23 +4254,23 @@
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\wigolo-review-2026</t>
+          <t>D:\AFFILATE BOT\data\research\astrbot-review-2026-comparison-and-alternatives</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>astrbot-review-2026</t>
+          <t>how-to-implement-free-ai-tools</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>AstrBot Review 2026</t>
+          <t>how to implement Free AI Tools</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>52.14</v>
+        <v>51.71</v>
       </c>
       <c r="D11" t="n">
         <v>72</v>
@@ -4290,13 +4290,13 @@
         <v>68</v>
       </c>
       <c r="I11" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J11" t="n">
         <v>45</v>
       </c>
       <c r="K11" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="L11" t="n">
         <v>20</v>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\astrbot-review-2026</t>
+          <t>D:\AFFILATE BOT\data\research\how-to-implement-free-ai-tools</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish ready daily articles 2026-07-23
</commit_message>
<xml_diff>
--- a/data/master_dashboard.xlsx
+++ b/data/master_dashboard.xlsx
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>89</v>
+        <v>99</v>
       </c>
     </row>
     <row r="9">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>89</v>
+        <v>99</v>
       </c>
     </row>
     <row r="10">
@@ -3532,42 +3532,42 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>free-ai-tools-comparison-and-alternatives</t>
+          <t>atlassian-team-launches-ai-native-jira-tools-for-the-full-development-workflow-pricing-cost-and-roi</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Free AI Tools comparison and alternatives</t>
+          <t>Atlassian (TEAM) Launches AI Native Jira Tools For The Full Development Workflow pricing cost and ROI</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>55.43</v>
+        <v>51.86</v>
       </c>
       <c r="D2" t="n">
         <v>72</v>
       </c>
       <c r="E2" t="n">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="F2" t="n">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H2" t="n">
         <v>68</v>
       </c>
       <c r="I2" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J2" t="n">
         <v>45</v>
       </c>
       <c r="K2" t="n">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="L2" t="n">
         <v>20</v>
@@ -3596,7 +3596,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -3606,49 +3606,49 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\free-ai-tools-comparison-and-alternatives</t>
+          <t>D:\AFFILATE BOT\data\research\atlassian-team-launches-ai-native-jira-tools-for-the-full-development-workflow-pricing-cost-and-roi</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>wrenai-review-2026-comparison-and-alternatives</t>
+          <t>free-ai-tools-pricing-cost-and-roi</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>WrenAI Review 2026 comparison and alternatives</t>
+          <t>Free AI Tools pricing cost and ROI</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>54.43</v>
+        <v>51.71</v>
       </c>
       <c r="D3" t="n">
         <v>72</v>
       </c>
       <c r="E3" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="F3" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H3" t="n">
         <v>68</v>
       </c>
       <c r="I3" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J3" t="n">
         <v>45</v>
       </c>
       <c r="K3" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="L3" t="n">
         <v>20</v>
@@ -3677,7 +3677,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -3687,43 +3687,43 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\wrenai-review-2026-comparison-and-alternatives</t>
+          <t>D:\AFFILATE BOT\data\research\free-ai-tools-pricing-cost-and-roi</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ktransformers-review-2026-comparison-and-alternatives</t>
+          <t>wrenai-review-2026-pricing-cost-and-roi</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ktransformers Review 2026 comparison and alternatives</t>
+          <t>WrenAI Review 2026 pricing cost and ROI</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>54.43</v>
+        <v>50.71</v>
       </c>
       <c r="D4" t="n">
         <v>72</v>
       </c>
       <c r="E4" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="F4" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H4" t="n">
         <v>68</v>
       </c>
       <c r="I4" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J4" t="n">
         <v>45</v>
@@ -3758,7 +3758,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -3768,43 +3768,43 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\ktransformers-review-2026-comparison-and-alternatives</t>
+          <t>D:\AFFILATE BOT\data\research\wrenai-review-2026-pricing-cost-and-roi</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>voicebox-review-2026-comparison-and-alternatives</t>
+          <t>ktransformers-review-2026-pricing-cost-and-roi</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>voicebox Review 2026 comparison and alternatives</t>
+          <t>ktransformers Review 2026 pricing cost and ROI</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>54.43</v>
+        <v>50.71</v>
       </c>
       <c r="D5" t="n">
         <v>72</v>
       </c>
       <c r="E5" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="F5" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H5" t="n">
         <v>68</v>
       </c>
       <c r="I5" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J5" t="n">
         <v>45</v>
@@ -3839,7 +3839,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -3849,43 +3849,43 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\voicebox-review-2026-comparison-and-alternatives</t>
+          <t>D:\AFFILATE BOT\data\research\ktransformers-review-2026-pricing-cost-and-roi</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>code-review-graph-review-2026-comparison-and-alternatives</t>
+          <t>voicebox-review-2026-pricing-cost-and-roi</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>code-review-graph Review 2026 comparison and alternatives</t>
+          <t>voicebox Review 2026 pricing cost and ROI</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>54.43</v>
+        <v>50.71</v>
       </c>
       <c r="D6" t="n">
         <v>72</v>
       </c>
       <c r="E6" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="F6" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H6" t="n">
         <v>68</v>
       </c>
       <c r="I6" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J6" t="n">
         <v>45</v>
@@ -3920,7 +3920,7 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -3930,43 +3930,43 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\code-review-graph-review-2026-comparison-and-alternatives</t>
+          <t>D:\AFFILATE BOT\data\research\voicebox-review-2026-pricing-cost-and-roi</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>copilot-sdk-review-2026-comparison-and-alternatives</t>
+          <t>code-review-graph-review-2026-pricing-cost-and-roi</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>copilot-sdk Review 2026 comparison and alternatives</t>
+          <t>code-review-graph Review 2026 pricing cost and ROI</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>54.43</v>
+        <v>50.71</v>
       </c>
       <c r="D7" t="n">
         <v>72</v>
       </c>
       <c r="E7" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="F7" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H7" t="n">
         <v>68</v>
       </c>
       <c r="I7" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J7" t="n">
         <v>45</v>
@@ -4001,7 +4001,7 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -4011,43 +4011,43 @@
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\copilot-sdk-review-2026-comparison-and-alternatives</t>
+          <t>D:\AFFILATE BOT\data\research\code-review-graph-review-2026-pricing-cost-and-roi</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>posthog-review-2026-comparison-and-alternatives</t>
+          <t>copilot-sdk-review-2026-pricing-cost-and-roi</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>posthog Review 2026 comparison and alternatives</t>
+          <t>copilot-sdk Review 2026 pricing cost and ROI</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>54.43</v>
+        <v>50.71</v>
       </c>
       <c r="D8" t="n">
         <v>72</v>
       </c>
       <c r="E8" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="F8" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H8" t="n">
         <v>68</v>
       </c>
       <c r="I8" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J8" t="n">
         <v>45</v>
@@ -4082,7 +4082,7 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -4092,43 +4092,43 @@
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\posthog-review-2026-comparison-and-alternatives</t>
+          <t>D:\AFFILATE BOT\data\research\copilot-sdk-review-2026-pricing-cost-and-roi</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>wigolo-review-2026-comparison-and-alternatives</t>
+          <t>posthog-review-2026-pricing-cost-and-roi</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>wigolo Review 2026 comparison and alternatives</t>
+          <t>posthog Review 2026 pricing cost and ROI</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>54.43</v>
+        <v>50.71</v>
       </c>
       <c r="D9" t="n">
         <v>72</v>
       </c>
       <c r="E9" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="F9" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H9" t="n">
         <v>68</v>
       </c>
       <c r="I9" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J9" t="n">
         <v>45</v>
@@ -4163,7 +4163,7 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -4173,43 +4173,43 @@
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\wigolo-review-2026-comparison-and-alternatives</t>
+          <t>D:\AFFILATE BOT\data\research\posthog-review-2026-pricing-cost-and-roi</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>astrbot-review-2026-comparison-and-alternatives</t>
+          <t>wigolo-review-2026-pricing-cost-and-roi</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>AstrBot Review 2026 comparison and alternatives</t>
+          <t>wigolo Review 2026 pricing cost and ROI</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>54.43</v>
+        <v>50.71</v>
       </c>
       <c r="D10" t="n">
         <v>72</v>
       </c>
       <c r="E10" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="F10" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H10" t="n">
         <v>68</v>
       </c>
       <c r="I10" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J10" t="n">
         <v>45</v>
@@ -4244,7 +4244,7 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -4254,23 +4254,23 @@
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\astrbot-review-2026-comparison-and-alternatives</t>
+          <t>D:\AFFILATE BOT\data\research\wigolo-review-2026-pricing-cost-and-roi</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>how-to-implement-free-ai-tools</t>
+          <t>astrbot-review-2026-pricing-cost-and-roi</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>how to implement Free AI Tools</t>
+          <t>AstrBot Review 2026 pricing cost and ROI</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>51.71</v>
+        <v>50.71</v>
       </c>
       <c r="D11" t="n">
         <v>72</v>
@@ -4296,7 +4296,7 @@
         <v>45</v>
       </c>
       <c r="K11" t="n">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="L11" t="n">
         <v>20</v>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\how-to-implement-free-ai-tools</t>
+          <t>D:\AFFILATE BOT\data\research\astrbot-review-2026-pricing-cost-and-roi</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish ready daily articles 2026-07-24
</commit_message>
<xml_diff>
--- a/data/master_dashboard.xlsx
+++ b/data/master_dashboard.xlsx
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>99</v>
+        <v>109</v>
       </c>
     </row>
     <row r="9">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>99</v>
+        <v>109</v>
       </c>
     </row>
     <row r="10">
@@ -3532,16 +3532,16 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>atlassian-team-launches-ai-native-jira-tools-for-the-full-development-workflow-pricing-cost-and-roi</t>
+          <t>best-atlassian-team-launches-ai-native-jira-tools-for-the-full-development-workflow-workflows-and-use-cases</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Atlassian (TEAM) Launches AI Native Jira Tools For The Full Development Workflow pricing cost and ROI</t>
+          <t>best Atlassian (TEAM) Launches AI Native Jira Tools For The Full Development Workflow workflows and use cases</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>51.86</v>
+        <v>53.29</v>
       </c>
       <c r="D2" t="n">
         <v>72</v>
@@ -3561,7 +3561,7 @@
         <v>68</v>
       </c>
       <c r="I2" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J2" t="n">
         <v>45</v>
@@ -3606,23 +3606,23 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\atlassian-team-launches-ai-native-jira-tools-for-the-full-development-workflow-pricing-cost-and-roi</t>
+          <t>D:\AFFILATE BOT\data\research\best-atlassian-team-launches-ai-native-jira-tools-for-the-full-development-workflow-workflows-and-use-cases</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>free-ai-tools-pricing-cost-and-roi</t>
+          <t>best-free-ai-tools-workflows-and-use-cases</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Free AI Tools pricing cost and ROI</t>
+          <t>best Free AI Tools workflows and use cases</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>51.71</v>
+        <v>53.14</v>
       </c>
       <c r="D3" t="n">
         <v>72</v>
@@ -3642,7 +3642,7 @@
         <v>68</v>
       </c>
       <c r="I3" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J3" t="n">
         <v>45</v>
@@ -3687,23 +3687,23 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\free-ai-tools-pricing-cost-and-roi</t>
+          <t>D:\AFFILATE BOT\data\research\best-free-ai-tools-workflows-and-use-cases</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>wrenai-review-2026-pricing-cost-and-roi</t>
+          <t>best-wrenai-review-2026-workflows-and-use-cases</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>WrenAI Review 2026 pricing cost and ROI</t>
+          <t>best WrenAI Review 2026 workflows and use cases</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>50.71</v>
+        <v>52.14</v>
       </c>
       <c r="D4" t="n">
         <v>72</v>
@@ -3723,7 +3723,7 @@
         <v>68</v>
       </c>
       <c r="I4" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J4" t="n">
         <v>45</v>
@@ -3768,23 +3768,23 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\wrenai-review-2026-pricing-cost-and-roi</t>
+          <t>D:\AFFILATE BOT\data\research\best-wrenai-review-2026-workflows-and-use-cases</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ktransformers-review-2026-pricing-cost-and-roi</t>
+          <t>best-ktransformers-review-2026-workflows-and-use-cases</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ktransformers Review 2026 pricing cost and ROI</t>
+          <t>best ktransformers Review 2026 workflows and use cases</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>50.71</v>
+        <v>52.14</v>
       </c>
       <c r="D5" t="n">
         <v>72</v>
@@ -3804,7 +3804,7 @@
         <v>68</v>
       </c>
       <c r="I5" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J5" t="n">
         <v>45</v>
@@ -3849,23 +3849,23 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\ktransformers-review-2026-pricing-cost-and-roi</t>
+          <t>D:\AFFILATE BOT\data\research\best-ktransformers-review-2026-workflows-and-use-cases</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>voicebox-review-2026-pricing-cost-and-roi</t>
+          <t>best-voicebox-review-2026-workflows-and-use-cases</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>voicebox Review 2026 pricing cost and ROI</t>
+          <t>best voicebox Review 2026 workflows and use cases</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>50.71</v>
+        <v>52.14</v>
       </c>
       <c r="D6" t="n">
         <v>72</v>
@@ -3885,7 +3885,7 @@
         <v>68</v>
       </c>
       <c r="I6" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J6" t="n">
         <v>45</v>
@@ -3930,23 +3930,23 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\voicebox-review-2026-pricing-cost-and-roi</t>
+          <t>D:\AFFILATE BOT\data\research\best-voicebox-review-2026-workflows-and-use-cases</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>code-review-graph-review-2026-pricing-cost-and-roi</t>
+          <t>best-code-review-graph-review-2026-workflows-and-use-cases</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>code-review-graph Review 2026 pricing cost and ROI</t>
+          <t>best code-review-graph Review 2026 workflows and use cases</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>50.71</v>
+        <v>52.14</v>
       </c>
       <c r="D7" t="n">
         <v>72</v>
@@ -3966,7 +3966,7 @@
         <v>68</v>
       </c>
       <c r="I7" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J7" t="n">
         <v>45</v>
@@ -4011,23 +4011,23 @@
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\code-review-graph-review-2026-pricing-cost-and-roi</t>
+          <t>D:\AFFILATE BOT\data\research\best-code-review-graph-review-2026-workflows-and-use-cases</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>copilot-sdk-review-2026-pricing-cost-and-roi</t>
+          <t>best-copilot-sdk-review-2026-workflows-and-use-cases</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>copilot-sdk Review 2026 pricing cost and ROI</t>
+          <t>best copilot-sdk Review 2026 workflows and use cases</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>50.71</v>
+        <v>52.14</v>
       </c>
       <c r="D8" t="n">
         <v>72</v>
@@ -4047,7 +4047,7 @@
         <v>68</v>
       </c>
       <c r="I8" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J8" t="n">
         <v>45</v>
@@ -4092,23 +4092,23 @@
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\copilot-sdk-review-2026-pricing-cost-and-roi</t>
+          <t>D:\AFFILATE BOT\data\research\best-copilot-sdk-review-2026-workflows-and-use-cases</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>posthog-review-2026-pricing-cost-and-roi</t>
+          <t>best-posthog-review-2026-workflows-and-use-cases</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>posthog Review 2026 pricing cost and ROI</t>
+          <t>best posthog Review 2026 workflows and use cases</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>50.71</v>
+        <v>52.14</v>
       </c>
       <c r="D9" t="n">
         <v>72</v>
@@ -4128,7 +4128,7 @@
         <v>68</v>
       </c>
       <c r="I9" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J9" t="n">
         <v>45</v>
@@ -4173,23 +4173,23 @@
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\posthog-review-2026-pricing-cost-and-roi</t>
+          <t>D:\AFFILATE BOT\data\research\best-posthog-review-2026-workflows-and-use-cases</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>wigolo-review-2026-pricing-cost-and-roi</t>
+          <t>best-wigolo-review-2026-workflows-and-use-cases</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>wigolo Review 2026 pricing cost and ROI</t>
+          <t>best wigolo Review 2026 workflows and use cases</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>50.71</v>
+        <v>52.14</v>
       </c>
       <c r="D10" t="n">
         <v>72</v>
@@ -4209,7 +4209,7 @@
         <v>68</v>
       </c>
       <c r="I10" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J10" t="n">
         <v>45</v>
@@ -4254,23 +4254,23 @@
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\wigolo-review-2026-pricing-cost-and-roi</t>
+          <t>D:\AFFILATE BOT\data\research\best-wigolo-review-2026-workflows-and-use-cases</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>astrbot-review-2026-pricing-cost-and-roi</t>
+          <t>best-astrbot-review-2026-workflows-and-use-cases</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>AstrBot Review 2026 pricing cost and ROI</t>
+          <t>best AstrBot Review 2026 workflows and use cases</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>50.71</v>
+        <v>52.14</v>
       </c>
       <c r="D11" t="n">
         <v>72</v>
@@ -4290,7 +4290,7 @@
         <v>68</v>
       </c>
       <c r="I11" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J11" t="n">
         <v>45</v>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\astrbot-review-2026-pricing-cost-and-roi</t>
+          <t>D:\AFFILATE BOT\data\research\best-astrbot-review-2026-workflows-and-use-cases</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish ready daily articles 2026-07-25
</commit_message>
<xml_diff>
--- a/data/master_dashboard.xlsx
+++ b/data/master_dashboard.xlsx
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>109</v>
+        <v>119</v>
       </c>
     </row>
     <row r="9">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>109</v>
+        <v>119</v>
       </c>
     </row>
     <row r="10">
@@ -3419,7 +3419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U11"/>
+  <dimension ref="A1:U2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3532,16 +3532,16 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>best-atlassian-team-launches-ai-native-jira-tools-for-the-full-development-workflow-workflows-and-use-cases</t>
+          <t>common-atlassian-team-launches-ai-native-jira-tools-for-the-full-development-workflow-mistakes-and-troubleshooting</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>best Atlassian (TEAM) Launches AI Native Jira Tools For The Full Development Workflow workflows and use cases</t>
+          <t>common Atlassian (TEAM) Launches AI Native Jira Tools For The Full Development Workflow mistakes and troubleshooting</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>53.29</v>
+        <v>51.86</v>
       </c>
       <c r="D2" t="n">
         <v>72</v>
@@ -3561,7 +3561,7 @@
         <v>68</v>
       </c>
       <c r="I2" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J2" t="n">
         <v>45</v>
@@ -3606,736 +3606,7 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\best-atlassian-team-launches-ai-native-jira-tools-for-the-full-development-workflow-workflows-and-use-cases</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>best-free-ai-tools-workflows-and-use-cases</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>best Free AI Tools workflows and use cases</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>53.14</v>
-      </c>
-      <c r="D3" t="n">
-        <v>72</v>
-      </c>
-      <c r="E3" t="n">
-        <v>36</v>
-      </c>
-      <c r="F3" t="n">
-        <v>36</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
-        </is>
-      </c>
-      <c r="H3" t="n">
-        <v>68</v>
-      </c>
-      <c r="I3" t="n">
-        <v>80</v>
-      </c>
-      <c r="J3" t="n">
-        <v>45</v>
-      </c>
-      <c r="K3" t="n">
-        <v>61</v>
-      </c>
-      <c r="L3" t="n">
-        <v>20</v>
-      </c>
-      <c r="M3" t="n">
-        <v>20</v>
-      </c>
-      <c r="N3" t="n">
-        <v>10</v>
-      </c>
-      <c r="O3" t="n">
-        <v>70</v>
-      </c>
-      <c r="P3" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>verified</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>needs enrichment</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>D:\AFFILATE BOT\data\research\best-free-ai-tools-workflows-and-use-cases</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>best-wrenai-review-2026-workflows-and-use-cases</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>best WrenAI Review 2026 workflows and use cases</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>52.14</v>
-      </c>
-      <c r="D4" t="n">
-        <v>72</v>
-      </c>
-      <c r="E4" t="n">
-        <v>36</v>
-      </c>
-      <c r="F4" t="n">
-        <v>36</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
-        </is>
-      </c>
-      <c r="H4" t="n">
-        <v>68</v>
-      </c>
-      <c r="I4" t="n">
-        <v>80</v>
-      </c>
-      <c r="J4" t="n">
-        <v>45</v>
-      </c>
-      <c r="K4" t="n">
-        <v>54</v>
-      </c>
-      <c r="L4" t="n">
-        <v>20</v>
-      </c>
-      <c r="M4" t="n">
-        <v>20</v>
-      </c>
-      <c r="N4" t="n">
-        <v>10</v>
-      </c>
-      <c r="O4" t="n">
-        <v>70</v>
-      </c>
-      <c r="P4" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>verified</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>needs enrichment</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>D:\AFFILATE BOT\data\research\best-wrenai-review-2026-workflows-and-use-cases</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>best-ktransformers-review-2026-workflows-and-use-cases</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>best ktransformers Review 2026 workflows and use cases</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>52.14</v>
-      </c>
-      <c r="D5" t="n">
-        <v>72</v>
-      </c>
-      <c r="E5" t="n">
-        <v>36</v>
-      </c>
-      <c r="F5" t="n">
-        <v>36</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
-        </is>
-      </c>
-      <c r="H5" t="n">
-        <v>68</v>
-      </c>
-      <c r="I5" t="n">
-        <v>80</v>
-      </c>
-      <c r="J5" t="n">
-        <v>45</v>
-      </c>
-      <c r="K5" t="n">
-        <v>54</v>
-      </c>
-      <c r="L5" t="n">
-        <v>20</v>
-      </c>
-      <c r="M5" t="n">
-        <v>20</v>
-      </c>
-      <c r="N5" t="n">
-        <v>10</v>
-      </c>
-      <c r="O5" t="n">
-        <v>70</v>
-      </c>
-      <c r="P5" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>verified</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>needs enrichment</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>D:\AFFILATE BOT\data\research\best-ktransformers-review-2026-workflows-and-use-cases</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>best-voicebox-review-2026-workflows-and-use-cases</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>best voicebox Review 2026 workflows and use cases</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>52.14</v>
-      </c>
-      <c r="D6" t="n">
-        <v>72</v>
-      </c>
-      <c r="E6" t="n">
-        <v>36</v>
-      </c>
-      <c r="F6" t="n">
-        <v>36</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
-        </is>
-      </c>
-      <c r="H6" t="n">
-        <v>68</v>
-      </c>
-      <c r="I6" t="n">
-        <v>80</v>
-      </c>
-      <c r="J6" t="n">
-        <v>45</v>
-      </c>
-      <c r="K6" t="n">
-        <v>54</v>
-      </c>
-      <c r="L6" t="n">
-        <v>20</v>
-      </c>
-      <c r="M6" t="n">
-        <v>20</v>
-      </c>
-      <c r="N6" t="n">
-        <v>10</v>
-      </c>
-      <c r="O6" t="n">
-        <v>70</v>
-      </c>
-      <c r="P6" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>verified</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>needs enrichment</t>
-        </is>
-      </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>D:\AFFILATE BOT\data\research\best-voicebox-review-2026-workflows-and-use-cases</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>best-code-review-graph-review-2026-workflows-and-use-cases</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>best code-review-graph Review 2026 workflows and use cases</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>52.14</v>
-      </c>
-      <c r="D7" t="n">
-        <v>72</v>
-      </c>
-      <c r="E7" t="n">
-        <v>36</v>
-      </c>
-      <c r="F7" t="n">
-        <v>36</v>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
-        </is>
-      </c>
-      <c r="H7" t="n">
-        <v>68</v>
-      </c>
-      <c r="I7" t="n">
-        <v>80</v>
-      </c>
-      <c r="J7" t="n">
-        <v>45</v>
-      </c>
-      <c r="K7" t="n">
-        <v>54</v>
-      </c>
-      <c r="L7" t="n">
-        <v>20</v>
-      </c>
-      <c r="M7" t="n">
-        <v>20</v>
-      </c>
-      <c r="N7" t="n">
-        <v>10</v>
-      </c>
-      <c r="O7" t="n">
-        <v>70</v>
-      </c>
-      <c r="P7" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>verified</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>needs enrichment</t>
-        </is>
-      </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
-        </is>
-      </c>
-      <c r="T7" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>D:\AFFILATE BOT\data\research\best-code-review-graph-review-2026-workflows-and-use-cases</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>best-copilot-sdk-review-2026-workflows-and-use-cases</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>best copilot-sdk Review 2026 workflows and use cases</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>52.14</v>
-      </c>
-      <c r="D8" t="n">
-        <v>72</v>
-      </c>
-      <c r="E8" t="n">
-        <v>36</v>
-      </c>
-      <c r="F8" t="n">
-        <v>36</v>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
-        </is>
-      </c>
-      <c r="H8" t="n">
-        <v>68</v>
-      </c>
-      <c r="I8" t="n">
-        <v>80</v>
-      </c>
-      <c r="J8" t="n">
-        <v>45</v>
-      </c>
-      <c r="K8" t="n">
-        <v>54</v>
-      </c>
-      <c r="L8" t="n">
-        <v>20</v>
-      </c>
-      <c r="M8" t="n">
-        <v>20</v>
-      </c>
-      <c r="N8" t="n">
-        <v>10</v>
-      </c>
-      <c r="O8" t="n">
-        <v>70</v>
-      </c>
-      <c r="P8" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>verified</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>needs enrichment</t>
-        </is>
-      </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
-        </is>
-      </c>
-      <c r="T8" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>D:\AFFILATE BOT\data\research\best-copilot-sdk-review-2026-workflows-and-use-cases</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>best-posthog-review-2026-workflows-and-use-cases</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>best posthog Review 2026 workflows and use cases</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>52.14</v>
-      </c>
-      <c r="D9" t="n">
-        <v>72</v>
-      </c>
-      <c r="E9" t="n">
-        <v>36</v>
-      </c>
-      <c r="F9" t="n">
-        <v>36</v>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
-        </is>
-      </c>
-      <c r="H9" t="n">
-        <v>68</v>
-      </c>
-      <c r="I9" t="n">
-        <v>80</v>
-      </c>
-      <c r="J9" t="n">
-        <v>45</v>
-      </c>
-      <c r="K9" t="n">
-        <v>54</v>
-      </c>
-      <c r="L9" t="n">
-        <v>20</v>
-      </c>
-      <c r="M9" t="n">
-        <v>20</v>
-      </c>
-      <c r="N9" t="n">
-        <v>10</v>
-      </c>
-      <c r="O9" t="n">
-        <v>70</v>
-      </c>
-      <c r="P9" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>verified</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>needs enrichment</t>
-        </is>
-      </c>
-      <c r="S9" t="inlineStr">
-        <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
-        </is>
-      </c>
-      <c r="T9" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>D:\AFFILATE BOT\data\research\best-posthog-review-2026-workflows-and-use-cases</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>best-wigolo-review-2026-workflows-and-use-cases</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>best wigolo Review 2026 workflows and use cases</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>52.14</v>
-      </c>
-      <c r="D10" t="n">
-        <v>72</v>
-      </c>
-      <c r="E10" t="n">
-        <v>36</v>
-      </c>
-      <c r="F10" t="n">
-        <v>36</v>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
-        </is>
-      </c>
-      <c r="H10" t="n">
-        <v>68</v>
-      </c>
-      <c r="I10" t="n">
-        <v>80</v>
-      </c>
-      <c r="J10" t="n">
-        <v>45</v>
-      </c>
-      <c r="K10" t="n">
-        <v>54</v>
-      </c>
-      <c r="L10" t="n">
-        <v>20</v>
-      </c>
-      <c r="M10" t="n">
-        <v>20</v>
-      </c>
-      <c r="N10" t="n">
-        <v>10</v>
-      </c>
-      <c r="O10" t="n">
-        <v>70</v>
-      </c>
-      <c r="P10" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>verified</t>
-        </is>
-      </c>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>needs enrichment</t>
-        </is>
-      </c>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
-        </is>
-      </c>
-      <c r="T10" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>D:\AFFILATE BOT\data\research\best-wigolo-review-2026-workflows-and-use-cases</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>best-astrbot-review-2026-workflows-and-use-cases</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>best AstrBot Review 2026 workflows and use cases</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>52.14</v>
-      </c>
-      <c r="D11" t="n">
-        <v>72</v>
-      </c>
-      <c r="E11" t="n">
-        <v>36</v>
-      </c>
-      <c r="F11" t="n">
-        <v>36</v>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
-        </is>
-      </c>
-      <c r="H11" t="n">
-        <v>68</v>
-      </c>
-      <c r="I11" t="n">
-        <v>80</v>
-      </c>
-      <c r="J11" t="n">
-        <v>45</v>
-      </c>
-      <c r="K11" t="n">
-        <v>54</v>
-      </c>
-      <c r="L11" t="n">
-        <v>20</v>
-      </c>
-      <c r="M11" t="n">
-        <v>20</v>
-      </c>
-      <c r="N11" t="n">
-        <v>10</v>
-      </c>
-      <c r="O11" t="n">
-        <v>70</v>
-      </c>
-      <c r="P11" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>verified</t>
-        </is>
-      </c>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t>needs enrichment</t>
-        </is>
-      </c>
-      <c r="S11" t="inlineStr">
-        <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
-        </is>
-      </c>
-      <c r="T11" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>D:\AFFILATE BOT\data\research\best-astrbot-review-2026-workflows-and-use-cases</t>
+          <t>D:\AFFILATE BOT\data\research\common-atlassian-team-launches-ai-native-jira-tools-for-the-full-development-workflow-mistakes-and-troubleshooting</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish ready daily articles 2026-07-26
</commit_message>
<xml_diff>
--- a/data/master_dashboard.xlsx
+++ b/data/master_dashboard.xlsx
@@ -472,7 +472,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6">
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>119</v>
+        <v>129</v>
       </c>
     </row>
     <row r="9">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>119</v>
+        <v>129</v>
       </c>
     </row>
     <row r="10">
@@ -3532,36 +3532,36 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>common-atlassian-team-launches-ai-native-jira-tools-for-the-full-development-workflow-mistakes-and-troubleshooting</t>
+          <t>is-atlassian-team-launches-ai-native-jira-tools-for-the-full-development-workflow-worth-it-for-small-business</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>common Atlassian (TEAM) Launches AI Native Jira Tools For The Full Development Workflow mistakes and troubleshooting</t>
+          <t>is Atlassian (TEAM) Launches AI Native Jira Tools For The Full Development Workflow worth it for small business</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>51.86</v>
+        <v>55.57</v>
       </c>
       <c r="D2" t="n">
         <v>72</v>
       </c>
       <c r="E2" t="n">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="F2" t="n">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H2" t="n">
         <v>68</v>
       </c>
       <c r="I2" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J2" t="n">
         <v>45</v>
@@ -3596,7 +3596,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -3606,7 +3606,7 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\common-atlassian-team-launches-ai-native-jira-tools-for-the-full-development-workflow-mistakes-and-troubleshooting</t>
+          <t>D:\AFFILATE BOT\data\research\is-atlassian-team-launches-ai-native-jira-tools-for-the-full-development-workflow-worth-it-for-small-business</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish ready daily articles 2026-07-27
</commit_message>
<xml_diff>
--- a/data/master_dashboard.xlsx
+++ b/data/master_dashboard.xlsx
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="9">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="10">
@@ -3419,7 +3419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U2"/>
+  <dimension ref="A1:U11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3532,29 +3532,29 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>is-atlassian-team-launches-ai-native-jira-tools-for-the-full-development-workflow-worth-it-for-small-business</t>
+          <t>impeccable-review-2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>is Atlassian (TEAM) Launches AI Native Jira Tools For The Full Development Workflow worth it for small business</t>
+          <t>impeccable Review 2026</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>55.57</v>
+        <v>52.14</v>
       </c>
       <c r="D2" t="n">
         <v>72</v>
       </c>
       <c r="E2" t="n">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="F2" t="n">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H2" t="n">
@@ -3596,17 +3596,746 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>D:\AFFILATE BOT\data\research\impeccable-review-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>chat2db-review-2026</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Chat2DB Review 2026</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>52.14</v>
+      </c>
+      <c r="D3" t="n">
+        <v>72</v>
+      </c>
+      <c r="E3" t="n">
+        <v>36</v>
+      </c>
+      <c r="F3" t="n">
+        <v>36</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>68</v>
+      </c>
+      <c r="I3" t="n">
+        <v>80</v>
+      </c>
+      <c r="J3" t="n">
+        <v>45</v>
+      </c>
+      <c r="K3" t="n">
+        <v>54</v>
+      </c>
+      <c r="L3" t="n">
+        <v>20</v>
+      </c>
+      <c r="M3" t="n">
+        <v>20</v>
+      </c>
+      <c r="N3" t="n">
+        <v>10</v>
+      </c>
+      <c r="O3" t="n">
+        <v>70</v>
+      </c>
+      <c r="P3" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>needs enrichment</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>D:\AFFILATE BOT\data\research\chat2db-review-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>instatic-review-2026</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Instatic Review 2026</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>52.14</v>
+      </c>
+      <c r="D4" t="n">
+        <v>72</v>
+      </c>
+      <c r="E4" t="n">
+        <v>36</v>
+      </c>
+      <c r="F4" t="n">
+        <v>36</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>68</v>
+      </c>
+      <c r="I4" t="n">
+        <v>80</v>
+      </c>
+      <c r="J4" t="n">
+        <v>45</v>
+      </c>
+      <c r="K4" t="n">
+        <v>54</v>
+      </c>
+      <c r="L4" t="n">
+        <v>20</v>
+      </c>
+      <c r="M4" t="n">
+        <v>20</v>
+      </c>
+      <c r="N4" t="n">
+        <v>10</v>
+      </c>
+      <c r="O4" t="n">
+        <v>70</v>
+      </c>
+      <c r="P4" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>needs enrichment</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>D:\AFFILATE BOT\data\research\instatic-review-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ego-lite-review-2026</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ego-lite Review 2026</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>52.14</v>
+      </c>
+      <c r="D5" t="n">
+        <v>72</v>
+      </c>
+      <c r="E5" t="n">
+        <v>36</v>
+      </c>
+      <c r="F5" t="n">
+        <v>36</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>68</v>
+      </c>
+      <c r="I5" t="n">
+        <v>80</v>
+      </c>
+      <c r="J5" t="n">
+        <v>45</v>
+      </c>
+      <c r="K5" t="n">
+        <v>54</v>
+      </c>
+      <c r="L5" t="n">
+        <v>20</v>
+      </c>
+      <c r="M5" t="n">
+        <v>20</v>
+      </c>
+      <c r="N5" t="n">
+        <v>10</v>
+      </c>
+      <c r="O5" t="n">
+        <v>70</v>
+      </c>
+      <c r="P5" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>needs enrichment</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>D:\AFFILATE BOT\data\research\ego-lite-review-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>open-code-review-review-2026</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>open-code-review Review 2026</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>53.14</v>
+      </c>
+      <c r="D6" t="n">
+        <v>72</v>
+      </c>
+      <c r="E6" t="n">
+        <v>36</v>
+      </c>
+      <c r="F6" t="n">
+        <v>36</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>68</v>
+      </c>
+      <c r="I6" t="n">
+        <v>80</v>
+      </c>
+      <c r="J6" t="n">
+        <v>45</v>
+      </c>
+      <c r="K6" t="n">
+        <v>61</v>
+      </c>
+      <c r="L6" t="n">
+        <v>20</v>
+      </c>
+      <c r="M6" t="n">
+        <v>20</v>
+      </c>
+      <c r="N6" t="n">
+        <v>10</v>
+      </c>
+      <c r="O6" t="n">
+        <v>70</v>
+      </c>
+      <c r="P6" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>needs enrichment</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>D:\AFFILATE BOT\data\research\open-code-review-review-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>is-atlassian-team-launches-ai-native-jira-tools-for-the-full-development-workflow-worth-it-for-small-business</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>is Atlassian (TEAM) Launches AI Native Jira Tools For The Full Development Workflow worth it for small business</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>55.57</v>
+      </c>
+      <c r="D7" t="n">
+        <v>72</v>
+      </c>
+      <c r="E7" t="n">
+        <v>60</v>
+      </c>
+      <c r="F7" t="n">
+        <v>60</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>["ai_tools", "companies", "affiliate_networks", "competitors", "product_categories"]</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>68</v>
+      </c>
+      <c r="I7" t="n">
+        <v>80</v>
+      </c>
+      <c r="J7" t="n">
+        <v>45</v>
+      </c>
+      <c r="K7" t="n">
+        <v>54</v>
+      </c>
+      <c r="L7" t="n">
+        <v>20</v>
+      </c>
+      <c r="M7" t="n">
+        <v>20</v>
+      </c>
+      <c r="N7" t="n">
+        <v>10</v>
+      </c>
+      <c r="O7" t="n">
+        <v>70</v>
+      </c>
+      <c r="P7" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>needs enrichment</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
           <t>["competitor coverage is limited"]</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="T7" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="U7" t="inlineStr">
         <is>
           <t>D:\AFFILATE BOT\data\research\is-atlassian-team-launches-ai-native-jira-tools-for-the-full-development-workflow-worth-it-for-small-business</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>is-free-ai-tools-worth-it-for-small-business</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>is Free AI Tools worth it for small business</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>55.43</v>
+      </c>
+      <c r="D8" t="n">
+        <v>72</v>
+      </c>
+      <c r="E8" t="n">
+        <v>52</v>
+      </c>
+      <c r="F8" t="n">
+        <v>52</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>68</v>
+      </c>
+      <c r="I8" t="n">
+        <v>80</v>
+      </c>
+      <c r="J8" t="n">
+        <v>45</v>
+      </c>
+      <c r="K8" t="n">
+        <v>61</v>
+      </c>
+      <c r="L8" t="n">
+        <v>20</v>
+      </c>
+      <c r="M8" t="n">
+        <v>20</v>
+      </c>
+      <c r="N8" t="n">
+        <v>10</v>
+      </c>
+      <c r="O8" t="n">
+        <v>70</v>
+      </c>
+      <c r="P8" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>needs enrichment</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>["competitor coverage is limited"]</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>D:\AFFILATE BOT\data\research\is-free-ai-tools-worth-it-for-small-business</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>is-wrenai-review-2026-worth-it-for-small-business</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>is WrenAI Review 2026 worth it for small business</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>54.43</v>
+      </c>
+      <c r="D9" t="n">
+        <v>72</v>
+      </c>
+      <c r="E9" t="n">
+        <v>52</v>
+      </c>
+      <c r="F9" t="n">
+        <v>52</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>68</v>
+      </c>
+      <c r="I9" t="n">
+        <v>80</v>
+      </c>
+      <c r="J9" t="n">
+        <v>45</v>
+      </c>
+      <c r="K9" t="n">
+        <v>54</v>
+      </c>
+      <c r="L9" t="n">
+        <v>20</v>
+      </c>
+      <c r="M9" t="n">
+        <v>20</v>
+      </c>
+      <c r="N9" t="n">
+        <v>10</v>
+      </c>
+      <c r="O9" t="n">
+        <v>70</v>
+      </c>
+      <c r="P9" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>needs enrichment</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>["competitor coverage is limited"]</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>D:\AFFILATE BOT\data\research\is-wrenai-review-2026-worth-it-for-small-business</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>is-ktransformers-review-2026-worth-it-for-small-business</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>is ktransformers Review 2026 worth it for small business</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>54.43</v>
+      </c>
+      <c r="D10" t="n">
+        <v>72</v>
+      </c>
+      <c r="E10" t="n">
+        <v>52</v>
+      </c>
+      <c r="F10" t="n">
+        <v>52</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>68</v>
+      </c>
+      <c r="I10" t="n">
+        <v>80</v>
+      </c>
+      <c r="J10" t="n">
+        <v>45</v>
+      </c>
+      <c r="K10" t="n">
+        <v>54</v>
+      </c>
+      <c r="L10" t="n">
+        <v>20</v>
+      </c>
+      <c r="M10" t="n">
+        <v>20</v>
+      </c>
+      <c r="N10" t="n">
+        <v>10</v>
+      </c>
+      <c r="O10" t="n">
+        <v>70</v>
+      </c>
+      <c r="P10" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>needs enrichment</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>["competitor coverage is limited"]</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>D:\AFFILATE BOT\data\research\is-ktransformers-review-2026-worth-it-for-small-business</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>is-voicebox-review-2026-worth-it-for-small-business</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>is voicebox Review 2026 worth it for small business</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>54.43</v>
+      </c>
+      <c r="D11" t="n">
+        <v>72</v>
+      </c>
+      <c r="E11" t="n">
+        <v>52</v>
+      </c>
+      <c r="F11" t="n">
+        <v>52</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>68</v>
+      </c>
+      <c r="I11" t="n">
+        <v>80</v>
+      </c>
+      <c r="J11" t="n">
+        <v>45</v>
+      </c>
+      <c r="K11" t="n">
+        <v>54</v>
+      </c>
+      <c r="L11" t="n">
+        <v>20</v>
+      </c>
+      <c r="M11" t="n">
+        <v>20</v>
+      </c>
+      <c r="N11" t="n">
+        <v>10</v>
+      </c>
+      <c r="O11" t="n">
+        <v>70</v>
+      </c>
+      <c r="P11" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>needs enrichment</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>["competitor coverage is limited"]</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>D:\AFFILATE BOT\data\research\is-voicebox-review-2026-worth-it-for-small-business</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish ready daily articles 2026-07-30
</commit_message>
<xml_diff>
--- a/data/master_dashboard.xlsx
+++ b/data/master_dashboard.xlsx
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="9">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="10">
@@ -3532,16 +3532,16 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>impeccable-review-2026</t>
+          <t>impeccable-review-2026-pricing-cost-and-roi</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>impeccable Review 2026</t>
+          <t>impeccable Review 2026 pricing cost and ROI</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>52.14</v>
+        <v>50.71</v>
       </c>
       <c r="D2" t="n">
         <v>72</v>
@@ -3561,7 +3561,7 @@
         <v>68</v>
       </c>
       <c r="I2" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J2" t="n">
         <v>45</v>
@@ -3606,23 +3606,23 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\impeccable-review-2026</t>
+          <t>D:\AFFILATE BOT\data\research\impeccable-review-2026-pricing-cost-and-roi</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>chat2db-review-2026</t>
+          <t>ego-lite-review-2026-pricing-cost-and-roi</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Chat2DB Review 2026</t>
+          <t>ego-lite Review 2026 pricing cost and ROI</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>52.14</v>
+        <v>50.71</v>
       </c>
       <c r="D3" t="n">
         <v>72</v>
@@ -3642,7 +3642,7 @@
         <v>68</v>
       </c>
       <c r="I3" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J3" t="n">
         <v>45</v>
@@ -3687,36 +3687,36 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\chat2db-review-2026</t>
+          <t>D:\AFFILATE BOT\data\research\ego-lite-review-2026-pricing-cost-and-roi</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>instatic-review-2026</t>
+          <t>impeccable-review-2026-comparison-and-alternatives</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Instatic Review 2026</t>
+          <t>impeccable Review 2026 comparison and alternatives</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>52.14</v>
+        <v>54.43</v>
       </c>
       <c r="D4" t="n">
         <v>72</v>
       </c>
       <c r="E4" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="F4" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H4" t="n">
@@ -3758,7 +3758,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -3768,36 +3768,36 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\instatic-review-2026</t>
+          <t>D:\AFFILATE BOT\data\research\impeccable-review-2026-comparison-and-alternatives</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ego-lite-review-2026</t>
+          <t>ego-lite-review-2026-comparison-and-alternatives</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ego-lite Review 2026</t>
+          <t>ego-lite Review 2026 comparison and alternatives</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>52.14</v>
+        <v>54.43</v>
       </c>
       <c r="D5" t="n">
         <v>72</v>
       </c>
       <c r="E5" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="F5" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H5" t="n">
@@ -3839,7 +3839,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -3849,23 +3849,23 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\ego-lite-review-2026</t>
+          <t>D:\AFFILATE BOT\data\research\ego-lite-review-2026-comparison-and-alternatives</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>open-code-review-review-2026</t>
+          <t>impeccable-review-2026</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>open-code-review Review 2026</t>
+          <t>impeccable Review 2026</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>53.14</v>
+        <v>52.14</v>
       </c>
       <c r="D6" t="n">
         <v>72</v>
@@ -3891,7 +3891,7 @@
         <v>45</v>
       </c>
       <c r="K6" t="n">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="L6" t="n">
         <v>20</v>
@@ -3930,36 +3930,36 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\open-code-review-review-2026</t>
+          <t>D:\AFFILATE BOT\data\research\impeccable-review-2026</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>is-atlassian-team-launches-ai-native-jira-tools-for-the-full-development-workflow-worth-it-for-small-business</t>
+          <t>chat2db-review-2026</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>is Atlassian (TEAM) Launches AI Native Jira Tools For The Full Development Workflow worth it for small business</t>
+          <t>Chat2DB Review 2026</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>55.57</v>
+        <v>52.14</v>
       </c>
       <c r="D7" t="n">
         <v>72</v>
       </c>
       <c r="E7" t="n">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="F7" t="n">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H7" t="n">
@@ -4001,7 +4001,7 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -4011,36 +4011,36 @@
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\is-atlassian-team-launches-ai-native-jira-tools-for-the-full-development-workflow-worth-it-for-small-business</t>
+          <t>D:\AFFILATE BOT\data\research\chat2db-review-2026</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>is-free-ai-tools-worth-it-for-small-business</t>
+          <t>instatic-review-2026</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>is Free AI Tools worth it for small business</t>
+          <t>Instatic Review 2026</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>55.43</v>
+        <v>52.14</v>
       </c>
       <c r="D8" t="n">
         <v>72</v>
       </c>
       <c r="E8" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="F8" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H8" t="n">
@@ -4053,7 +4053,7 @@
         <v>45</v>
       </c>
       <c r="K8" t="n">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="L8" t="n">
         <v>20</v>
@@ -4082,7 +4082,7 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -4092,36 +4092,36 @@
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\is-free-ai-tools-worth-it-for-small-business</t>
+          <t>D:\AFFILATE BOT\data\research\instatic-review-2026</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>is-wrenai-review-2026-worth-it-for-small-business</t>
+          <t>ego-lite-review-2026</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>is WrenAI Review 2026 worth it for small business</t>
+          <t>ego-lite Review 2026</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>54.43</v>
+        <v>52.14</v>
       </c>
       <c r="D9" t="n">
         <v>72</v>
       </c>
       <c r="E9" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="F9" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H9" t="n">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -4173,36 +4173,36 @@
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\is-wrenai-review-2026-worth-it-for-small-business</t>
+          <t>D:\AFFILATE BOT\data\research\ego-lite-review-2026</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>is-ktransformers-review-2026-worth-it-for-small-business</t>
+          <t>open-code-review-review-2026</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>is ktransformers Review 2026 worth it for small business</t>
+          <t>open-code-review Review 2026</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>54.43</v>
+        <v>53.14</v>
       </c>
       <c r="D10" t="n">
         <v>72</v>
       </c>
       <c r="E10" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="F10" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H10" t="n">
@@ -4215,7 +4215,7 @@
         <v>45</v>
       </c>
       <c r="K10" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="L10" t="n">
         <v>20</v>
@@ -4244,7 +4244,7 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -4254,36 +4254,36 @@
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\is-ktransformers-review-2026-worth-it-for-small-business</t>
+          <t>D:\AFFILATE BOT\data\research\open-code-review-review-2026</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>is-voicebox-review-2026-worth-it-for-small-business</t>
+          <t>is-atlassian-team-launches-ai-native-jira-tools-for-the-full-development-workflow-worth-it-for-small-business</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>is voicebox Review 2026 worth it for small business</t>
+          <t>is Atlassian (TEAM) Launches AI Native Jira Tools For The Full Development Workflow worth it for small business</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>54.43</v>
+        <v>55.57</v>
       </c>
       <c r="D11" t="n">
         <v>72</v>
       </c>
       <c r="E11" t="n">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="F11" t="n">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H11" t="n">
@@ -4335,7 +4335,7 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\is-voicebox-review-2026-worth-it-for-small-business</t>
+          <t>D:\AFFILATE BOT\data\research\is-atlassian-team-launches-ai-native-jira-tools-for-the-full-development-workflow-worth-it-for-small-business</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish ready daily articles 2026-07-31
</commit_message>
<xml_diff>
--- a/data/master_dashboard.xlsx
+++ b/data/master_dashboard.xlsx
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="9">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="10">
@@ -3532,16 +3532,16 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>impeccable-review-2026-pricing-cost-and-roi</t>
+          <t>best-impeccable-review-2026-workflows-and-use-cases</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>impeccable Review 2026 pricing cost and ROI</t>
+          <t>best impeccable Review 2026 workflows and use cases</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>50.71</v>
+        <v>52.14</v>
       </c>
       <c r="D2" t="n">
         <v>72</v>
@@ -3561,7 +3561,7 @@
         <v>68</v>
       </c>
       <c r="I2" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J2" t="n">
         <v>45</v>
@@ -3606,23 +3606,23 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\impeccable-review-2026-pricing-cost-and-roi</t>
+          <t>D:\AFFILATE BOT\data\research\best-impeccable-review-2026-workflows-and-use-cases</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ego-lite-review-2026-pricing-cost-and-roi</t>
+          <t>best-ego-lite-review-2026-workflows-and-use-cases</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ego-lite Review 2026 pricing cost and ROI</t>
+          <t>best ego-lite Review 2026 workflows and use cases</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>50.71</v>
+        <v>52.14</v>
       </c>
       <c r="D3" t="n">
         <v>72</v>
@@ -3642,7 +3642,7 @@
         <v>68</v>
       </c>
       <c r="I3" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J3" t="n">
         <v>45</v>
@@ -3687,43 +3687,43 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\ego-lite-review-2026-pricing-cost-and-roi</t>
+          <t>D:\AFFILATE BOT\data\research\best-ego-lite-review-2026-workflows-and-use-cases</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>impeccable-review-2026-comparison-and-alternatives</t>
+          <t>impeccable-review-2026-pricing-cost-and-roi</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>impeccable Review 2026 comparison and alternatives</t>
+          <t>impeccable Review 2026 pricing cost and ROI</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>54.43</v>
+        <v>50.71</v>
       </c>
       <c r="D4" t="n">
         <v>72</v>
       </c>
       <c r="E4" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="F4" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H4" t="n">
         <v>68</v>
       </c>
       <c r="I4" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J4" t="n">
         <v>45</v>
@@ -3758,7 +3758,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -3768,43 +3768,43 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\impeccable-review-2026-comparison-and-alternatives</t>
+          <t>D:\AFFILATE BOT\data\research\impeccable-review-2026-pricing-cost-and-roi</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ego-lite-review-2026-comparison-and-alternatives</t>
+          <t>ego-lite-review-2026-pricing-cost-and-roi</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ego-lite Review 2026 comparison and alternatives</t>
+          <t>ego-lite Review 2026 pricing cost and ROI</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>54.43</v>
+        <v>50.71</v>
       </c>
       <c r="D5" t="n">
         <v>72</v>
       </c>
       <c r="E5" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="F5" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H5" t="n">
         <v>68</v>
       </c>
       <c r="I5" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J5" t="n">
         <v>45</v>
@@ -3839,7 +3839,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -3849,36 +3849,36 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\ego-lite-review-2026-comparison-and-alternatives</t>
+          <t>D:\AFFILATE BOT\data\research\ego-lite-review-2026-pricing-cost-and-roi</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>impeccable-review-2026</t>
+          <t>impeccable-review-2026-comparison-and-alternatives</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>impeccable Review 2026</t>
+          <t>impeccable Review 2026 comparison and alternatives</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>52.14</v>
+        <v>54.43</v>
       </c>
       <c r="D6" t="n">
         <v>72</v>
       </c>
       <c r="E6" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="F6" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H6" t="n">
@@ -3920,7 +3920,7 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -3930,36 +3930,36 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\impeccable-review-2026</t>
+          <t>D:\AFFILATE BOT\data\research\impeccable-review-2026-comparison-and-alternatives</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>chat2db-review-2026</t>
+          <t>ego-lite-review-2026-comparison-and-alternatives</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Chat2DB Review 2026</t>
+          <t>ego-lite Review 2026 comparison and alternatives</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>52.14</v>
+        <v>54.43</v>
       </c>
       <c r="D7" t="n">
         <v>72</v>
       </c>
       <c r="E7" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="F7" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H7" t="n">
@@ -4001,7 +4001,7 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -4011,19 +4011,19 @@
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\chat2db-review-2026</t>
+          <t>D:\AFFILATE BOT\data\research\ego-lite-review-2026-comparison-and-alternatives</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>instatic-review-2026</t>
+          <t>impeccable-review-2026</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Instatic Review 2026</t>
+          <t>impeccable Review 2026</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -4092,19 +4092,19 @@
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\instatic-review-2026</t>
+          <t>D:\AFFILATE BOT\data\research\impeccable-review-2026</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ego-lite-review-2026</t>
+          <t>chat2db-review-2026</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ego-lite Review 2026</t>
+          <t>Chat2DB Review 2026</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -4173,23 +4173,23 @@
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\ego-lite-review-2026</t>
+          <t>D:\AFFILATE BOT\data\research\chat2db-review-2026</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>open-code-review-review-2026</t>
+          <t>instatic-review-2026</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>open-code-review Review 2026</t>
+          <t>Instatic Review 2026</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>53.14</v>
+        <v>52.14</v>
       </c>
       <c r="D10" t="n">
         <v>72</v>
@@ -4215,7 +4215,7 @@
         <v>45</v>
       </c>
       <c r="K10" t="n">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="L10" t="n">
         <v>20</v>
@@ -4254,36 +4254,36 @@
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\open-code-review-review-2026</t>
+          <t>D:\AFFILATE BOT\data\research\instatic-review-2026</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>is-atlassian-team-launches-ai-native-jira-tools-for-the-full-development-workflow-worth-it-for-small-business</t>
+          <t>ego-lite-review-2026</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>is Atlassian (TEAM) Launches AI Native Jira Tools For The Full Development Workflow worth it for small business</t>
+          <t>ego-lite Review 2026</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>55.57</v>
+        <v>52.14</v>
       </c>
       <c r="D11" t="n">
         <v>72</v>
       </c>
       <c r="E11" t="n">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="F11" t="n">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H11" t="n">
@@ -4325,7 +4325,7 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -4335,7 +4335,7 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\is-atlassian-team-launches-ai-native-jira-tools-for-the-full-development-workflow-worth-it-for-small-business</t>
+          <t>D:\AFFILATE BOT\data\research\ego-lite-review-2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish ready daily articles 2026-08-01
</commit_message>
<xml_diff>
--- a/data/master_dashboard.xlsx
+++ b/data/master_dashboard.xlsx
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="9">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="10">
@@ -3532,12 +3532,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>best-impeccable-review-2026-workflows-and-use-cases</t>
+          <t>common-impeccable-review-2026-mistakes-and-troubleshooting</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>best impeccable Review 2026 workflows and use cases</t>
+          <t>common impeccable Review 2026 mistakes and troubleshooting</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -3606,19 +3606,19 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\best-impeccable-review-2026-workflows-and-use-cases</t>
+          <t>D:\AFFILATE BOT\data\research\common-impeccable-review-2026-mistakes-and-troubleshooting</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>best-ego-lite-review-2026-workflows-and-use-cases</t>
+          <t>common-ego-lite-review-2026-mistakes-and-troubleshooting</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>best ego-lite Review 2026 workflows and use cases</t>
+          <t>common ego-lite Review 2026 mistakes and troubleshooting</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -3687,23 +3687,23 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\best-ego-lite-review-2026-workflows-and-use-cases</t>
+          <t>D:\AFFILATE BOT\data\research\common-ego-lite-review-2026-mistakes-and-troubleshooting</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>impeccable-review-2026-pricing-cost-and-roi</t>
+          <t>best-impeccable-review-2026-workflows-and-use-cases</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>impeccable Review 2026 pricing cost and ROI</t>
+          <t>best impeccable Review 2026 workflows and use cases</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>50.71</v>
+        <v>52.14</v>
       </c>
       <c r="D4" t="n">
         <v>72</v>
@@ -3723,7 +3723,7 @@
         <v>68</v>
       </c>
       <c r="I4" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J4" t="n">
         <v>45</v>
@@ -3768,23 +3768,23 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\impeccable-review-2026-pricing-cost-and-roi</t>
+          <t>D:\AFFILATE BOT\data\research\best-impeccable-review-2026-workflows-and-use-cases</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ego-lite-review-2026-pricing-cost-and-roi</t>
+          <t>best-ego-lite-review-2026-workflows-and-use-cases</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ego-lite Review 2026 pricing cost and ROI</t>
+          <t>best ego-lite Review 2026 workflows and use cases</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>50.71</v>
+        <v>52.14</v>
       </c>
       <c r="D5" t="n">
         <v>72</v>
@@ -3804,7 +3804,7 @@
         <v>68</v>
       </c>
       <c r="I5" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J5" t="n">
         <v>45</v>
@@ -3849,43 +3849,43 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\ego-lite-review-2026-pricing-cost-and-roi</t>
+          <t>D:\AFFILATE BOT\data\research\best-ego-lite-review-2026-workflows-and-use-cases</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>impeccable-review-2026-comparison-and-alternatives</t>
+          <t>impeccable-review-2026-pricing-cost-and-roi</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>impeccable Review 2026 comparison and alternatives</t>
+          <t>impeccable Review 2026 pricing cost and ROI</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>54.43</v>
+        <v>50.71</v>
       </c>
       <c r="D6" t="n">
         <v>72</v>
       </c>
       <c r="E6" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="F6" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H6" t="n">
         <v>68</v>
       </c>
       <c r="I6" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J6" t="n">
         <v>45</v>
@@ -3920,7 +3920,7 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -3930,43 +3930,43 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\impeccable-review-2026-comparison-and-alternatives</t>
+          <t>D:\AFFILATE BOT\data\research\impeccable-review-2026-pricing-cost-and-roi</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ego-lite-review-2026-comparison-and-alternatives</t>
+          <t>ego-lite-review-2026-pricing-cost-and-roi</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ego-lite Review 2026 comparison and alternatives</t>
+          <t>ego-lite Review 2026 pricing cost and ROI</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>54.43</v>
+        <v>50.71</v>
       </c>
       <c r="D7" t="n">
         <v>72</v>
       </c>
       <c r="E7" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="F7" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H7" t="n">
         <v>68</v>
       </c>
       <c r="I7" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J7" t="n">
         <v>45</v>
@@ -4001,7 +4001,7 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -4011,36 +4011,36 @@
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\ego-lite-review-2026-comparison-and-alternatives</t>
+          <t>D:\AFFILATE BOT\data\research\ego-lite-review-2026-pricing-cost-and-roi</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>impeccable-review-2026</t>
+          <t>impeccable-review-2026-comparison-and-alternatives</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>impeccable Review 2026</t>
+          <t>impeccable Review 2026 comparison and alternatives</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>52.14</v>
+        <v>54.43</v>
       </c>
       <c r="D8" t="n">
         <v>72</v>
       </c>
       <c r="E8" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="F8" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H8" t="n">
@@ -4082,7 +4082,7 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -4092,36 +4092,36 @@
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\impeccable-review-2026</t>
+          <t>D:\AFFILATE BOT\data\research\impeccable-review-2026-comparison-and-alternatives</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>chat2db-review-2026</t>
+          <t>ego-lite-review-2026-comparison-and-alternatives</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Chat2DB Review 2026</t>
+          <t>ego-lite Review 2026 comparison and alternatives</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>52.14</v>
+        <v>54.43</v>
       </c>
       <c r="D9" t="n">
         <v>72</v>
       </c>
       <c r="E9" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="F9" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H9" t="n">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -4173,19 +4173,19 @@
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\chat2db-review-2026</t>
+          <t>D:\AFFILATE BOT\data\research\ego-lite-review-2026-comparison-and-alternatives</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>instatic-review-2026</t>
+          <t>impeccable-review-2026</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Instatic Review 2026</t>
+          <t>impeccable Review 2026</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -4254,19 +4254,19 @@
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\instatic-review-2026</t>
+          <t>D:\AFFILATE BOT\data\research\impeccable-review-2026</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ego-lite-review-2026</t>
+          <t>chat2db-review-2026</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ego-lite Review 2026</t>
+          <t>Chat2DB Review 2026</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -4335,7 +4335,7 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\ego-lite-review-2026</t>
+          <t>D:\AFFILATE BOT\data\research\chat2db-review-2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish ready daily articles 2026-08-03
</commit_message>
<xml_diff>
--- a/data/master_dashboard.xlsx
+++ b/data/master_dashboard.xlsx
@@ -472,7 +472,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6">
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="9">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="10">
@@ -3532,57 +3532,57 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>common-impeccable-review-2026-mistakes-and-troubleshooting</t>
+          <t>ai-productivity-tools-pricing</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>common impeccable Review 2026 mistakes and troubleshooting</t>
+          <t>ai productivity tools pricing</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>52.14</v>
+        <v>60.79</v>
       </c>
       <c r="D2" t="n">
         <v>72</v>
       </c>
       <c r="E2" t="n">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="F2" t="n">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["affiliate_networks", "integrations", "use_cases", "target_audience", "competitors"]</t>
         </is>
       </c>
       <c r="H2" t="n">
         <v>68</v>
       </c>
       <c r="I2" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J2" t="n">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="K2" t="n">
-        <v>54</v>
+        <v>88.5</v>
       </c>
       <c r="L2" t="n">
-        <v>20</v>
+        <v>98</v>
       </c>
       <c r="M2" t="n">
-        <v>20</v>
+        <v>98</v>
       </c>
       <c r="N2" t="n">
-        <v>10</v>
+        <v>95</v>
       </c>
       <c r="O2" t="n">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="P2" t="n">
-        <v>80</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -3591,51 +3591,51 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>needs enrichment</t>
+          <t>ready</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["Notion", "Gamma", "Notion AI"]</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\common-impeccable-review-2026-mistakes-and-troubleshooting</t>
+          <t>D:\AFFILATE BOT\data\research\ai-productivity-tools-pricing</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>common-ego-lite-review-2026-mistakes-and-troubleshooting</t>
+          <t>ai-meeting-software-alternatives</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>common ego-lite Review 2026 mistakes and troubleshooting</t>
+          <t>ai meeting software alternatives</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>52.14</v>
+        <v>59.93</v>
       </c>
       <c r="D3" t="n">
         <v>72</v>
       </c>
       <c r="E3" t="n">
-        <v>36</v>
+        <v>76</v>
       </c>
       <c r="F3" t="n">
-        <v>36</v>
+        <v>76</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["affiliate_networks", "integrations", "competitors", "use_cases", "target_audience"]</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -3645,25 +3645,25 @@
         <v>80</v>
       </c>
       <c r="J3" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="K3" t="n">
-        <v>54</v>
+        <v>64.5</v>
       </c>
       <c r="L3" t="n">
-        <v>20</v>
+        <v>97</v>
       </c>
       <c r="M3" t="n">
-        <v>20</v>
+        <v>98</v>
       </c>
       <c r="N3" t="n">
-        <v>10</v>
+        <v>97</v>
       </c>
       <c r="O3" t="n">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="P3" t="n">
-        <v>80</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -3677,29 +3677,29 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["Reclaim AI"]</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\common-ego-lite-review-2026-mistakes-and-troubleshooting</t>
+          <t>D:\AFFILATE BOT\data\research\ai-meeting-software-alternatives</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>best-impeccable-review-2026-workflows-and-use-cases</t>
+          <t>common-impeccable-review-2026-mistakes-and-troubleshooting</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>best impeccable Review 2026 workflows and use cases</t>
+          <t>common impeccable Review 2026 mistakes and troubleshooting</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -3768,19 +3768,19 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\best-impeccable-review-2026-workflows-and-use-cases</t>
+          <t>D:\AFFILATE BOT\data\research\common-impeccable-review-2026-mistakes-and-troubleshooting</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>best-ego-lite-review-2026-workflows-and-use-cases</t>
+          <t>common-ego-lite-review-2026-mistakes-and-troubleshooting</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>best ego-lite Review 2026 workflows and use cases</t>
+          <t>common ego-lite Review 2026 mistakes and troubleshooting</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -3849,23 +3849,23 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\best-ego-lite-review-2026-workflows-and-use-cases</t>
+          <t>D:\AFFILATE BOT\data\research\common-ego-lite-review-2026-mistakes-and-troubleshooting</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>impeccable-review-2026-pricing-cost-and-roi</t>
+          <t>best-impeccable-review-2026-workflows-and-use-cases</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>impeccable Review 2026 pricing cost and ROI</t>
+          <t>best impeccable Review 2026 workflows and use cases</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>50.71</v>
+        <v>52.14</v>
       </c>
       <c r="D6" t="n">
         <v>72</v>
@@ -3885,7 +3885,7 @@
         <v>68</v>
       </c>
       <c r="I6" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J6" t="n">
         <v>45</v>
@@ -3930,23 +3930,23 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\impeccable-review-2026-pricing-cost-and-roi</t>
+          <t>D:\AFFILATE BOT\data\research\best-impeccable-review-2026-workflows-and-use-cases</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ego-lite-review-2026-pricing-cost-and-roi</t>
+          <t>best-ego-lite-review-2026-workflows-and-use-cases</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ego-lite Review 2026 pricing cost and ROI</t>
+          <t>best ego-lite Review 2026 workflows and use cases</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>50.71</v>
+        <v>52.14</v>
       </c>
       <c r="D7" t="n">
         <v>72</v>
@@ -3966,7 +3966,7 @@
         <v>68</v>
       </c>
       <c r="I7" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J7" t="n">
         <v>45</v>
@@ -4011,43 +4011,43 @@
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\ego-lite-review-2026-pricing-cost-and-roi</t>
+          <t>D:\AFFILATE BOT\data\research\best-ego-lite-review-2026-workflows-and-use-cases</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>impeccable-review-2026-comparison-and-alternatives</t>
+          <t>impeccable-review-2026-pricing-cost-and-roi</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>impeccable Review 2026 comparison and alternatives</t>
+          <t>impeccable Review 2026 pricing cost and ROI</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>54.43</v>
+        <v>50.71</v>
       </c>
       <c r="D8" t="n">
         <v>72</v>
       </c>
       <c r="E8" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="F8" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H8" t="n">
         <v>68</v>
       </c>
       <c r="I8" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J8" t="n">
         <v>45</v>
@@ -4082,7 +4082,7 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -4092,43 +4092,43 @@
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\impeccable-review-2026-comparison-and-alternatives</t>
+          <t>D:\AFFILATE BOT\data\research\impeccable-review-2026-pricing-cost-and-roi</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ego-lite-review-2026-comparison-and-alternatives</t>
+          <t>ego-lite-review-2026-pricing-cost-and-roi</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ego-lite Review 2026 comparison and alternatives</t>
+          <t>ego-lite Review 2026 pricing cost and ROI</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>54.43</v>
+        <v>50.71</v>
       </c>
       <c r="D9" t="n">
         <v>72</v>
       </c>
       <c r="E9" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="F9" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H9" t="n">
         <v>68</v>
       </c>
       <c r="I9" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J9" t="n">
         <v>45</v>
@@ -4163,7 +4163,7 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -4173,36 +4173,36 @@
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\ego-lite-review-2026-comparison-and-alternatives</t>
+          <t>D:\AFFILATE BOT\data\research\ego-lite-review-2026-pricing-cost-and-roi</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>impeccable-review-2026</t>
+          <t>impeccable-review-2026-comparison-and-alternatives</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>impeccable Review 2026</t>
+          <t>impeccable Review 2026 comparison and alternatives</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>52.14</v>
+        <v>54.43</v>
       </c>
       <c r="D10" t="n">
         <v>72</v>
       </c>
       <c r="E10" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="F10" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H10" t="n">
@@ -4244,7 +4244,7 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -4254,36 +4254,36 @@
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\impeccable-review-2026</t>
+          <t>D:\AFFILATE BOT\data\research\impeccable-review-2026-comparison-and-alternatives</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>chat2db-review-2026</t>
+          <t>ego-lite-review-2026-comparison-and-alternatives</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Chat2DB Review 2026</t>
+          <t>ego-lite Review 2026 comparison and alternatives</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>52.14</v>
+        <v>54.43</v>
       </c>
       <c r="D11" t="n">
         <v>72</v>
       </c>
       <c r="E11" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="F11" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H11" t="n">
@@ -4325,7 +4325,7 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -4335,7 +4335,7 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\chat2db-review-2026</t>
+          <t>D:\AFFILATE BOT\data\research\ego-lite-review-2026-comparison-and-alternatives</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish ready daily articles 2026-08-04
</commit_message>
<xml_diff>
--- a/data/master_dashboard.xlsx
+++ b/data/master_dashboard.xlsx
@@ -472,7 +472,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6">
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="9">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="10">
@@ -3532,12 +3532,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ai-productivity-tools-pricing</t>
+          <t>how-to-implement-ai-productivity-tools-pricing</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ai productivity tools pricing</t>
+          <t>how to implement ai productivity tools pricing</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -3606,23 +3606,23 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\ai-productivity-tools-pricing</t>
+          <t>D:\AFFILATE BOT\data\research\how-to-implement-ai-productivity-tools-pricing</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ai-meeting-software-alternatives</t>
+          <t>how-to-implement-ai-meeting-software-alternatives</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ai meeting software alternatives</t>
+          <t>how to implement ai meeting software alternatives</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>59.93</v>
+        <v>62.93</v>
       </c>
       <c r="D3" t="n">
         <v>72</v>
@@ -3648,7 +3648,7 @@
         <v>49</v>
       </c>
       <c r="K3" t="n">
-        <v>64.5</v>
+        <v>85.5</v>
       </c>
       <c r="L3" t="n">
         <v>97</v>
@@ -3672,7 +3672,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>needs enrichment</t>
+          <t>ready</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -3687,64 +3687,64 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\ai-meeting-software-alternatives</t>
+          <t>D:\AFFILATE BOT\data\research\how-to-implement-ai-meeting-software-alternatives</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>common-impeccable-review-2026-mistakes-and-troubleshooting</t>
+          <t>ai-productivity-tools-pricing</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>common impeccable Review 2026 mistakes and troubleshooting</t>
+          <t>ai productivity tools pricing</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>52.14</v>
+        <v>60.79</v>
       </c>
       <c r="D4" t="n">
         <v>72</v>
       </c>
       <c r="E4" t="n">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="F4" t="n">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["affiliate_networks", "integrations", "use_cases", "target_audience", "competitors"]</t>
         </is>
       </c>
       <c r="H4" t="n">
         <v>68</v>
       </c>
       <c r="I4" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J4" t="n">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="K4" t="n">
-        <v>54</v>
+        <v>88.5</v>
       </c>
       <c r="L4" t="n">
-        <v>20</v>
+        <v>98</v>
       </c>
       <c r="M4" t="n">
-        <v>20</v>
+        <v>98</v>
       </c>
       <c r="N4" t="n">
-        <v>10</v>
+        <v>95</v>
       </c>
       <c r="O4" t="n">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="P4" t="n">
-        <v>80</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -3753,51 +3753,51 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>needs enrichment</t>
+          <t>ready</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["Notion", "Gamma", "Notion AI"]</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\common-impeccable-review-2026-mistakes-and-troubleshooting</t>
+          <t>D:\AFFILATE BOT\data\research\ai-productivity-tools-pricing</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>common-ego-lite-review-2026-mistakes-and-troubleshooting</t>
+          <t>ai-meeting-software-alternatives</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>common ego-lite Review 2026 mistakes and troubleshooting</t>
+          <t>ai meeting software alternatives</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>52.14</v>
+        <v>59.93</v>
       </c>
       <c r="D5" t="n">
         <v>72</v>
       </c>
       <c r="E5" t="n">
-        <v>36</v>
+        <v>76</v>
       </c>
       <c r="F5" t="n">
-        <v>36</v>
+        <v>76</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["affiliate_networks", "integrations", "competitors", "use_cases", "target_audience"]</t>
         </is>
       </c>
       <c r="H5" t="n">
@@ -3807,25 +3807,25 @@
         <v>80</v>
       </c>
       <c r="J5" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="K5" t="n">
-        <v>54</v>
+        <v>64.5</v>
       </c>
       <c r="L5" t="n">
-        <v>20</v>
+        <v>97</v>
       </c>
       <c r="M5" t="n">
-        <v>20</v>
+        <v>98</v>
       </c>
       <c r="N5" t="n">
-        <v>10</v>
+        <v>97</v>
       </c>
       <c r="O5" t="n">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="P5" t="n">
-        <v>80</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -3839,29 +3839,29 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["Reclaim AI"]</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\common-ego-lite-review-2026-mistakes-and-troubleshooting</t>
+          <t>D:\AFFILATE BOT\data\research\ai-meeting-software-alternatives</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>best-impeccable-review-2026-workflows-and-use-cases</t>
+          <t>common-impeccable-review-2026-mistakes-and-troubleshooting</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>best impeccable Review 2026 workflows and use cases</t>
+          <t>common impeccable Review 2026 mistakes and troubleshooting</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -3930,19 +3930,19 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\best-impeccable-review-2026-workflows-and-use-cases</t>
+          <t>D:\AFFILATE BOT\data\research\common-impeccable-review-2026-mistakes-and-troubleshooting</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>best-ego-lite-review-2026-workflows-and-use-cases</t>
+          <t>common-ego-lite-review-2026-mistakes-and-troubleshooting</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>best ego-lite Review 2026 workflows and use cases</t>
+          <t>common ego-lite Review 2026 mistakes and troubleshooting</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -4011,23 +4011,23 @@
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\best-ego-lite-review-2026-workflows-and-use-cases</t>
+          <t>D:\AFFILATE BOT\data\research\common-ego-lite-review-2026-mistakes-and-troubleshooting</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>impeccable-review-2026-pricing-cost-and-roi</t>
+          <t>best-impeccable-review-2026-workflows-and-use-cases</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>impeccable Review 2026 pricing cost and ROI</t>
+          <t>best impeccable Review 2026 workflows and use cases</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>50.71</v>
+        <v>52.14</v>
       </c>
       <c r="D8" t="n">
         <v>72</v>
@@ -4047,7 +4047,7 @@
         <v>68</v>
       </c>
       <c r="I8" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J8" t="n">
         <v>45</v>
@@ -4092,23 +4092,23 @@
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\impeccable-review-2026-pricing-cost-and-roi</t>
+          <t>D:\AFFILATE BOT\data\research\best-impeccable-review-2026-workflows-and-use-cases</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ego-lite-review-2026-pricing-cost-and-roi</t>
+          <t>best-ego-lite-review-2026-workflows-and-use-cases</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ego-lite Review 2026 pricing cost and ROI</t>
+          <t>best ego-lite Review 2026 workflows and use cases</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>50.71</v>
+        <v>52.14</v>
       </c>
       <c r="D9" t="n">
         <v>72</v>
@@ -4128,7 +4128,7 @@
         <v>68</v>
       </c>
       <c r="I9" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J9" t="n">
         <v>45</v>
@@ -4173,43 +4173,43 @@
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\ego-lite-review-2026-pricing-cost-and-roi</t>
+          <t>D:\AFFILATE BOT\data\research\best-ego-lite-review-2026-workflows-and-use-cases</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>impeccable-review-2026-comparison-and-alternatives</t>
+          <t>impeccable-review-2026-pricing-cost-and-roi</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>impeccable Review 2026 comparison and alternatives</t>
+          <t>impeccable Review 2026 pricing cost and ROI</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>54.43</v>
+        <v>50.71</v>
       </c>
       <c r="D10" t="n">
         <v>72</v>
       </c>
       <c r="E10" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="F10" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H10" t="n">
         <v>68</v>
       </c>
       <c r="I10" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J10" t="n">
         <v>45</v>
@@ -4244,7 +4244,7 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -4254,43 +4254,43 @@
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\impeccable-review-2026-comparison-and-alternatives</t>
+          <t>D:\AFFILATE BOT\data\research\impeccable-review-2026-pricing-cost-and-roi</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ego-lite-review-2026-comparison-and-alternatives</t>
+          <t>ego-lite-review-2026-pricing-cost-and-roi</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ego-lite Review 2026 comparison and alternatives</t>
+          <t>ego-lite Review 2026 pricing cost and ROI</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>54.43</v>
+        <v>50.71</v>
       </c>
       <c r="D11" t="n">
         <v>72</v>
       </c>
       <c r="E11" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="F11" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H11" t="n">
         <v>68</v>
       </c>
       <c r="I11" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J11" t="n">
         <v>45</v>
@@ -4325,7 +4325,7 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -4335,7 +4335,7 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\ego-lite-review-2026-comparison-and-alternatives</t>
+          <t>D:\AFFILATE BOT\data\research\ego-lite-review-2026-pricing-cost-and-roi</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish ready daily articles 2026-08-08
</commit_message>
<xml_diff>
--- a/data/master_dashboard.xlsx
+++ b/data/master_dashboard.xlsx
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="9">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="10">
@@ -3532,12 +3532,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>how-to-implement-ai-productivity-tools-pricing</t>
+          <t>common-ai-productivity-tools-pricing-mistakes-and-troubleshooting</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>how to implement ai productivity tools pricing</t>
+          <t>common ai productivity tools pricing mistakes and troubleshooting</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -3606,19 +3606,19 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\how-to-implement-ai-productivity-tools-pricing</t>
+          <t>D:\AFFILATE BOT\data\research\common-ai-productivity-tools-pricing-mistakes-and-troubleshooting</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>how-to-implement-ai-meeting-software-alternatives</t>
+          <t>common-ai-meeting-software-alternatives-mistakes-and-troubleshooting</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>how to implement ai meeting software alternatives</t>
+          <t>common ai meeting software alternatives mistakes and troubleshooting</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -3657,7 +3657,7 @@
         <v>98</v>
       </c>
       <c r="N3" t="n">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="O3" t="n">
         <v>77</v>
@@ -3687,19 +3687,19 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\how-to-implement-ai-meeting-software-alternatives</t>
+          <t>D:\AFFILATE BOT\data\research\common-ai-meeting-software-alternatives-mistakes-and-troubleshooting</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ai-productivity-tools-pricing</t>
+          <t>how-to-implement-ai-productivity-tools-pricing</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ai productivity tools pricing</t>
+          <t>how to implement ai productivity tools pricing</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -3768,23 +3768,23 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\ai-productivity-tools-pricing</t>
+          <t>D:\AFFILATE BOT\data\research\how-to-implement-ai-productivity-tools-pricing</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ai-meeting-software-alternatives</t>
+          <t>how-to-implement-ai-meeting-software-alternatives</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ai meeting software alternatives</t>
+          <t>how to implement ai meeting software alternatives</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>59.93</v>
+        <v>62.93</v>
       </c>
       <c r="D5" t="n">
         <v>72</v>
@@ -3810,7 +3810,7 @@
         <v>49</v>
       </c>
       <c r="K5" t="n">
-        <v>64.5</v>
+        <v>85.5</v>
       </c>
       <c r="L5" t="n">
         <v>97</v>
@@ -3834,7 +3834,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>needs enrichment</t>
+          <t>ready</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -3849,64 +3849,64 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\ai-meeting-software-alternatives</t>
+          <t>D:\AFFILATE BOT\data\research\how-to-implement-ai-meeting-software-alternatives</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>common-impeccable-review-2026-mistakes-and-troubleshooting</t>
+          <t>ai-productivity-tools-pricing</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>common impeccable Review 2026 mistakes and troubleshooting</t>
+          <t>ai productivity tools pricing</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>52.14</v>
+        <v>60.79</v>
       </c>
       <c r="D6" t="n">
         <v>72</v>
       </c>
       <c r="E6" t="n">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="F6" t="n">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["affiliate_networks", "integrations", "use_cases", "target_audience", "competitors"]</t>
         </is>
       </c>
       <c r="H6" t="n">
         <v>68</v>
       </c>
       <c r="I6" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J6" t="n">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="K6" t="n">
-        <v>54</v>
+        <v>88.5</v>
       </c>
       <c r="L6" t="n">
-        <v>20</v>
+        <v>98</v>
       </c>
       <c r="M6" t="n">
-        <v>20</v>
+        <v>98</v>
       </c>
       <c r="N6" t="n">
-        <v>10</v>
+        <v>95</v>
       </c>
       <c r="O6" t="n">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="P6" t="n">
-        <v>80</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -3915,51 +3915,51 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>needs enrichment</t>
+          <t>ready</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["Notion", "Gamma", "Notion AI"]</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\common-impeccable-review-2026-mistakes-and-troubleshooting</t>
+          <t>D:\AFFILATE BOT\data\research\ai-productivity-tools-pricing</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>common-ego-lite-review-2026-mistakes-and-troubleshooting</t>
+          <t>ai-meeting-software-alternatives</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>common ego-lite Review 2026 mistakes and troubleshooting</t>
+          <t>ai meeting software alternatives</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>52.14</v>
+        <v>59.93</v>
       </c>
       <c r="D7" t="n">
         <v>72</v>
       </c>
       <c r="E7" t="n">
-        <v>36</v>
+        <v>76</v>
       </c>
       <c r="F7" t="n">
-        <v>36</v>
+        <v>76</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["affiliate_networks", "integrations", "competitors", "use_cases", "target_audience"]</t>
         </is>
       </c>
       <c r="H7" t="n">
@@ -3969,25 +3969,25 @@
         <v>80</v>
       </c>
       <c r="J7" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="K7" t="n">
-        <v>54</v>
+        <v>64.5</v>
       </c>
       <c r="L7" t="n">
-        <v>20</v>
+        <v>97</v>
       </c>
       <c r="M7" t="n">
-        <v>20</v>
+        <v>98</v>
       </c>
       <c r="N7" t="n">
-        <v>10</v>
+        <v>97</v>
       </c>
       <c r="O7" t="n">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="P7" t="n">
-        <v>80</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -4001,29 +4001,29 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["Reclaim AI"]</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\common-ego-lite-review-2026-mistakes-and-troubleshooting</t>
+          <t>D:\AFFILATE BOT\data\research\ai-meeting-software-alternatives</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>best-impeccable-review-2026-workflows-and-use-cases</t>
+          <t>common-impeccable-review-2026-mistakes-and-troubleshooting</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>best impeccable Review 2026 workflows and use cases</t>
+          <t>common impeccable Review 2026 mistakes and troubleshooting</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -4092,19 +4092,19 @@
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\best-impeccable-review-2026-workflows-and-use-cases</t>
+          <t>D:\AFFILATE BOT\data\research\common-impeccable-review-2026-mistakes-and-troubleshooting</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>best-ego-lite-review-2026-workflows-and-use-cases</t>
+          <t>common-ego-lite-review-2026-mistakes-and-troubleshooting</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>best ego-lite Review 2026 workflows and use cases</t>
+          <t>common ego-lite Review 2026 mistakes and troubleshooting</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -4173,23 +4173,23 @@
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\best-ego-lite-review-2026-workflows-and-use-cases</t>
+          <t>D:\AFFILATE BOT\data\research\common-ego-lite-review-2026-mistakes-and-troubleshooting</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>impeccable-review-2026-pricing-cost-and-roi</t>
+          <t>best-impeccable-review-2026-workflows-and-use-cases</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>impeccable Review 2026 pricing cost and ROI</t>
+          <t>best impeccable Review 2026 workflows and use cases</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>50.71</v>
+        <v>52.14</v>
       </c>
       <c r="D10" t="n">
         <v>72</v>
@@ -4209,7 +4209,7 @@
         <v>68</v>
       </c>
       <c r="I10" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J10" t="n">
         <v>45</v>
@@ -4254,23 +4254,23 @@
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\impeccable-review-2026-pricing-cost-and-roi</t>
+          <t>D:\AFFILATE BOT\data\research\best-impeccable-review-2026-workflows-and-use-cases</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ego-lite-review-2026-pricing-cost-and-roi</t>
+          <t>best-ego-lite-review-2026-workflows-and-use-cases</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ego-lite Review 2026 pricing cost and ROI</t>
+          <t>best ego-lite Review 2026 workflows and use cases</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>50.71</v>
+        <v>52.14</v>
       </c>
       <c r="D11" t="n">
         <v>72</v>
@@ -4290,7 +4290,7 @@
         <v>68</v>
       </c>
       <c r="I11" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J11" t="n">
         <v>45</v>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\ego-lite-review-2026-pricing-cost-and-roi</t>
+          <t>D:\AFFILATE BOT\data\research\best-ego-lite-review-2026-workflows-and-use-cases</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish ready daily articles 2026-08-09
</commit_message>
<xml_diff>
--- a/data/master_dashboard.xlsx
+++ b/data/master_dashboard.xlsx
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="9">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="10">
@@ -3532,29 +3532,29 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>common-ai-productivity-tools-pricing-mistakes-and-troubleshooting</t>
+          <t>is-ai-productivity-tools-pricing-worth-it-for-small-business</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>common ai productivity tools pricing mistakes and troubleshooting</t>
+          <t>is ai productivity tools pricing worth it for small business</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>60.79</v>
+        <v>63.07</v>
       </c>
       <c r="D2" t="n">
         <v>72</v>
       </c>
       <c r="E2" t="n">
-        <v>60</v>
+        <v>76</v>
       </c>
       <c r="F2" t="n">
-        <v>60</v>
+        <v>76</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>["affiliate_networks", "integrations", "use_cases", "target_audience", "competitors"]</t>
+          <t>["affiliate_networks", "integrations", "competitors", "use_cases", "target_audience"]</t>
         </is>
       </c>
       <c r="H2" t="n">
@@ -3606,19 +3606,19 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\common-ai-productivity-tools-pricing-mistakes-and-troubleshooting</t>
+          <t>D:\AFFILATE BOT\data\research\is-ai-productivity-tools-pricing-worth-it-for-small-business</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>common-ai-meeting-software-alternatives-mistakes-and-troubleshooting</t>
+          <t>is-ai-meeting-software-alternatives-worth-it-for-small-business</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>common ai meeting software alternatives mistakes and troubleshooting</t>
+          <t>is ai meeting software alternatives worth it for small business</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -3687,19 +3687,19 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\common-ai-meeting-software-alternatives-mistakes-and-troubleshooting</t>
+          <t>D:\AFFILATE BOT\data\research\is-ai-meeting-software-alternatives-worth-it-for-small-business</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>how-to-implement-ai-productivity-tools-pricing</t>
+          <t>common-ai-productivity-tools-pricing-mistakes-and-troubleshooting</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>how to implement ai productivity tools pricing</t>
+          <t>common ai productivity tools pricing mistakes and troubleshooting</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -3768,19 +3768,19 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\how-to-implement-ai-productivity-tools-pricing</t>
+          <t>D:\AFFILATE BOT\data\research\common-ai-productivity-tools-pricing-mistakes-and-troubleshooting</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>how-to-implement-ai-meeting-software-alternatives</t>
+          <t>common-ai-meeting-software-alternatives-mistakes-and-troubleshooting</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>how to implement ai meeting software alternatives</t>
+          <t>common ai meeting software alternatives mistakes and troubleshooting</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -3819,7 +3819,7 @@
         <v>98</v>
       </c>
       <c r="N5" t="n">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="O5" t="n">
         <v>77</v>
@@ -3849,19 +3849,19 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\how-to-implement-ai-meeting-software-alternatives</t>
+          <t>D:\AFFILATE BOT\data\research\common-ai-meeting-software-alternatives-mistakes-and-troubleshooting</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ai-productivity-tools-pricing</t>
+          <t>how-to-implement-ai-productivity-tools-pricing</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ai productivity tools pricing</t>
+          <t>how to implement ai productivity tools pricing</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -3930,23 +3930,23 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\ai-productivity-tools-pricing</t>
+          <t>D:\AFFILATE BOT\data\research\how-to-implement-ai-productivity-tools-pricing</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ai-meeting-software-alternatives</t>
+          <t>how-to-implement-ai-meeting-software-alternatives</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ai meeting software alternatives</t>
+          <t>how to implement ai meeting software alternatives</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>59.93</v>
+        <v>62.93</v>
       </c>
       <c r="D7" t="n">
         <v>72</v>
@@ -3972,7 +3972,7 @@
         <v>49</v>
       </c>
       <c r="K7" t="n">
-        <v>64.5</v>
+        <v>85.5</v>
       </c>
       <c r="L7" t="n">
         <v>97</v>
@@ -3996,7 +3996,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>needs enrichment</t>
+          <t>ready</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -4011,64 +4011,64 @@
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\ai-meeting-software-alternatives</t>
+          <t>D:\AFFILATE BOT\data\research\how-to-implement-ai-meeting-software-alternatives</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>common-impeccable-review-2026-mistakes-and-troubleshooting</t>
+          <t>ai-productivity-tools-pricing</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>common impeccable Review 2026 mistakes and troubleshooting</t>
+          <t>ai productivity tools pricing</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>52.14</v>
+        <v>60.79</v>
       </c>
       <c r="D8" t="n">
         <v>72</v>
       </c>
       <c r="E8" t="n">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="F8" t="n">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["affiliate_networks", "integrations", "use_cases", "target_audience", "competitors"]</t>
         </is>
       </c>
       <c r="H8" t="n">
         <v>68</v>
       </c>
       <c r="I8" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J8" t="n">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="K8" t="n">
-        <v>54</v>
+        <v>88.5</v>
       </c>
       <c r="L8" t="n">
-        <v>20</v>
+        <v>98</v>
       </c>
       <c r="M8" t="n">
-        <v>20</v>
+        <v>98</v>
       </c>
       <c r="N8" t="n">
-        <v>10</v>
+        <v>95</v>
       </c>
       <c r="O8" t="n">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="P8" t="n">
-        <v>80</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -4077,51 +4077,51 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>needs enrichment</t>
+          <t>ready</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["Notion", "Gamma", "Notion AI"]</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\common-impeccable-review-2026-mistakes-and-troubleshooting</t>
+          <t>D:\AFFILATE BOT\data\research\ai-productivity-tools-pricing</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>common-ego-lite-review-2026-mistakes-and-troubleshooting</t>
+          <t>ai-meeting-software-alternatives</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>common ego-lite Review 2026 mistakes and troubleshooting</t>
+          <t>ai meeting software alternatives</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>52.14</v>
+        <v>59.93</v>
       </c>
       <c r="D9" t="n">
         <v>72</v>
       </c>
       <c r="E9" t="n">
-        <v>36</v>
+        <v>76</v>
       </c>
       <c r="F9" t="n">
-        <v>36</v>
+        <v>76</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["affiliate_networks", "integrations", "competitors", "use_cases", "target_audience"]</t>
         </is>
       </c>
       <c r="H9" t="n">
@@ -4131,25 +4131,25 @@
         <v>80</v>
       </c>
       <c r="J9" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="K9" t="n">
-        <v>54</v>
+        <v>64.5</v>
       </c>
       <c r="L9" t="n">
-        <v>20</v>
+        <v>97</v>
       </c>
       <c r="M9" t="n">
-        <v>20</v>
+        <v>98</v>
       </c>
       <c r="N9" t="n">
-        <v>10</v>
+        <v>97</v>
       </c>
       <c r="O9" t="n">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="P9" t="n">
-        <v>80</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -4163,29 +4163,29 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["Reclaim AI"]</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\common-ego-lite-review-2026-mistakes-and-troubleshooting</t>
+          <t>D:\AFFILATE BOT\data\research\ai-meeting-software-alternatives</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>best-impeccable-review-2026-workflows-and-use-cases</t>
+          <t>common-impeccable-review-2026-mistakes-and-troubleshooting</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>best impeccable Review 2026 workflows and use cases</t>
+          <t>common impeccable Review 2026 mistakes and troubleshooting</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -4254,19 +4254,19 @@
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\best-impeccable-review-2026-workflows-and-use-cases</t>
+          <t>D:\AFFILATE BOT\data\research\common-impeccable-review-2026-mistakes-and-troubleshooting</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>best-ego-lite-review-2026-workflows-and-use-cases</t>
+          <t>common-ego-lite-review-2026-mistakes-and-troubleshooting</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>best ego-lite Review 2026 workflows and use cases</t>
+          <t>common ego-lite Review 2026 mistakes and troubleshooting</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -4335,7 +4335,7 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\best-ego-lite-review-2026-workflows-and-use-cases</t>
+          <t>D:\AFFILATE BOT\data\research\common-ego-lite-review-2026-mistakes-and-troubleshooting</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish ready daily articles 2026-08-24
</commit_message>
<xml_diff>
--- a/data/master_dashboard.xlsx
+++ b/data/master_dashboard.xlsx
@@ -462,7 +462,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5">
@@ -472,7 +472,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6">
@@ -482,7 +482,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -492,7 +492,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>147</v>
+        <v>151</v>
       </c>
     </row>
     <row r="9">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>147</v>
+        <v>151</v>
       </c>
     </row>
     <row r="10">
@@ -2391,7 +2391,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2463,6 +2463,34 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>tooljet-review-2026</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ToolJet Review 2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>needs_human_review</t>
+        </is>
+      </c>
+      <c r="D3" t="b">
+        <v>1</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-08-20T14:21:17.570501+00:00</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2475,861 +2503,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R11"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>topic</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>slug</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>missing_sources</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>missing_competitors</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>missing_entities</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>missing_affiliate_data</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>priority</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>reason</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>created_at</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>score</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>started_at</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>checked_at</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>latest_score</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>latest_missing_information</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>missing_verified_sources</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>source_status</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>source_confidence</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>meetily Review 2026</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>meetily-review-2026</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>7</v>
-      </c>
-      <c r="D2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E2" t="n">
-        <v>8</v>
-      </c>
-      <c r="F2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>trusted sources are thin; official sources are insufficiently verified; pricing sources need verification; affiliate sources need verification; competitor coverage is limited; entity extraction needs richer tool coverage; 0 usable sources below critical minimum 1; research_quality_score 45.14 below initial threshold 50.0; official_docs_score 0.0 below 20.0; pricing_source_score 0.0 below 20.0; affiliate_source_score 0.0 below 10.0; total_verified_source_score 0.0 below 35.0; verified_sources 0 below 2; official_verified_sources 0 below 1; entity_coverage_score 36.0 below initial threshold 40.0; competitor_coverage_score 10.0 below initial threshold 30.0; freshness_score 0.0 below initial threshold 40.0</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>2026-07-15T22:05:03.930298+00:00</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="K2" t="n">
-        <v>45.14</v>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>2026-07-07T09:38:56.464596+00:00</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-07-07T09:38:56.621091+00:00</t>
-        </is>
-      </c>
-      <c r="N2" t="n">
-        <v>45.14</v>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>["trusted sources are thin", "official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>["official_docs", "pricing_page", "affiliate_program_page", "release_notes", "competitor_article"]</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="R2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>system_prompts_leaks Review 2026</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>system-prompts-leaks-review-2026</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>12</v>
-      </c>
-      <c r="D3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" t="n">
-        <v>8</v>
-      </c>
-      <c r="F3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>trusted sources are thin; official sources are insufficiently verified; pricing sources need verification; affiliate sources need verification; competitor coverage is limited; entity extraction needs richer tool coverage; 0 usable sources below critical minimum 1; research_quality_score 45.14 below initial threshold 50.0; official_docs_score 0.0 below 20.0; pricing_source_score 0.0 below 20.0; affiliate_source_score 0.0 below 10.0; total_verified_source_score 0.0 below 35.0; verified_sources 0 below 2; official_verified_sources 0 below 1; entity_coverage_score 36.0 below initial threshold 40.0; competitor_coverage_score 10.0 below initial threshold 30.0; freshness_score 0.0 below initial threshold 40.0</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>2026-07-15T22:05:04.963085+00:00</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="K3" t="n">
-        <v>45.14</v>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>2026-07-07T09:38:56.645213+00:00</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-07-07T09:38:56.888756+00:00</t>
-        </is>
-      </c>
-      <c r="N3" t="n">
-        <v>45.14</v>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>["trusted sources are thin", "official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>["official_docs", "pricing_page", "affiliate_program_page", "release_notes", "competitor_article"]</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="R3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>agent-skills Review 2026</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>agent-skills-review-2026</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>7</v>
-      </c>
-      <c r="D4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" t="n">
-        <v>8</v>
-      </c>
-      <c r="F4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>trusted sources are thin; official sources are insufficiently verified; pricing sources need verification; affiliate sources need verification; competitor coverage is limited; entity extraction needs richer tool coverage; 0 usable sources below critical minimum 1; research_quality_score 45.14 below initial threshold 50.0; official_docs_score 0.0 below 20.0; pricing_source_score 0.0 below 20.0; affiliate_source_score 0.0 below 10.0; total_verified_source_score 0.0 below 35.0; verified_sources 0 below 2; official_verified_sources 0 below 1; entity_coverage_score 36.0 below initial threshold 40.0; competitor_coverage_score 10.0 below initial threshold 30.0; freshness_score 0.0 below initial threshold 40.0</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>2026-07-15T22:05:02.724397+00:00</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="K4" t="n">
-        <v>45.14</v>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>2026-07-07T09:38:56.917709+00:00</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-07-07T09:38:57.134982+00:00</t>
-        </is>
-      </c>
-      <c r="N4" t="n">
-        <v>45.14</v>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>["trusted sources are thin", "official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>["official_docs", "pricing_page", "affiliate_program_page", "release_notes", "competitor_article"]</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="R4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>last30days-skill Review 2026</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>last30days-skill-review-2026</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>7</v>
-      </c>
-      <c r="D5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" t="n">
-        <v>8</v>
-      </c>
-      <c r="F5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>trusted sources are thin; official sources are insufficiently verified; pricing sources need verification; affiliate sources need verification; competitor coverage is limited; entity extraction needs richer tool coverage; official_docs_score 0.0 below 20.0; pricing_source_score 0.0 below 20.0; affiliate_source_score 0.0 below 10.0; total_verified_source_score 0.0 below 35.0; verified_sources 0 below 1; official_verified_sources 0 below 1</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>2026-07-07T09:39:33.209943+00:00</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="K5" t="n">
-        <v>45.14</v>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>2026-07-07T09:38:57.168661+00:00</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>2026-07-07T09:38:57.331513+00:00</t>
-        </is>
-      </c>
-      <c r="N5" t="n">
-        <v>45.14</v>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>["trusted sources are thin", "official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>["official_docs", "pricing_page", "affiliate_program_page", "release_notes", "competitor_article"]</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="R5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>taste-skill Review 2026</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>taste-skill-review-2026</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>7</v>
-      </c>
-      <c r="D6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" t="n">
-        <v>8</v>
-      </c>
-      <c r="F6" t="n">
-        <v>1</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>trusted sources are thin; official sources are insufficiently verified; pricing sources need verification; affiliate sources need verification; competitor coverage is limited; entity extraction needs richer tool coverage; official_docs_score 0.0 below 20.0; pricing_source_score 0.0 below 20.0; affiliate_source_score 0.0 below 10.0; total_verified_source_score 0.0 below 35.0; verified_sources 0 below 1; official_verified_sources 0 below 1</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>2026-07-07T09:39:33.242931+00:00</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="K6" t="n">
-        <v>45.14</v>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>2026-07-07T09:38:57.363197+00:00</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>2026-07-07T09:38:57.526114+00:00</t>
-        </is>
-      </c>
-      <c r="N6" t="n">
-        <v>45.14</v>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>["trusted sources are thin", "official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>["official_docs", "pricing_page", "affiliate_program_page", "release_notes", "competitor_article"]</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="R6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>karakeep Review 2026</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>karakeep-review-2026</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>7</v>
-      </c>
-      <c r="D7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" t="n">
-        <v>8</v>
-      </c>
-      <c r="F7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>trusted sources are thin; official sources are insufficiently verified; pricing sources need verification; affiliate sources need verification; competitor coverage is limited; entity extraction needs richer tool coverage; official_docs_score 0.0 below 20.0; pricing_source_score 0.0 below 20.0; affiliate_source_score 0.0 below 10.0; total_verified_source_score 0.0 below 35.0; verified_sources 0 below 1; official_verified_sources 0 below 1</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>2026-07-07T09:39:33.271421+00:00</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="K7" t="n">
-        <v>45.14</v>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>2026-07-07T09:38:57.561816+00:00</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>2026-07-07T09:38:57.752632+00:00</t>
-        </is>
-      </c>
-      <c r="N7" t="n">
-        <v>45.14</v>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>["trusted sources are thin", "official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>["official_docs", "pricing_page", "affiliate_program_page", "release_notes", "competitor_article"]</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="R7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>best ai meeting software</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>best-ai-meeting-software</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>9</v>
-      </c>
-      <c r="D8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" t="n">
-        <v>5</v>
-      </c>
-      <c r="F8" t="n">
-        <v>1</v>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>competitor coverage is limited</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>2026-07-07T09:39:48.182992+00:00</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="K8" t="n">
-        <v>57.79</v>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>2026-07-07T09:38:57.779286+00:00</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>2026-07-07T09:38:57.989936+00:00</t>
-        </is>
-      </c>
-      <c r="N8" t="n">
-        <v>57.79</v>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>["competitor coverage is limited"]</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>["competitor_article"]</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>verified</t>
-        </is>
-      </c>
-      <c r="R8" t="n">
-        <v>91.59999999999999</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>best ai voice software</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>best-ai-voice-software</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>9</v>
-      </c>
-      <c r="D9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" t="n">
-        <v>5</v>
-      </c>
-      <c r="F9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>competitor coverage is limited</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>2026-07-07T09:39:48.204668+00:00</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="K9" t="n">
-        <v>57.79</v>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>2026-07-07T09:38:58.035479+00:00</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>2026-07-07T09:38:58.300049+00:00</t>
-        </is>
-      </c>
-      <c r="N9" t="n">
-        <v>57.79</v>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>["competitor coverage is limited"]</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>["competitor_article"]</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>verified</t>
-        </is>
-      </c>
-      <c r="R9" t="n">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>The SaaS Apocalypse Is Real. Causal AI Is the Escape Route</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>the-saas-apocalypse-is-real-causal-ai-is-the-escape-route</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>12</v>
-      </c>
-      <c r="D10" t="n">
-        <v>1</v>
-      </c>
-      <c r="E10" t="n">
-        <v>8</v>
-      </c>
-      <c r="F10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>trusted sources are thin; official sources are insufficiently verified; pricing sources need verification; affiliate sources need verification; competitor coverage is limited; entity extraction needs richer tool coverage; official_docs_score 0.0 below 20.0; pricing_source_score 0.0 below 20.0; affiliate_source_score 0.0 below 10.0; total_verified_source_score 0.0 below 35.0; verified_sources 0 below 1; official_verified_sources 0 below 1</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>2026-07-07T09:39:48.139069+00:00</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="K10" t="n">
-        <v>43.71</v>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>2026-07-07T09:38:58.325848+00:00</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>2026-07-07T09:38:58.485959+00:00</t>
-        </is>
-      </c>
-      <c r="N10" t="n">
-        <v>43.71</v>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>["trusted sources are thin", "official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>["official_docs", "pricing_page", "affiliate_program_page", "release_notes", "competitor_article"]</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="R10" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Impartner Redefines Partner Marketing Automation with Full Automation, AdTech and AI to Drive Measurable Revenue</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>impartner-redefines-partner-marketing-automation-with-full-automation-adtech-and-ai-to-drive-measurable-revenue</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>20</v>
-      </c>
-      <c r="D11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E11" t="n">
-        <v>5</v>
-      </c>
-      <c r="F11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>competitor coverage is limited; official_docs_score 0.0 below 20.0; pricing_source_score 0.0 below 20.0; affiliate_source_score 0.0 below 10.0; total_verified_source_score 0.0 below 35.0; verified_sources 0 below 1; official_verified_sources 0 below 1</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>2026-07-07T09:39:48.231145+00:00</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="K11" t="n">
-        <v>62.43</v>
-      </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="R11" t="n">
-        <v>0</v>
+          <t>empty</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -3532,57 +2713,57 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>is-ai-productivity-tools-pricing-worth-it-for-small-business</t>
+          <t>best-copilot-sdk-review-2026-workflows-and-use-cases-security</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>is ai productivity tools pricing worth it for small business</t>
+          <t>copilot-sdk review 2026: security and privacy</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>63.07</v>
+        <v>52.14</v>
       </c>
       <c r="D2" t="n">
         <v>72</v>
       </c>
       <c r="E2" t="n">
-        <v>76</v>
+        <v>36</v>
       </c>
       <c r="F2" t="n">
-        <v>76</v>
+        <v>36</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>["affiliate_networks", "integrations", "competitors", "use_cases", "target_audience"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H2" t="n">
         <v>68</v>
       </c>
       <c r="I2" t="n">
+        <v>80</v>
+      </c>
+      <c r="J2" t="n">
+        <v>45</v>
+      </c>
+      <c r="K2" t="n">
+        <v>54</v>
+      </c>
+      <c r="L2" t="n">
+        <v>20</v>
+      </c>
+      <c r="M2" t="n">
+        <v>20</v>
+      </c>
+      <c r="N2" t="n">
+        <v>10</v>
+      </c>
+      <c r="O2" t="n">
         <v>70</v>
       </c>
-      <c r="J2" t="n">
-        <v>57</v>
-      </c>
-      <c r="K2" t="n">
-        <v>88.5</v>
-      </c>
-      <c r="L2" t="n">
-        <v>98</v>
-      </c>
-      <c r="M2" t="n">
-        <v>98</v>
-      </c>
-      <c r="N2" t="n">
-        <v>95</v>
-      </c>
-      <c r="O2" t="n">
-        <v>77</v>
-      </c>
       <c r="P2" t="n">
-        <v>91.59999999999999</v>
+        <v>80</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -3591,80 +2772,80 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>ready</t>
+          <t>needs enrichment</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>["Notion", "Gamma", "Notion AI"]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\is-ai-productivity-tools-pricing-worth-it-for-small-business</t>
+          <t>D:\AFFILATE BOT\data\research\best-copilot-sdk-review-2026-workflows-and-use-cases-security</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>is-ai-meeting-software-alternatives-worth-it-for-small-business</t>
+          <t>best-ai-in-healthcare-marketing-moving-from-automation-to-intelligent-engagement-workflows-and-use-cases-pricing</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>is ai meeting software alternatives worth it for small business</t>
+          <t>ai in healthcare marketing: moving from automation to intelligent engagement: pricing, cost, and roi</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>62.93</v>
+        <v>60.86</v>
       </c>
       <c r="D3" t="n">
         <v>72</v>
       </c>
       <c r="E3" t="n">
-        <v>76</v>
+        <v>60</v>
       </c>
       <c r="F3" t="n">
-        <v>76</v>
+        <v>60</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>["affiliate_networks", "integrations", "competitors", "use_cases", "target_audience"]</t>
+          <t>["affiliate_networks", "integrations", "use_cases", "target_audience", "competitors"]</t>
         </is>
       </c>
       <c r="H3" t="n">
         <v>68</v>
       </c>
       <c r="I3" t="n">
+        <v>70</v>
+      </c>
+      <c r="J3" t="n">
+        <v>61</v>
+      </c>
+      <c r="K3" t="n">
+        <v>85</v>
+      </c>
+      <c r="L3" t="n">
+        <v>20</v>
+      </c>
+      <c r="M3" t="n">
+        <v>20</v>
+      </c>
+      <c r="N3" t="n">
+        <v>10</v>
+      </c>
+      <c r="O3" t="n">
+        <v>70</v>
+      </c>
+      <c r="P3" t="n">
         <v>80</v>
       </c>
-      <c r="J3" t="n">
-        <v>49</v>
-      </c>
-      <c r="K3" t="n">
-        <v>85.5</v>
-      </c>
-      <c r="L3" t="n">
-        <v>97</v>
-      </c>
-      <c r="M3" t="n">
-        <v>98</v>
-      </c>
-      <c r="N3" t="n">
-        <v>96</v>
-      </c>
-      <c r="O3" t="n">
-        <v>77</v>
-      </c>
-      <c r="P3" t="n">
-        <v>91.59999999999999</v>
-      </c>
       <c r="Q3" t="inlineStr">
         <is>
           <t>verified</t>
@@ -3682,41 +2863,41 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>["Reclaim AI"]</t>
+          <t>["Make", "AdCreative AI", "Zapier"]</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\is-ai-meeting-software-alternatives-worth-it-for-small-business</t>
+          <t>D:\AFFILATE BOT\data\research\best-ai-in-healthcare-marketing-moving-from-automation-to-intelligent-engagement-workflows-and-use-cases-pricing</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>common-ai-productivity-tools-pricing-mistakes-and-troubleshooting</t>
+          <t>fpt-software</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>common ai productivity tools pricing mistakes and troubleshooting</t>
+          <t>FPT Software</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>60.79</v>
+        <v>55.14</v>
       </c>
       <c r="D4" t="n">
         <v>72</v>
       </c>
       <c r="E4" t="n">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="F4" t="n">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>["affiliate_networks", "integrations", "use_cases", "target_audience", "competitors"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H4" t="n">
@@ -3726,25 +2907,25 @@
         <v>70</v>
       </c>
       <c r="J4" t="n">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="K4" t="n">
-        <v>88.5</v>
+        <v>85</v>
       </c>
       <c r="L4" t="n">
-        <v>98</v>
+        <v>20</v>
       </c>
       <c r="M4" t="n">
-        <v>98</v>
+        <v>20</v>
       </c>
       <c r="N4" t="n">
-        <v>95</v>
+        <v>10</v>
       </c>
       <c r="O4" t="n">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="P4" t="n">
-        <v>91.59999999999999</v>
+        <v>80</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -3753,51 +2934,51 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>ready</t>
+          <t>needs enrichment</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>["Notion", "Gamma", "Notion AI"]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\common-ai-productivity-tools-pricing-mistakes-and-troubleshooting</t>
+          <t>D:\AFFILATE BOT\data\research\fpt-software</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>common-ai-meeting-software-alternatives-mistakes-and-troubleshooting</t>
+          <t>tooljet-review-2026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>common ai meeting software alternatives mistakes and troubleshooting</t>
+          <t>ToolJet Review 2026</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>62.93</v>
+        <v>52.14</v>
       </c>
       <c r="D5" t="n">
         <v>72</v>
       </c>
       <c r="E5" t="n">
-        <v>76</v>
+        <v>36</v>
       </c>
       <c r="F5" t="n">
-        <v>76</v>
+        <v>36</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>["affiliate_networks", "integrations", "competitors", "use_cases", "target_audience"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H5" t="n">
@@ -3807,25 +2988,25 @@
         <v>80</v>
       </c>
       <c r="J5" t="n">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="K5" t="n">
-        <v>85.5</v>
+        <v>54</v>
       </c>
       <c r="L5" t="n">
-        <v>97</v>
+        <v>20</v>
       </c>
       <c r="M5" t="n">
-        <v>98</v>
+        <v>20</v>
       </c>
       <c r="N5" t="n">
-        <v>96</v>
+        <v>10</v>
       </c>
       <c r="O5" t="n">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="P5" t="n">
-        <v>91.59999999999999</v>
+        <v>80</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -3834,79 +3015,79 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>ready</t>
+          <t>needs enrichment</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>["Reclaim AI"]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\common-ai-meeting-software-alternatives-mistakes-and-troubleshooting</t>
+          <t>D:\AFFILATE BOT\data\research\tooljet-review-2026</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>how-to-implement-ai-productivity-tools-pricing</t>
+          <t>common-ai-accounting-automation-software-comparison-mistakes-and-troubleshooting</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>how to implement ai productivity tools pricing</t>
+          <t>common ai accounting automation software comparison mistakes and troubleshooting</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>60.79</v>
+        <v>64.56999999999999</v>
       </c>
       <c r="D6" t="n">
         <v>72</v>
       </c>
       <c r="E6" t="n">
-        <v>60</v>
+        <v>76</v>
       </c>
       <c r="F6" t="n">
-        <v>60</v>
+        <v>76</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>["affiliate_networks", "integrations", "use_cases", "target_audience", "competitors"]</t>
+          <t>["affiliate_networks", "integrations", "competitors", "use_cases", "target_audience"]</t>
         </is>
       </c>
       <c r="H6" t="n">
         <v>68</v>
       </c>
       <c r="I6" t="n">
+        <v>80</v>
+      </c>
+      <c r="J6" t="n">
+        <v>61</v>
+      </c>
+      <c r="K6" t="n">
+        <v>85</v>
+      </c>
+      <c r="L6" t="n">
+        <v>20</v>
+      </c>
+      <c r="M6" t="n">
+        <v>20</v>
+      </c>
+      <c r="N6" t="n">
+        <v>10</v>
+      </c>
+      <c r="O6" t="n">
         <v>70</v>
       </c>
-      <c r="J6" t="n">
-        <v>57</v>
-      </c>
-      <c r="K6" t="n">
-        <v>88.5</v>
-      </c>
-      <c r="L6" t="n">
-        <v>98</v>
-      </c>
-      <c r="M6" t="n">
-        <v>98</v>
-      </c>
-      <c r="N6" t="n">
-        <v>95</v>
-      </c>
-      <c r="O6" t="n">
-        <v>77</v>
-      </c>
       <c r="P6" t="n">
-        <v>91.59999999999999</v>
+        <v>80</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -3925,41 +3106,41 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>["Notion", "Gamma", "Notion AI"]</t>
+          <t>["Make", "Zapier"]</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\how-to-implement-ai-productivity-tools-pricing</t>
+          <t>D:\AFFILATE BOT\data\research\common-ai-accounting-automation-software-comparison-mistakes-and-troubleshooting</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>how-to-implement-ai-meeting-software-alternatives</t>
+          <t>ai-contract-review-tools-for-small-business</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>how to implement ai meeting software alternatives</t>
+          <t>ai contract review tools for small business</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>62.93</v>
+        <v>47.43</v>
       </c>
       <c r="D7" t="n">
         <v>72</v>
       </c>
       <c r="E7" t="n">
-        <v>76</v>
+        <v>52</v>
       </c>
       <c r="F7" t="n">
-        <v>76</v>
+        <v>52</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>["affiliate_networks", "integrations", "competitors", "use_cases", "target_audience"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H7" t="n">
@@ -3969,146 +3150,146 @@
         <v>80</v>
       </c>
       <c r="J7" t="n">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="K7" t="n">
-        <v>85.5</v>
+        <v>5</v>
       </c>
       <c r="L7" t="n">
-        <v>97</v>
+        <v>0</v>
       </c>
       <c r="M7" t="n">
-        <v>98</v>
+        <v>0</v>
       </c>
       <c r="N7" t="n">
-        <v>97</v>
+        <v>0</v>
       </c>
       <c r="O7" t="n">
-        <v>77</v>
+        <v>0</v>
       </c>
       <c r="P7" t="n">
-        <v>91.59999999999999</v>
+        <v>0</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>verified</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>ready</t>
+          <t>needs enrichment</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["trusted sources are thin", "official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>["Reclaim AI"]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\how-to-implement-ai-meeting-software-alternatives</t>
+          <t>D:\AFFILATE BOT\data\research\ai-contract-review-tools-for-small-business</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ai-productivity-tools-pricing</t>
+          <t>ai-accounting-automation-software-comparison</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ai productivity tools pricing</t>
+          <t>ai accounting automation software comparison</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>60.79</v>
+        <v>59.57</v>
       </c>
       <c r="D8" t="n">
         <v>72</v>
       </c>
       <c r="E8" t="n">
-        <v>60</v>
+        <v>76</v>
       </c>
       <c r="F8" t="n">
-        <v>60</v>
+        <v>76</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>["affiliate_networks", "integrations", "use_cases", "target_audience", "competitors"]</t>
+          <t>["affiliate_networks", "integrations", "competitors", "use_cases", "target_audience"]</t>
         </is>
       </c>
       <c r="H8" t="n">
         <v>68</v>
       </c>
       <c r="I8" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J8" t="n">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="K8" t="n">
-        <v>88.5</v>
+        <v>50</v>
       </c>
       <c r="L8" t="n">
-        <v>98</v>
+        <v>0</v>
       </c>
       <c r="M8" t="n">
-        <v>98</v>
+        <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="O8" t="n">
-        <v>77</v>
+        <v>0</v>
       </c>
       <c r="P8" t="n">
-        <v>91.59999999999999</v>
+        <v>0</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>verified</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>ready</t>
+          <t>needs enrichment</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>["Notion", "Gamma", "Notion AI"]</t>
+          <t>["Make", "Zapier"]</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\ai-productivity-tools-pricing</t>
+          <t>D:\AFFILATE BOT\data\research\ai-accounting-automation-software-comparison</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ai-meeting-software-alternatives</t>
+          <t>is-ai-productivity-tools-pricing-worth-it-for-small-business</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ai meeting software alternatives</t>
+          <t>is ai productivity tools pricing worth it for small business</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>59.93</v>
+        <v>63.07</v>
       </c>
       <c r="D9" t="n">
         <v>72</v>
@@ -4128,22 +3309,22 @@
         <v>68</v>
       </c>
       <c r="I9" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J9" t="n">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="K9" t="n">
-        <v>64.5</v>
+        <v>88.5</v>
       </c>
       <c r="L9" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="M9" t="n">
         <v>98</v>
       </c>
       <c r="N9" t="n">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="O9" t="n">
         <v>77</v>
@@ -4158,7 +3339,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>needs enrichment</t>
+          <t>ready</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -4168,41 +3349,41 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>["Reclaim AI"]</t>
+          <t>["Notion", "Gamma", "Notion AI"]</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\ai-meeting-software-alternatives</t>
+          <t>D:\AFFILATE BOT\data\research\is-ai-productivity-tools-pricing-worth-it-for-small-business</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>common-impeccable-review-2026-mistakes-and-troubleshooting</t>
+          <t>is-ai-meeting-software-alternatives-worth-it-for-small-business</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>common impeccable Review 2026 mistakes and troubleshooting</t>
+          <t>is ai meeting software alternatives worth it for small business</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>52.14</v>
+        <v>62.93</v>
       </c>
       <c r="D10" t="n">
         <v>72</v>
       </c>
       <c r="E10" t="n">
-        <v>36</v>
+        <v>76</v>
       </c>
       <c r="F10" t="n">
-        <v>36</v>
+        <v>76</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["affiliate_networks", "integrations", "competitors", "use_cases", "target_audience"]</t>
         </is>
       </c>
       <c r="H10" t="n">
@@ -4212,25 +3393,25 @@
         <v>80</v>
       </c>
       <c r="J10" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="K10" t="n">
-        <v>54</v>
+        <v>85.5</v>
       </c>
       <c r="L10" t="n">
-        <v>20</v>
+        <v>97</v>
       </c>
       <c r="M10" t="n">
-        <v>20</v>
+        <v>98</v>
       </c>
       <c r="N10" t="n">
-        <v>10</v>
+        <v>96</v>
       </c>
       <c r="O10" t="n">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="P10" t="n">
-        <v>80</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -4239,79 +3420,79 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>needs enrichment</t>
+          <t>ready</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["Reclaim AI"]</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\common-impeccable-review-2026-mistakes-and-troubleshooting</t>
+          <t>D:\AFFILATE BOT\data\research\is-ai-meeting-software-alternatives-worth-it-for-small-business</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>common-ego-lite-review-2026-mistakes-and-troubleshooting</t>
+          <t>common-ai-productivity-tools-pricing-mistakes-and-troubleshooting</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>common ego-lite Review 2026 mistakes and troubleshooting</t>
+          <t>common ai productivity tools pricing mistakes and troubleshooting</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>52.14</v>
+        <v>60.79</v>
       </c>
       <c r="D11" t="n">
         <v>72</v>
       </c>
       <c r="E11" t="n">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="F11" t="n">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["affiliate_networks", "integrations", "use_cases", "target_audience", "competitors"]</t>
         </is>
       </c>
       <c r="H11" t="n">
         <v>68</v>
       </c>
       <c r="I11" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J11" t="n">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="K11" t="n">
-        <v>54</v>
+        <v>88.5</v>
       </c>
       <c r="L11" t="n">
-        <v>20</v>
+        <v>98</v>
       </c>
       <c r="M11" t="n">
-        <v>20</v>
+        <v>98</v>
       </c>
       <c r="N11" t="n">
-        <v>10</v>
+        <v>95</v>
       </c>
       <c r="O11" t="n">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="P11" t="n">
-        <v>80</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -4320,22 +3501,22 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>needs enrichment</t>
+          <t>ready</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["Notion", "Gamma", "Notion AI"]</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\common-ego-lite-review-2026-mistakes-and-troubleshooting</t>
+          <t>D:\AFFILATE BOT\data\research\common-ai-productivity-tools-pricing-mistakes-and-troubleshooting</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish exact approved article how-to-implement-copilot-sdk-review-2026-security-and-privacy
</commit_message>
<xml_diff>
--- a/data/master_dashboard.xlsx
+++ b/data/master_dashboard.xlsx
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="9">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="10">
@@ -2713,16 +2713,16 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>best-copilot-sdk-review-2026-workflows-and-use-cases-security</t>
+          <t>how-to-implement-copilot-sdk-review-2026-security-and-privacy</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>copilot-sdk review 2026: security and privacy</t>
+          <t>how to implement copilot-sdk review 2026: security and privacy</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>52.14</v>
+        <v>50.71</v>
       </c>
       <c r="D2" t="n">
         <v>72</v>
@@ -2742,7 +2742,7 @@
         <v>68</v>
       </c>
       <c r="I2" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J2" t="n">
         <v>45</v>
@@ -2787,49 +2787,49 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\best-copilot-sdk-review-2026-workflows-and-use-cases-security</t>
+          <t>D:\AFFILATE BOT\data\research\how-to-implement-copilot-sdk-review-2026-security-and-privacy</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>best-ai-in-healthcare-marketing-moving-from-automation-to-intelligent-engagement-workflows-and-use-cases-pricing</t>
+          <t>best-copilot-sdk-review-2026-workflows-and-use-cases-security</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ai in healthcare marketing: moving from automation to intelligent engagement: pricing, cost, and roi</t>
+          <t>copilot-sdk review 2026: security and privacy</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>60.86</v>
+        <v>52.14</v>
       </c>
       <c r="D3" t="n">
         <v>72</v>
       </c>
       <c r="E3" t="n">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="F3" t="n">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>["affiliate_networks", "integrations", "use_cases", "target_audience", "competitors"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H3" t="n">
         <v>68</v>
       </c>
       <c r="I3" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J3" t="n">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="K3" t="n">
-        <v>85</v>
+        <v>54</v>
       </c>
       <c r="L3" t="n">
         <v>20</v>
@@ -2853,51 +2853,51 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>ready</t>
+          <t>needs enrichment</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>["Make", "AdCreative AI", "Zapier"]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\best-ai-in-healthcare-marketing-moving-from-automation-to-intelligent-engagement-workflows-and-use-cases-pricing</t>
+          <t>D:\AFFILATE BOT\data\research\best-copilot-sdk-review-2026-workflows-and-use-cases-security</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>fpt-software</t>
+          <t>best-ai-in-healthcare-marketing-moving-from-automation-to-intelligent-engagement-workflows-and-use-cases-pricing</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>FPT Software</t>
+          <t>ai in healthcare marketing: moving from automation to intelligent engagement: pricing, cost, and roi</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>55.14</v>
+        <v>60.86</v>
       </c>
       <c r="D4" t="n">
         <v>72</v>
       </c>
       <c r="E4" t="n">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="F4" t="n">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["affiliate_networks", "integrations", "use_cases", "target_audience", "competitors"]</t>
         </is>
       </c>
       <c r="H4" t="n">
@@ -2907,7 +2907,7 @@
         <v>70</v>
       </c>
       <c r="J4" t="n">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="K4" t="n">
         <v>85</v>
@@ -2934,38 +2934,38 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>needs enrichment</t>
+          <t>ready</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["Make", "AdCreative AI", "Zapier"]</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\fpt-software</t>
+          <t>D:\AFFILATE BOT\data\research\best-ai-in-healthcare-marketing-moving-from-automation-to-intelligent-engagement-workflows-and-use-cases-pricing</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>tooljet-review-2026</t>
+          <t>fpt-software</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ToolJet Review 2026</t>
+          <t>FPT Software</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>52.14</v>
+        <v>55.14</v>
       </c>
       <c r="D5" t="n">
         <v>72</v>
@@ -2985,13 +2985,13 @@
         <v>68</v>
       </c>
       <c r="I5" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J5" t="n">
         <v>45</v>
       </c>
       <c r="K5" t="n">
-        <v>54</v>
+        <v>85</v>
       </c>
       <c r="L5" t="n">
         <v>20</v>
@@ -3030,36 +3030,36 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\tooljet-review-2026</t>
+          <t>D:\AFFILATE BOT\data\research\fpt-software</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>common-ai-accounting-automation-software-comparison-mistakes-and-troubleshooting</t>
+          <t>tooljet-review-2026</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>common ai accounting automation software comparison mistakes and troubleshooting</t>
+          <t>ToolJet Review 2026</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>64.56999999999999</v>
+        <v>52.14</v>
       </c>
       <c r="D6" t="n">
         <v>72</v>
       </c>
       <c r="E6" t="n">
-        <v>76</v>
+        <v>36</v>
       </c>
       <c r="F6" t="n">
-        <v>76</v>
+        <v>36</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>["affiliate_networks", "integrations", "competitors", "use_cases", "target_audience"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H6" t="n">
@@ -3069,10 +3069,10 @@
         <v>80</v>
       </c>
       <c r="J6" t="n">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="K6" t="n">
-        <v>85</v>
+        <v>54</v>
       </c>
       <c r="L6" t="n">
         <v>20</v>
@@ -3096,51 +3096,51 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>ready</t>
+          <t>needs enrichment</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>["Make", "Zapier"]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\common-ai-accounting-automation-software-comparison-mistakes-and-troubleshooting</t>
+          <t>D:\AFFILATE BOT\data\research\tooljet-review-2026</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ai-contract-review-tools-for-small-business</t>
+          <t>common-ai-accounting-automation-software-comparison-mistakes-and-troubleshooting</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ai contract review tools for small business</t>
+          <t>common ai accounting automation software comparison mistakes and troubleshooting</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>47.43</v>
+        <v>64.56999999999999</v>
       </c>
       <c r="D7" t="n">
         <v>72</v>
       </c>
       <c r="E7" t="n">
-        <v>52</v>
+        <v>76</v>
       </c>
       <c r="F7" t="n">
-        <v>52</v>
+        <v>76</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+          <t>["affiliate_networks", "integrations", "competitors", "use_cases", "target_audience"]</t>
         </is>
       </c>
       <c r="H7" t="n">
@@ -3150,78 +3150,78 @@
         <v>80</v>
       </c>
       <c r="J7" t="n">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="K7" t="n">
-        <v>5</v>
+        <v>85</v>
       </c>
       <c r="L7" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="M7" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="N7" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O7" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="P7" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>needs enrichment</t>
+          <t>ready</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>["trusted sources are thin", "official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["Make", "Zapier"]</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\ai-contract-review-tools-for-small-business</t>
+          <t>D:\AFFILATE BOT\data\research\common-ai-accounting-automation-software-comparison-mistakes-and-troubleshooting</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ai-accounting-automation-software-comparison</t>
+          <t>ai-contract-review-tools-for-small-business</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ai accounting automation software comparison</t>
+          <t>ai contract review tools for small business</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>59.57</v>
+        <v>47.43</v>
       </c>
       <c r="D8" t="n">
         <v>72</v>
       </c>
       <c r="E8" t="n">
-        <v>76</v>
+        <v>52</v>
       </c>
       <c r="F8" t="n">
-        <v>76</v>
+        <v>52</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>["affiliate_networks", "integrations", "competitors", "use_cases", "target_audience"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H8" t="n">
@@ -3231,10 +3231,10 @@
         <v>80</v>
       </c>
       <c r="J8" t="n">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="K8" t="n">
-        <v>50</v>
+        <v>5</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
@@ -3263,33 +3263,33 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>["official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited"]</t>
+          <t>["trusted sources are thin", "official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>["Make", "Zapier"]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\ai-accounting-automation-software-comparison</t>
+          <t>D:\AFFILATE BOT\data\research\ai-contract-review-tools-for-small-business</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>is-ai-productivity-tools-pricing-worth-it-for-small-business</t>
+          <t>ai-accounting-automation-software-comparison</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>is ai productivity tools pricing worth it for small business</t>
+          <t>ai accounting automation software comparison</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>63.07</v>
+        <v>59.57</v>
       </c>
       <c r="D9" t="n">
         <v>72</v>
@@ -3309,68 +3309,68 @@
         <v>68</v>
       </c>
       <c r="I9" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J9" t="n">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="K9" t="n">
-        <v>88.5</v>
+        <v>50</v>
       </c>
       <c r="L9" t="n">
-        <v>98</v>
+        <v>0</v>
       </c>
       <c r="M9" t="n">
-        <v>98</v>
+        <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="O9" t="n">
-        <v>77</v>
+        <v>0</v>
       </c>
       <c r="P9" t="n">
-        <v>91.59999999999999</v>
+        <v>0</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>verified</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>ready</t>
+          <t>needs enrichment</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>["Notion", "Gamma", "Notion AI"]</t>
+          <t>["Make", "Zapier"]</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\is-ai-productivity-tools-pricing-worth-it-for-small-business</t>
+          <t>D:\AFFILATE BOT\data\research\ai-accounting-automation-software-comparison</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>is-ai-meeting-software-alternatives-worth-it-for-small-business</t>
+          <t>is-ai-productivity-tools-pricing-worth-it-for-small-business</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>is ai meeting software alternatives worth it for small business</t>
+          <t>is ai productivity tools pricing worth it for small business</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>62.93</v>
+        <v>63.07</v>
       </c>
       <c r="D10" t="n">
         <v>72</v>
@@ -3390,22 +3390,22 @@
         <v>68</v>
       </c>
       <c r="I10" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J10" t="n">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="K10" t="n">
-        <v>85.5</v>
+        <v>88.5</v>
       </c>
       <c r="L10" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="M10" t="n">
         <v>98</v>
       </c>
       <c r="N10" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="O10" t="n">
         <v>77</v>
@@ -3430,63 +3430,63 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>["Reclaim AI"]</t>
+          <t>["Notion", "Gamma", "Notion AI"]</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\is-ai-meeting-software-alternatives-worth-it-for-small-business</t>
+          <t>D:\AFFILATE BOT\data\research\is-ai-productivity-tools-pricing-worth-it-for-small-business</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>common-ai-productivity-tools-pricing-mistakes-and-troubleshooting</t>
+          <t>is-ai-meeting-software-alternatives-worth-it-for-small-business</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>common ai productivity tools pricing mistakes and troubleshooting</t>
+          <t>is ai meeting software alternatives worth it for small business</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>60.79</v>
+        <v>62.93</v>
       </c>
       <c r="D11" t="n">
         <v>72</v>
       </c>
       <c r="E11" t="n">
-        <v>60</v>
+        <v>76</v>
       </c>
       <c r="F11" t="n">
-        <v>60</v>
+        <v>76</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>["affiliate_networks", "integrations", "use_cases", "target_audience", "competitors"]</t>
+          <t>["affiliate_networks", "integrations", "competitors", "use_cases", "target_audience"]</t>
         </is>
       </c>
       <c r="H11" t="n">
         <v>68</v>
       </c>
       <c r="I11" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J11" t="n">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="K11" t="n">
-        <v>88.5</v>
+        <v>85.5</v>
       </c>
       <c r="L11" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="M11" t="n">
         <v>98</v>
       </c>
       <c r="N11" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="O11" t="n">
         <v>77</v>
@@ -3511,12 +3511,12 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>["Notion", "Gamma", "Notion AI"]</t>
+          <t>["Reclaim AI"]</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\common-ai-productivity-tools-pricing-mistakes-and-troubleshooting</t>
+          <t>D:\AFFILATE BOT\data\research\is-ai-meeting-software-alternatives-worth-it-for-small-business</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish ready daily articles 2026-08-26
</commit_message>
<xml_diff>
--- a/data/master_dashboard.xlsx
+++ b/data/master_dashboard.xlsx
@@ -472,7 +472,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6">
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="9">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="10">
@@ -2713,36 +2713,36 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>how-to-implement-copilot-sdk-review-2026-security-and-privacy</t>
+          <t>copilot-sdk-review-2026-security-and-privacy-comparison-and-alternatives</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>how to implement copilot-sdk review 2026: security and privacy</t>
+          <t>copilot-sdk review 2026: security and privacy comparison and alternatives</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>50.71</v>
+        <v>54.43</v>
       </c>
       <c r="D2" t="n">
         <v>72</v>
       </c>
       <c r="E2" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="F2" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H2" t="n">
         <v>68</v>
       </c>
       <c r="I2" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J2" t="n">
         <v>45</v>
@@ -2777,7 +2777,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -2787,23 +2787,23 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\how-to-implement-copilot-sdk-review-2026-security-and-privacy</t>
+          <t>D:\AFFILATE BOT\data\research\copilot-sdk-review-2026-security-and-privacy-comparison-and-alternatives</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>best-copilot-sdk-review-2026-workflows-and-use-cases-security</t>
+          <t>how-to-implement-copilot-sdk-review-2026-security-and-privacy</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>copilot-sdk review 2026: security and privacy</t>
+          <t>how to implement copilot-sdk review 2026: security and privacy</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>52.14</v>
+        <v>50.71</v>
       </c>
       <c r="D3" t="n">
         <v>72</v>
@@ -2823,7 +2823,7 @@
         <v>68</v>
       </c>
       <c r="I3" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J3" t="n">
         <v>45</v>
@@ -2868,49 +2868,49 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\best-copilot-sdk-review-2026-workflows-and-use-cases-security</t>
+          <t>D:\AFFILATE BOT\data\research\how-to-implement-copilot-sdk-review-2026-security-and-privacy</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>best-ai-in-healthcare-marketing-moving-from-automation-to-intelligent-engagement-workflows-and-use-cases-pricing</t>
+          <t>best-copilot-sdk-review-2026-workflows-and-use-cases-security</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ai in healthcare marketing: moving from automation to intelligent engagement: pricing, cost, and roi</t>
+          <t>copilot-sdk review 2026: security and privacy</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>60.86</v>
+        <v>52.14</v>
       </c>
       <c r="D4" t="n">
         <v>72</v>
       </c>
       <c r="E4" t="n">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="F4" t="n">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>["affiliate_networks", "integrations", "use_cases", "target_audience", "competitors"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H4" t="n">
         <v>68</v>
       </c>
       <c r="I4" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J4" t="n">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="K4" t="n">
-        <v>85</v>
+        <v>54</v>
       </c>
       <c r="L4" t="n">
         <v>20</v>
@@ -2934,51 +2934,51 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>ready</t>
+          <t>needs enrichment</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>["Make", "AdCreative AI", "Zapier"]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\best-ai-in-healthcare-marketing-moving-from-automation-to-intelligent-engagement-workflows-and-use-cases-pricing</t>
+          <t>D:\AFFILATE BOT\data\research\best-copilot-sdk-review-2026-workflows-and-use-cases-security</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>fpt-software</t>
+          <t>best-ai-in-healthcare-marketing-moving-from-automation-to-intelligent-engagement-workflows-and-use-cases-pricing</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>FPT Software</t>
+          <t>ai in healthcare marketing: moving from automation to intelligent engagement: pricing, cost, and roi</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>55.14</v>
+        <v>60.86</v>
       </c>
       <c r="D5" t="n">
         <v>72</v>
       </c>
       <c r="E5" t="n">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="F5" t="n">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
+          <t>["affiliate_networks", "integrations", "use_cases", "target_audience", "competitors"]</t>
         </is>
       </c>
       <c r="H5" t="n">
@@ -2988,7 +2988,7 @@
         <v>70</v>
       </c>
       <c r="J5" t="n">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="K5" t="n">
         <v>85</v>
@@ -3015,38 +3015,38 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>needs enrichment</t>
+          <t>ready</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["Make", "AdCreative AI", "Zapier"]</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\fpt-software</t>
+          <t>D:\AFFILATE BOT\data\research\best-ai-in-healthcare-marketing-moving-from-automation-to-intelligent-engagement-workflows-and-use-cases-pricing</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>tooljet-review-2026</t>
+          <t>fpt-software</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ToolJet Review 2026</t>
+          <t>FPT Software</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>52.14</v>
+        <v>55.14</v>
       </c>
       <c r="D6" t="n">
         <v>72</v>
@@ -3066,13 +3066,13 @@
         <v>68</v>
       </c>
       <c r="I6" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J6" t="n">
         <v>45</v>
       </c>
       <c r="K6" t="n">
-        <v>54</v>
+        <v>85</v>
       </c>
       <c r="L6" t="n">
         <v>20</v>
@@ -3111,36 +3111,36 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\tooljet-review-2026</t>
+          <t>D:\AFFILATE BOT\data\research\fpt-software</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>common-ai-accounting-automation-software-comparison-mistakes-and-troubleshooting</t>
+          <t>tooljet-review-2026</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>common ai accounting automation software comparison mistakes and troubleshooting</t>
+          <t>ToolJet Review 2026</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>64.56999999999999</v>
+        <v>52.14</v>
       </c>
       <c r="D7" t="n">
         <v>72</v>
       </c>
       <c r="E7" t="n">
-        <v>76</v>
+        <v>36</v>
       </c>
       <c r="F7" t="n">
-        <v>76</v>
+        <v>36</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>["affiliate_networks", "integrations", "competitors", "use_cases", "target_audience"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "use_cases", "target_audience", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H7" t="n">
@@ -3150,10 +3150,10 @@
         <v>80</v>
       </c>
       <c r="J7" t="n">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="K7" t="n">
-        <v>85</v>
+        <v>54</v>
       </c>
       <c r="L7" t="n">
         <v>20</v>
@@ -3177,51 +3177,51 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>ready</t>
+          <t>needs enrichment</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited", "entity extraction needs richer tool coverage"]</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>["Make", "Zapier"]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\common-ai-accounting-automation-software-comparison-mistakes-and-troubleshooting</t>
+          <t>D:\AFFILATE BOT\data\research\tooljet-review-2026</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ai-contract-review-tools-for-small-business</t>
+          <t>common-ai-accounting-automation-software-comparison-mistakes-and-troubleshooting</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ai contract review tools for small business</t>
+          <t>common ai accounting automation software comparison mistakes and troubleshooting</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>47.43</v>
+        <v>64.56999999999999</v>
       </c>
       <c r="D8" t="n">
         <v>72</v>
       </c>
       <c r="E8" t="n">
-        <v>52</v>
+        <v>76</v>
       </c>
       <c r="F8" t="n">
-        <v>52</v>
+        <v>76</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
+          <t>["affiliate_networks", "integrations", "competitors", "use_cases", "target_audience"]</t>
         </is>
       </c>
       <c r="H8" t="n">
@@ -3231,78 +3231,78 @@
         <v>80</v>
       </c>
       <c r="J8" t="n">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="K8" t="n">
-        <v>5</v>
+        <v>85</v>
       </c>
       <c r="L8" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="M8" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="N8" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="P8" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>needs enrichment</t>
+          <t>ready</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>["trusted sources are thin", "official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited"]</t>
+          <t>["competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["Make", "Zapier"]</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\ai-contract-review-tools-for-small-business</t>
+          <t>D:\AFFILATE BOT\data\research\common-ai-accounting-automation-software-comparison-mistakes-and-troubleshooting</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ai-accounting-automation-software-comparison</t>
+          <t>ai-contract-review-tools-for-small-business</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ai accounting automation software comparison</t>
+          <t>ai contract review tools for small business</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>59.57</v>
+        <v>47.43</v>
       </c>
       <c r="D9" t="n">
         <v>72</v>
       </c>
       <c r="E9" t="n">
-        <v>76</v>
+        <v>52</v>
       </c>
       <c r="F9" t="n">
-        <v>76</v>
+        <v>52</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>["affiliate_networks", "integrations", "competitors", "use_cases", "target_audience"]</t>
+          <t>["ai_tools", "companies", "affiliate_networks", "integrations", "competitors", "product_categories"]</t>
         </is>
       </c>
       <c r="H9" t="n">
@@ -3312,10 +3312,10 @@
         <v>80</v>
       </c>
       <c r="J9" t="n">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="K9" t="n">
-        <v>50</v>
+        <v>5</v>
       </c>
       <c r="L9" t="n">
         <v>0</v>
@@ -3344,33 +3344,33 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>["official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited"]</t>
+          <t>["trusted sources are thin", "official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>["Make", "Zapier"]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\ai-accounting-automation-software-comparison</t>
+          <t>D:\AFFILATE BOT\data\research\ai-contract-review-tools-for-small-business</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>is-ai-productivity-tools-pricing-worth-it-for-small-business</t>
+          <t>ai-accounting-automation-software-comparison</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>is ai productivity tools pricing worth it for small business</t>
+          <t>ai accounting automation software comparison</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>63.07</v>
+        <v>59.57</v>
       </c>
       <c r="D10" t="n">
         <v>72</v>
@@ -3390,68 +3390,68 @@
         <v>68</v>
       </c>
       <c r="I10" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J10" t="n">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="K10" t="n">
-        <v>88.5</v>
+        <v>50</v>
       </c>
       <c r="L10" t="n">
-        <v>98</v>
+        <v>0</v>
       </c>
       <c r="M10" t="n">
-        <v>98</v>
+        <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="O10" t="n">
-        <v>77</v>
+        <v>0</v>
       </c>
       <c r="P10" t="n">
-        <v>91.59999999999999</v>
+        <v>0</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>verified</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>ready</t>
+          <t>needs enrichment</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>["competitor coverage is limited"]</t>
+          <t>["official sources are insufficiently verified", "pricing sources need verification", "affiliate sources need verification", "competitor coverage is limited"]</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>["Notion", "Gamma", "Notion AI"]</t>
+          <t>["Make", "Zapier"]</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\is-ai-productivity-tools-pricing-worth-it-for-small-business</t>
+          <t>D:\AFFILATE BOT\data\research\ai-accounting-automation-software-comparison</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>is-ai-meeting-software-alternatives-worth-it-for-small-business</t>
+          <t>is-ai-productivity-tools-pricing-worth-it-for-small-business</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>is ai meeting software alternatives worth it for small business</t>
+          <t>is ai productivity tools pricing worth it for small business</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>62.93</v>
+        <v>63.07</v>
       </c>
       <c r="D11" t="n">
         <v>72</v>
@@ -3471,22 +3471,22 @@
         <v>68</v>
       </c>
       <c r="I11" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="J11" t="n">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="K11" t="n">
-        <v>85.5</v>
+        <v>88.5</v>
       </c>
       <c r="L11" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="M11" t="n">
         <v>98</v>
       </c>
       <c r="N11" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="O11" t="n">
         <v>77</v>
@@ -3511,12 +3511,12 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>["Reclaim AI"]</t>
+          <t>["Notion", "Gamma", "Notion AI"]</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>D:\AFFILATE BOT\data\research\is-ai-meeting-software-alternatives-worth-it-for-small-business</t>
+          <t>D:\AFFILATE BOT\data\research\is-ai-productivity-tools-pricing-worth-it-for-small-business</t>
         </is>
       </c>
     </row>

</xml_diff>